<commit_message>
Auto Update: Market & Industry Thermometer [Sun Sep 13 13:54:16 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.7</v>
       </c>
       <c r="E2" t="n">
+        <v>97.8</v>
+      </c>
+      <c r="F2" t="n">
         <v>98.2</v>
       </c>
-      <c r="F2" t="n">
-        <v>98.5</v>
-      </c>
       <c r="G2" t="n">
-        <v>98.40000000000001</v>
+        <v>98</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>0.99</v>
       </c>
       <c r="E3" t="n">
-        <v>79.90000000000001</v>
+        <v>79.7</v>
       </c>
       <c r="F3" t="n">
-        <v>60.6</v>
+        <v>60.5</v>
       </c>
       <c r="G3" t="n">
-        <v>70.3</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>2.03</v>
       </c>
       <c r="E4" t="n">
-        <v>91.59999999999999</v>
+        <v>91.3</v>
       </c>
       <c r="F4" t="n">
-        <v>30.7</v>
+        <v>30.8</v>
       </c>
       <c r="G4" t="n">
         <v>61.1</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>1.73</v>
       </c>
       <c r="E5" t="n">
-        <v>82.8</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>34.3</v>
+        <v>34.4</v>
       </c>
       <c r="G5" t="n">
-        <v>58.6</v>
+        <v>58.5</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>1.84</v>
       </c>
       <c r="E6" t="n">
-        <v>19.7</v>
+        <v>19.9</v>
       </c>
       <c r="F6" t="n">
-        <v>86.09999999999999</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="G6" t="n">
         <v>52.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="7">
@@ -642,7 +642,7 @@
         <v>3.55</v>
       </c>
       <c r="E7" t="n">
-        <v>35.8</v>
+        <v>35.9</v>
       </c>
       <c r="F7" t="n">
         <v>58</v>
@@ -651,7 +651,7 @@
         <v>46.9</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>1.36</v>
       </c>
       <c r="E8" t="n">
-        <v>22.6</v>
+        <v>22.8</v>
       </c>
       <c r="F8" t="n">
-        <v>65</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="G8" t="n">
         <v>43.8</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>2.85</v>
       </c>
       <c r="E9" t="n">
-        <v>41.2</v>
+        <v>41.3</v>
       </c>
       <c r="F9" t="n">
-        <v>45.6</v>
+        <v>45.7</v>
       </c>
       <c r="G9" t="n">
-        <v>43.4</v>
+        <v>43.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.03</v>
       </c>
       <c r="E10" t="n">
-        <v>22.3</v>
+        <v>22.5</v>
       </c>
       <c r="F10" t="n">
-        <v>59.5</v>
+        <v>59.4</v>
       </c>
       <c r="G10" t="n">
         <v>40.9</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="11">
@@ -762,7 +762,7 @@
         <v>2.34</v>
       </c>
       <c r="E11" t="n">
-        <v>26.3</v>
+        <v>26.4</v>
       </c>
       <c r="F11" t="n">
         <v>53.6</v>
@@ -771,7 +771,7 @@
         <v>40</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>1.63</v>
       </c>
       <c r="E12" t="n">
-        <v>38.3</v>
+        <v>38.4</v>
       </c>
       <c r="F12" t="n">
-        <v>37.6</v>
+        <v>37.7</v>
       </c>
       <c r="G12" t="n">
         <v>38</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>2.02</v>
       </c>
       <c r="E13" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="F13" t="n">
-        <v>42.7</v>
+        <v>42.8</v>
       </c>
       <c r="G13" t="n">
-        <v>37.2</v>
+        <v>37.3</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.85</v>
       </c>
       <c r="E14" t="n">
-        <v>29.6</v>
+        <v>29.7</v>
       </c>
       <c r="F14" t="n">
         <v>43.8</v>
       </c>
       <c r="G14" t="n">
-        <v>36.7</v>
+        <v>36.8</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.22</v>
       </c>
       <c r="E15" t="n">
-        <v>22.3</v>
+        <v>22.5</v>
       </c>
       <c r="F15" t="n">
         <v>50.7</v>
       </c>
       <c r="G15" t="n">
-        <v>36.5</v>
+        <v>36.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>1.98</v>
       </c>
       <c r="E16" t="n">
-        <v>25.2</v>
+        <v>25.4</v>
       </c>
       <c r="F16" t="n">
-        <v>40.5</v>
+        <v>40.6</v>
       </c>
       <c r="G16" t="n">
-        <v>32.8</v>
+        <v>33</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>2.34</v>
       </c>
       <c r="E17" t="n">
-        <v>23</v>
+        <v>23.2</v>
       </c>
       <c r="F17" t="n">
         <v>38</v>
       </c>
       <c r="G17" t="n">
-        <v>30.5</v>
+        <v>30.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>3.63</v>
       </c>
       <c r="E18" t="n">
-        <v>18.6</v>
+        <v>18.8</v>
       </c>
       <c r="F18" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="G18" t="n">
-        <v>25.2</v>
+        <v>25.4</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>2.58</v>
       </c>
       <c r="E19" t="n">
-        <v>18.6</v>
+        <v>18.8</v>
       </c>
       <c r="F19" t="n">
-        <v>27.7</v>
+        <v>27.9</v>
       </c>
       <c r="G19" t="n">
-        <v>25</v>
+        <v>25.2</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>7.62</v>
       </c>
       <c r="E20" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="F20" t="n">
-        <v>41.2</v>
+        <v>41.3</v>
       </c>
       <c r="G20" t="n">
-        <v>22.3</v>
+        <v>22.5</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="21">
@@ -1065,13 +1065,13 @@
         <v>44.2</v>
       </c>
       <c r="F21" t="n">
-        <v>6.6</v>
+        <v>6.9</v>
       </c>
       <c r="G21" t="n">
-        <v>17.8</v>
+        <v>18.1</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>3.2</v>
       </c>
       <c r="E22" t="n">
-        <v>14.2</v>
+        <v>14.5</v>
       </c>
       <c r="F22" t="n">
-        <v>19.3</v>
+        <v>19.6</v>
       </c>
       <c r="G22" t="n">
-        <v>17.8</v>
+        <v>18</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>3.61</v>
       </c>
       <c r="E23" t="n">
-        <v>5.5</v>
+        <v>5.8</v>
       </c>
       <c r="F23" t="n">
-        <v>19</v>
+        <v>19.2</v>
       </c>
       <c r="G23" t="n">
-        <v>14.9</v>
+        <v>15.2</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>0.93</v>
       </c>
       <c r="E24" t="n">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="F24" t="n">
-        <v>17.2</v>
+        <v>17.4</v>
       </c>
       <c r="G24" t="n">
-        <v>12.8</v>
+        <v>13</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.2</v>
       </c>
       <c r="E25" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="F25" t="n">
-        <v>16.1</v>
+        <v>16.3</v>
       </c>
       <c r="G25" t="n">
-        <v>11.6</v>
+        <v>11.8</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.3</v>
       </c>
       <c r="E26" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="F26" t="n">
-        <v>14.6</v>
+        <v>14.9</v>
       </c>
       <c r="G26" t="n">
-        <v>10.5</v>
+        <v>10.8</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.3</v>
       </c>
       <c r="E27" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="F27" t="n">
-        <v>13.9</v>
+        <v>14.1</v>
       </c>
       <c r="G27" t="n">
-        <v>10</v>
+        <v>10.3</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>3.23</v>
       </c>
       <c r="E28" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="F28" t="n">
-        <v>9.9</v>
+        <v>10.1</v>
       </c>
       <c r="G28" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>3.73</v>
       </c>
       <c r="E29" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="F29" t="n">
-        <v>8.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G29" t="n">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.42</v>
       </c>
       <c r="E30" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="F30" t="n">
-        <v>6.9</v>
+        <v>7.2</v>
       </c>
       <c r="G30" t="n">
-        <v>5.8</v>
+        <v>6.2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>2</v>
       </c>
       <c r="E31" t="n">
-        <v>12.8</v>
+        <v>13</v>
       </c>
       <c r="F31" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
       <c r="G31" t="n">
-        <v>5.1</v>
+        <v>5.4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.9</v>
       </c>
       <c r="E32" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="F32" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="G32" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon Sep 14 16:00:18 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.37</v>
+        <v>7.43</v>
       </c>
       <c r="D2" t="n">
         <v>0.7</v>
       </c>
       <c r="E2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F2" t="n">
         <v>97.8</v>
       </c>
-      <c r="F2" t="n">
-        <v>98.2</v>
-      </c>
       <c r="G2" t="n">
-        <v>98</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="3">
@@ -516,352 +516,352 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.29</v>
+        <v>20.31</v>
       </c>
       <c r="D3" t="n">
         <v>0.99</v>
       </c>
       <c r="E3" t="n">
-        <v>79.7</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>60.5</v>
+        <v>60.4</v>
       </c>
       <c r="G3" t="n">
-        <v>70.09999999999999</v>
+        <v>70.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>33.84</v>
+        <v>20.46</v>
       </c>
       <c r="D4" t="n">
-        <v>2.03</v>
+        <v>1.73</v>
       </c>
       <c r="E4" t="n">
-        <v>91.3</v>
+        <v>83.8</v>
       </c>
       <c r="F4" t="n">
-        <v>30.8</v>
+        <v>34.5</v>
       </c>
       <c r="G4" t="n">
-        <v>61.1</v>
+        <v>59.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>20.42</v>
+        <v>19.83</v>
       </c>
       <c r="D5" t="n">
-        <v>1.73</v>
+        <v>3.56</v>
       </c>
       <c r="E5" t="n">
-        <v>82.59999999999999</v>
+        <v>42.1</v>
       </c>
       <c r="F5" t="n">
-        <v>34.4</v>
+        <v>61.5</v>
       </c>
       <c r="G5" t="n">
-        <v>58.5</v>
+        <v>51.8</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>17.08</v>
+        <v>19.65</v>
       </c>
       <c r="D6" t="n">
-        <v>1.84</v>
+        <v>1.64</v>
       </c>
       <c r="E6" t="n">
-        <v>19.9</v>
+        <v>50.4</v>
       </c>
       <c r="F6" t="n">
-        <v>85.90000000000001</v>
+        <v>44.2</v>
       </c>
       <c r="G6" t="n">
-        <v>52.9</v>
+        <v>47.3</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>19.78</v>
+        <v>16.87</v>
       </c>
       <c r="D7" t="n">
-        <v>3.55</v>
+        <v>1.82</v>
       </c>
       <c r="E7" t="n">
-        <v>35.9</v>
+        <v>12.9</v>
       </c>
       <c r="F7" t="n">
-        <v>58</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>46.9</v>
+        <v>46</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>12.94</v>
+        <v>32.8</v>
       </c>
       <c r="D8" t="n">
-        <v>1.36</v>
+        <v>2.04</v>
       </c>
       <c r="E8" t="n">
-        <v>22.8</v>
+        <v>25.2</v>
       </c>
       <c r="F8" t="n">
-        <v>64.90000000000001</v>
+        <v>65.5</v>
       </c>
       <c r="G8" t="n">
-        <v>43.8</v>
+        <v>45.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>29.71</v>
+        <v>15.3</v>
       </c>
       <c r="D9" t="n">
-        <v>2.85</v>
+        <v>2.35</v>
       </c>
       <c r="E9" t="n">
-        <v>41.3</v>
+        <v>31.7</v>
       </c>
       <c r="F9" t="n">
-        <v>45.7</v>
+        <v>56.1</v>
       </c>
       <c r="G9" t="n">
-        <v>43.5</v>
+        <v>43.9</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>32.52</v>
+        <v>21.87</v>
       </c>
       <c r="D10" t="n">
         <v>2.03</v>
       </c>
       <c r="E10" t="n">
-        <v>22.5</v>
+        <v>37.4</v>
       </c>
       <c r="F10" t="n">
-        <v>59.4</v>
+        <v>47.1</v>
       </c>
       <c r="G10" t="n">
-        <v>40.9</v>
+        <v>42.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>15.25</v>
+        <v>21.74</v>
       </c>
       <c r="D11" t="n">
-        <v>2.34</v>
+        <v>1.85</v>
       </c>
       <c r="E11" t="n">
-        <v>26.4</v>
+        <v>30.9</v>
       </c>
       <c r="F11" t="n">
-        <v>53.6</v>
+        <v>43.9</v>
       </c>
       <c r="G11" t="n">
-        <v>40</v>
+        <v>37.4</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>19.51</v>
+        <v>33.14</v>
       </c>
       <c r="D12" t="n">
-        <v>1.63</v>
+        <v>1.99</v>
       </c>
       <c r="E12" t="n">
-        <v>38.4</v>
+        <v>87.8</v>
       </c>
       <c r="F12" t="n">
-        <v>37.7</v>
+        <v>14.4</v>
       </c>
       <c r="G12" t="n">
-        <v>38</v>
+        <v>36.4</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>21.73</v>
+        <v>27.47</v>
       </c>
       <c r="D13" t="n">
-        <v>2.02</v>
+        <v>2.63</v>
       </c>
       <c r="E13" t="n">
-        <v>31.9</v>
+        <v>24.5</v>
       </c>
       <c r="F13" t="n">
-        <v>42.8</v>
+        <v>48.2</v>
       </c>
       <c r="G13" t="n">
-        <v>37.3</v>
+        <v>36.3</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>21.73</v>
+        <v>12.78</v>
       </c>
       <c r="D14" t="n">
-        <v>1.85</v>
+        <v>1.34</v>
       </c>
       <c r="E14" t="n">
-        <v>29.7</v>
+        <v>15.8</v>
       </c>
       <c r="F14" t="n">
-        <v>43.8</v>
+        <v>56.1</v>
       </c>
       <c r="G14" t="n">
-        <v>36.8</v>
+        <v>36</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="15">
@@ -876,262 +876,262 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>14.47</v>
+        <v>14.46</v>
       </c>
       <c r="D15" t="n">
         <v>1.22</v>
       </c>
       <c r="E15" t="n">
-        <v>22.5</v>
+        <v>20.9</v>
       </c>
       <c r="F15" t="n">
         <v>50.7</v>
       </c>
       <c r="G15" t="n">
-        <v>36.6</v>
+        <v>35.8</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>23.59</v>
+        <v>29.79</v>
       </c>
       <c r="D16" t="n">
-        <v>1.98</v>
+        <v>2.34</v>
       </c>
       <c r="E16" t="n">
-        <v>25.4</v>
+        <v>23.4</v>
       </c>
       <c r="F16" t="n">
-        <v>40.6</v>
+        <v>38.1</v>
       </c>
       <c r="G16" t="n">
-        <v>33</v>
+        <v>30.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>29.79</v>
+        <v>29.22</v>
       </c>
       <c r="D17" t="n">
-        <v>2.34</v>
+        <v>2.8</v>
       </c>
       <c r="E17" t="n">
-        <v>23.2</v>
+        <v>23.4</v>
       </c>
       <c r="F17" t="n">
-        <v>38</v>
+        <v>33.5</v>
       </c>
       <c r="G17" t="n">
-        <v>30.6</v>
+        <v>28.4</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>52.99</v>
+        <v>23.36</v>
       </c>
       <c r="D18" t="n">
-        <v>3.63</v>
+        <v>1.96</v>
       </c>
       <c r="E18" t="n">
-        <v>18.8</v>
+        <v>16.9</v>
       </c>
       <c r="F18" t="n">
-        <v>31.9</v>
+        <v>37.4</v>
       </c>
       <c r="G18" t="n">
-        <v>25.4</v>
+        <v>27.2</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>26.87</v>
+        <v>36.59</v>
       </c>
       <c r="D19" t="n">
-        <v>2.58</v>
+        <v>3.21</v>
       </c>
       <c r="E19" t="n">
-        <v>18.8</v>
+        <v>17.3</v>
       </c>
       <c r="F19" t="n">
-        <v>27.9</v>
+        <v>21.6</v>
       </c>
       <c r="G19" t="n">
-        <v>25.2</v>
+        <v>20.3</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>51.36</v>
+        <v>52.03</v>
       </c>
       <c r="D20" t="n">
-        <v>7.62</v>
+        <v>3.56</v>
       </c>
       <c r="E20" t="n">
-        <v>3.6</v>
+        <v>10.8</v>
       </c>
       <c r="F20" t="n">
-        <v>41.3</v>
+        <v>23.4</v>
       </c>
       <c r="G20" t="n">
-        <v>22.5</v>
+        <v>19.6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>10.68</v>
+        <v>50.61</v>
       </c>
       <c r="D21" t="n">
-        <v>0.63</v>
+        <v>7.51</v>
       </c>
       <c r="E21" t="n">
-        <v>44.2</v>
+        <v>2.9</v>
       </c>
       <c r="F21" t="n">
-        <v>6.9</v>
+        <v>33.1</v>
       </c>
       <c r="G21" t="n">
-        <v>18.1</v>
+        <v>18</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>36.42</v>
+        <v>10.64</v>
       </c>
       <c r="D22" t="n">
-        <v>3.2</v>
+        <v>0.63</v>
       </c>
       <c r="E22" t="n">
-        <v>14.5</v>
+        <v>42.8</v>
       </c>
       <c r="F22" t="n">
-        <v>19.6</v>
+        <v>7.2</v>
       </c>
       <c r="G22" t="n">
-        <v>18</v>
+        <v>17.9</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>68.12</v>
+        <v>25.8</v>
       </c>
       <c r="D23" t="n">
-        <v>3.61</v>
+        <v>2.31</v>
       </c>
       <c r="E23" t="n">
-        <v>5.8</v>
+        <v>2.9</v>
       </c>
       <c r="F23" t="n">
-        <v>19.2</v>
+        <v>18</v>
       </c>
       <c r="G23" t="n">
-        <v>15.2</v>
+        <v>13.5</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="24">
@@ -1146,232 +1146,232 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>8.42</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="D24" t="n">
         <v>0.93</v>
       </c>
       <c r="E24" t="n">
-        <v>2.9</v>
+        <v>2.2</v>
       </c>
       <c r="F24" t="n">
-        <v>17.4</v>
+        <v>17.6</v>
       </c>
       <c r="G24" t="n">
         <v>13</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>7.77</v>
+        <v>67.44</v>
       </c>
       <c r="D25" t="n">
-        <v>1.2</v>
+        <v>3.57</v>
       </c>
       <c r="E25" t="n">
-        <v>1.4</v>
+        <v>4.3</v>
       </c>
       <c r="F25" t="n">
-        <v>16.3</v>
+        <v>16.5</v>
       </c>
       <c r="G25" t="n">
-        <v>11.8</v>
+        <v>12.9</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>25.72</v>
+        <v>22.14</v>
       </c>
       <c r="D26" t="n">
-        <v>2.3</v>
+        <v>2.31</v>
       </c>
       <c r="E26" t="n">
-        <v>1.4</v>
+        <v>2.9</v>
       </c>
       <c r="F26" t="n">
-        <v>14.9</v>
+        <v>16.2</v>
       </c>
       <c r="G26" t="n">
-        <v>10.8</v>
+        <v>12.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>22.04</v>
+        <v>7.75</v>
       </c>
       <c r="D27" t="n">
-        <v>2.3</v>
+        <v>1.2</v>
       </c>
       <c r="E27" t="n">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="F27" t="n">
-        <v>14.1</v>
+        <v>16.5</v>
       </c>
       <c r="G27" t="n">
-        <v>10.3</v>
+        <v>11.8</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>17.24</v>
+        <v>18.68</v>
       </c>
       <c r="D28" t="n">
-        <v>3.23</v>
+        <v>1.43</v>
       </c>
       <c r="E28" t="n">
-        <v>1.4</v>
+        <v>5</v>
       </c>
       <c r="F28" t="n">
-        <v>10.1</v>
+        <v>11.5</v>
       </c>
       <c r="G28" t="n">
-        <v>7.5</v>
+        <v>9.6</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>40.05</v>
+        <v>22.47</v>
       </c>
       <c r="D29" t="n">
-        <v>3.73</v>
+        <v>2.02</v>
       </c>
       <c r="E29" t="n">
-        <v>1.4</v>
+        <v>16.5</v>
       </c>
       <c r="F29" t="n">
-        <v>8.699999999999999</v>
+        <v>6.5</v>
       </c>
       <c r="G29" t="n">
-        <v>6.5</v>
+        <v>9.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>18.58</v>
+        <v>40.18</v>
       </c>
       <c r="D30" t="n">
-        <v>1.42</v>
+        <v>3.74</v>
       </c>
       <c r="E30" t="n">
-        <v>3.6</v>
+        <v>2.9</v>
       </c>
       <c r="F30" t="n">
-        <v>7.2</v>
+        <v>10.8</v>
       </c>
       <c r="G30" t="n">
-        <v>6.2</v>
+        <v>8.4</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>22.26</v>
+        <v>17.15</v>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>3.21</v>
       </c>
       <c r="E31" t="n">
-        <v>13</v>
+        <v>0.7</v>
       </c>
       <c r="F31" t="n">
-        <v>2.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G31" t="n">
-        <v>5.4</v>
+        <v>6</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25.74</v>
+        <v>25.95</v>
       </c>
       <c r="D32" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="E32" t="n">
         <v>2.9</v>
       </c>
-      <c r="E32" t="n">
-        <v>1.4</v>
-      </c>
       <c r="F32" t="n">
-        <v>1.4</v>
+        <v>2.9</v>
       </c>
       <c r="G32" t="n">
-        <v>1.4</v>
+        <v>2.9</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue Sep 15 14:29:34 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.43</v>
+        <v>7.34</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>97.8</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>98.90000000000001</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="3">
@@ -516,202 +516,202 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.31</v>
+        <v>20.24</v>
       </c>
       <c r="D3" t="n">
         <v>0.99</v>
       </c>
       <c r="E3" t="n">
-        <v>80.59999999999999</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="F3" t="n">
         <v>60.4</v>
       </c>
       <c r="G3" t="n">
-        <v>70.5</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>20.46</v>
+        <v>33.33</v>
       </c>
       <c r="D4" t="n">
-        <v>1.73</v>
+        <v>2.08</v>
       </c>
       <c r="E4" t="n">
-        <v>83.8</v>
+        <v>26.4</v>
       </c>
       <c r="F4" t="n">
-        <v>34.5</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>59.2</v>
+        <v>48.8</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>19.83</v>
+        <v>16.8</v>
       </c>
       <c r="D5" t="n">
-        <v>3.56</v>
+        <v>1.81</v>
       </c>
       <c r="E5" t="n">
-        <v>42.1</v>
+        <v>12.1</v>
       </c>
       <c r="F5" t="n">
-        <v>61.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>51.8</v>
+        <v>45</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>19.65</v>
+        <v>19.71</v>
       </c>
       <c r="D6" t="n">
-        <v>1.64</v>
+        <v>3.53</v>
       </c>
       <c r="E6" t="n">
-        <v>50.4</v>
+        <v>32.9</v>
       </c>
       <c r="F6" t="n">
-        <v>44.2</v>
+        <v>52.1</v>
       </c>
       <c r="G6" t="n">
-        <v>47.3</v>
+        <v>42.5</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>16.87</v>
+        <v>20.33</v>
       </c>
       <c r="D7" t="n">
-        <v>1.82</v>
+        <v>1.72</v>
       </c>
       <c r="E7" t="n">
-        <v>12.9</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>79.09999999999999</v>
+        <v>25</v>
       </c>
       <c r="G7" t="n">
-        <v>46</v>
+        <v>40.9</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>32.8</v>
+        <v>15.25</v>
       </c>
       <c r="D8" t="n">
-        <v>2.04</v>
+        <v>2.34</v>
       </c>
       <c r="E8" t="n">
-        <v>25.2</v>
+        <v>26.4</v>
       </c>
       <c r="F8" t="n">
-        <v>65.5</v>
+        <v>53.2</v>
       </c>
       <c r="G8" t="n">
-        <v>45.3</v>
+        <v>39.8</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>15.3</v>
+        <v>14.42</v>
       </c>
       <c r="D9" t="n">
-        <v>2.35</v>
+        <v>1.22</v>
       </c>
       <c r="E9" t="n">
-        <v>31.7</v>
+        <v>19.3</v>
       </c>
       <c r="F9" t="n">
-        <v>56.1</v>
+        <v>50.7</v>
       </c>
       <c r="G9" t="n">
-        <v>43.9</v>
+        <v>35</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="10">
@@ -726,262 +726,262 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>21.87</v>
+        <v>21.65</v>
       </c>
       <c r="D10" t="n">
-        <v>2.03</v>
+        <v>2.01</v>
       </c>
       <c r="E10" t="n">
-        <v>37.4</v>
+        <v>26.4</v>
       </c>
       <c r="F10" t="n">
-        <v>47.1</v>
+        <v>40</v>
       </c>
       <c r="G10" t="n">
-        <v>42.3</v>
+        <v>33.2</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>21.74</v>
+        <v>12.71</v>
       </c>
       <c r="D11" t="n">
-        <v>1.85</v>
+        <v>1.33</v>
       </c>
       <c r="E11" t="n">
-        <v>30.9</v>
+        <v>15</v>
       </c>
       <c r="F11" t="n">
-        <v>43.9</v>
+        <v>49.6</v>
       </c>
       <c r="G11" t="n">
-        <v>37.4</v>
+        <v>32.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>33.14</v>
+        <v>27.2</v>
       </c>
       <c r="D12" t="n">
-        <v>1.99</v>
+        <v>2.61</v>
       </c>
       <c r="E12" t="n">
-        <v>87.8</v>
+        <v>22.1</v>
       </c>
       <c r="F12" t="n">
-        <v>14.4</v>
+        <v>41.8</v>
       </c>
       <c r="G12" t="n">
-        <v>36.4</v>
+        <v>32</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>27.47</v>
+        <v>19.4</v>
       </c>
       <c r="D13" t="n">
-        <v>2.63</v>
+        <v>1.62</v>
       </c>
       <c r="E13" t="n">
-        <v>24.5</v>
+        <v>31.1</v>
       </c>
       <c r="F13" t="n">
-        <v>48.2</v>
+        <v>30</v>
       </c>
       <c r="G13" t="n">
-        <v>36.3</v>
+        <v>30.5</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>12.78</v>
+        <v>32.45</v>
       </c>
       <c r="D14" t="n">
-        <v>1.34</v>
+        <v>1.95</v>
       </c>
       <c r="E14" t="n">
-        <v>15.8</v>
+        <v>85.7</v>
       </c>
       <c r="F14" t="n">
-        <v>56.1</v>
+        <v>6.4</v>
       </c>
       <c r="G14" t="n">
-        <v>36</v>
+        <v>30.2</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>14.46</v>
+        <v>29.09</v>
       </c>
       <c r="D15" t="n">
-        <v>1.22</v>
+        <v>2.79</v>
       </c>
       <c r="E15" t="n">
-        <v>20.9</v>
+        <v>19.6</v>
       </c>
       <c r="F15" t="n">
-        <v>50.7</v>
+        <v>29.6</v>
       </c>
       <c r="G15" t="n">
-        <v>35.8</v>
+        <v>26.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>29.79</v>
+        <v>21.13</v>
       </c>
       <c r="D16" t="n">
-        <v>2.34</v>
+        <v>1.8</v>
       </c>
       <c r="E16" t="n">
-        <v>23.4</v>
+        <v>15</v>
       </c>
       <c r="F16" t="n">
-        <v>38.1</v>
+        <v>25.7</v>
       </c>
       <c r="G16" t="n">
-        <v>30.8</v>
+        <v>22.5</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>29.22</v>
+        <v>23.18</v>
       </c>
       <c r="D17" t="n">
-        <v>2.8</v>
+        <v>1.94</v>
       </c>
       <c r="E17" t="n">
-        <v>23.4</v>
+        <v>12.1</v>
       </c>
       <c r="F17" t="n">
-        <v>33.5</v>
+        <v>31.8</v>
       </c>
       <c r="G17" t="n">
-        <v>28.4</v>
+        <v>22</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>23.36</v>
+        <v>50.9</v>
       </c>
       <c r="D18" t="n">
-        <v>1.96</v>
+        <v>7.55</v>
       </c>
       <c r="E18" t="n">
-        <v>16.9</v>
+        <v>3.6</v>
       </c>
       <c r="F18" t="n">
-        <v>37.4</v>
+        <v>36.4</v>
       </c>
       <c r="G18" t="n">
-        <v>27.2</v>
+        <v>20</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="19">
@@ -996,382 +996,382 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>36.59</v>
+        <v>36.34</v>
       </c>
       <c r="D19" t="n">
-        <v>3.21</v>
+        <v>3.19</v>
       </c>
       <c r="E19" t="n">
-        <v>17.3</v>
+        <v>13.6</v>
       </c>
       <c r="F19" t="n">
-        <v>21.6</v>
+        <v>18.6</v>
       </c>
       <c r="G19" t="n">
-        <v>20.3</v>
+        <v>17.1</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>52.03</v>
+        <v>29.14</v>
       </c>
       <c r="D20" t="n">
-        <v>3.56</v>
+        <v>2.29</v>
       </c>
       <c r="E20" t="n">
-        <v>10.8</v>
+        <v>11.4</v>
       </c>
       <c r="F20" t="n">
-        <v>23.4</v>
+        <v>18.6</v>
       </c>
       <c r="G20" t="n">
-        <v>19.6</v>
+        <v>16.4</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>50.61</v>
+        <v>51.55</v>
       </c>
       <c r="D21" t="n">
-        <v>7.51</v>
+        <v>3.53</v>
       </c>
       <c r="E21" t="n">
-        <v>2.9</v>
+        <v>5</v>
       </c>
       <c r="F21" t="n">
-        <v>33.1</v>
+        <v>19.3</v>
       </c>
       <c r="G21" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>10.64</v>
+        <v>66.87</v>
       </c>
       <c r="D22" t="n">
-        <v>0.63</v>
+        <v>3.55</v>
       </c>
       <c r="E22" t="n">
-        <v>42.8</v>
+        <v>4.3</v>
       </c>
       <c r="F22" t="n">
-        <v>7.2</v>
+        <v>16.4</v>
       </c>
       <c r="G22" t="n">
-        <v>17.9</v>
+        <v>12.8</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>25.8</v>
+        <v>10.5</v>
       </c>
       <c r="D23" t="n">
-        <v>2.31</v>
+        <v>0.62</v>
       </c>
       <c r="E23" t="n">
-        <v>2.9</v>
+        <v>37.9</v>
       </c>
       <c r="F23" t="n">
-        <v>18</v>
+        <v>0.7</v>
       </c>
       <c r="G23" t="n">
-        <v>13.5</v>
+        <v>11.9</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>8.289999999999999</v>
+        <v>22.08</v>
       </c>
       <c r="D24" t="n">
-        <v>0.93</v>
+        <v>2.3</v>
       </c>
       <c r="E24" t="n">
-        <v>2.2</v>
+        <v>2.9</v>
       </c>
       <c r="F24" t="n">
-        <v>17.6</v>
+        <v>14.3</v>
       </c>
       <c r="G24" t="n">
-        <v>13</v>
+        <v>10.9</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>67.44</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="D25" t="n">
-        <v>3.57</v>
+        <v>0.92</v>
       </c>
       <c r="E25" t="n">
-        <v>4.3</v>
+        <v>2.9</v>
       </c>
       <c r="F25" t="n">
-        <v>16.5</v>
+        <v>10.7</v>
       </c>
       <c r="G25" t="n">
-        <v>12.9</v>
+        <v>8.4</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>22.14</v>
+        <v>7.68</v>
       </c>
       <c r="D26" t="n">
-        <v>2.31</v>
+        <v>1.19</v>
       </c>
       <c r="E26" t="n">
-        <v>2.9</v>
+        <v>0.7</v>
       </c>
       <c r="F26" t="n">
-        <v>16.2</v>
+        <v>10</v>
       </c>
       <c r="G26" t="n">
-        <v>12.2</v>
+        <v>7.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>7.75</v>
+        <v>25.4</v>
       </c>
       <c r="D27" t="n">
-        <v>1.2</v>
+        <v>2.27</v>
       </c>
       <c r="E27" t="n">
         <v>0.7</v>
       </c>
       <c r="F27" t="n">
-        <v>16.5</v>
+        <v>7.9</v>
       </c>
       <c r="G27" t="n">
-        <v>11.8</v>
+        <v>5.7</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>18.68</v>
+        <v>17.01</v>
       </c>
       <c r="D28" t="n">
-        <v>1.43</v>
+        <v>3.18</v>
       </c>
       <c r="E28" t="n">
-        <v>5</v>
+        <v>0.7</v>
       </c>
       <c r="F28" t="n">
-        <v>11.5</v>
+        <v>7.1</v>
       </c>
       <c r="G28" t="n">
-        <v>9.6</v>
+        <v>5.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>22.47</v>
+        <v>39.89</v>
       </c>
       <c r="D29" t="n">
-        <v>2.02</v>
+        <v>3.72</v>
       </c>
       <c r="E29" t="n">
-        <v>16.5</v>
+        <v>0.7</v>
       </c>
       <c r="F29" t="n">
-        <v>6.5</v>
+        <v>7.1</v>
       </c>
       <c r="G29" t="n">
-        <v>9.5</v>
+        <v>5.2</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>40.18</v>
+        <v>22.19</v>
       </c>
       <c r="D30" t="n">
-        <v>3.74</v>
+        <v>1.99</v>
       </c>
       <c r="E30" t="n">
-        <v>2.9</v>
+        <v>12.1</v>
       </c>
       <c r="F30" t="n">
-        <v>10.8</v>
+        <v>1.4</v>
       </c>
       <c r="G30" t="n">
-        <v>8.4</v>
+        <v>4.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>17.15</v>
+        <v>18.47</v>
       </c>
       <c r="D31" t="n">
-        <v>3.21</v>
+        <v>1.41</v>
       </c>
       <c r="E31" t="n">
         <v>0.7</v>
       </c>
       <c r="F31" t="n">
-        <v>8.300000000000001</v>
+        <v>4.6</v>
       </c>
       <c r="G31" t="n">
-        <v>6</v>
+        <v>3.5</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25.95</v>
+        <v>25.52</v>
       </c>
       <c r="D32" t="n">
-        <v>2.92</v>
+        <v>2.87</v>
       </c>
       <c r="E32" t="n">
-        <v>2.9</v>
+        <v>0.7</v>
       </c>
       <c r="F32" t="n">
-        <v>2.9</v>
+        <v>0.7</v>
       </c>
       <c r="G32" t="n">
-        <v>2.9</v>
+        <v>0.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Wed Sep 16 14:22:24 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.34</v>
+        <v>7.3</v>
       </c>
       <c r="D2" t="n">
         <v>0.6899999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>92.90000000000001</v>
+        <v>90.8</v>
       </c>
       <c r="F2" t="n">
-        <v>92.90000000000001</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>92.90000000000001</v>
+        <v>91.7</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="3">
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.24</v>
+        <v>20.12</v>
       </c>
       <c r="D3" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="E3" t="n">
-        <v>76.40000000000001</v>
+        <v>69.5</v>
       </c>
       <c r="F3" t="n">
-        <v>60.4</v>
+        <v>54.6</v>
       </c>
       <c r="G3" t="n">
-        <v>68.40000000000001</v>
+        <v>62.1</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="4">
@@ -546,292 +546,292 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>33.33</v>
+        <v>33.66</v>
       </c>
       <c r="D4" t="n">
-        <v>2.08</v>
+        <v>2.1</v>
       </c>
       <c r="E4" t="n">
-        <v>26.4</v>
+        <v>34</v>
       </c>
       <c r="F4" t="n">
-        <v>71.09999999999999</v>
+        <v>74.5</v>
       </c>
       <c r="G4" t="n">
-        <v>48.8</v>
+        <v>54.3</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>16.8</v>
+        <v>29.81</v>
       </c>
       <c r="D5" t="n">
-        <v>1.81</v>
+        <v>2.86</v>
       </c>
       <c r="E5" t="n">
-        <v>12.1</v>
+        <v>44.7</v>
       </c>
       <c r="F5" t="n">
-        <v>77.90000000000001</v>
+        <v>49.3</v>
       </c>
       <c r="G5" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>19.71</v>
+        <v>16.8</v>
       </c>
       <c r="D6" t="n">
-        <v>3.53</v>
+        <v>1.81</v>
       </c>
       <c r="E6" t="n">
-        <v>32.9</v>
+        <v>12.4</v>
       </c>
       <c r="F6" t="n">
-        <v>52.1</v>
+        <v>77.7</v>
       </c>
       <c r="G6" t="n">
-        <v>42.5</v>
+        <v>45</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>20.33</v>
+        <v>21.85</v>
       </c>
       <c r="D7" t="n">
-        <v>1.72</v>
+        <v>2.03</v>
       </c>
       <c r="E7" t="n">
-        <v>77.90000000000001</v>
+        <v>37.6</v>
       </c>
       <c r="F7" t="n">
-        <v>25</v>
+        <v>47.5</v>
       </c>
       <c r="G7" t="n">
-        <v>40.9</v>
+        <v>42.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>15.25</v>
+        <v>20.34</v>
       </c>
       <c r="D8" t="n">
-        <v>2.34</v>
+        <v>1.72</v>
       </c>
       <c r="E8" t="n">
-        <v>26.4</v>
+        <v>78</v>
       </c>
       <c r="F8" t="n">
-        <v>53.2</v>
+        <v>25.2</v>
       </c>
       <c r="G8" t="n">
-        <v>39.8</v>
+        <v>41</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>14.42</v>
+        <v>19.56</v>
       </c>
       <c r="D9" t="n">
-        <v>1.22</v>
+        <v>1.63</v>
       </c>
       <c r="E9" t="n">
-        <v>19.3</v>
+        <v>43.3</v>
       </c>
       <c r="F9" t="n">
-        <v>50.7</v>
+        <v>37.9</v>
       </c>
       <c r="G9" t="n">
-        <v>35</v>
+        <v>40.6</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>21.65</v>
+        <v>19.61</v>
       </c>
       <c r="D10" t="n">
-        <v>2.01</v>
+        <v>3.52</v>
       </c>
       <c r="E10" t="n">
-        <v>26.4</v>
+        <v>30.5</v>
       </c>
       <c r="F10" t="n">
-        <v>40</v>
+        <v>48.9</v>
       </c>
       <c r="G10" t="n">
-        <v>33.2</v>
+        <v>39.7</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>12.71</v>
+        <v>27.34</v>
       </c>
       <c r="D11" t="n">
-        <v>1.33</v>
+        <v>2.63</v>
       </c>
       <c r="E11" t="n">
-        <v>15</v>
+        <v>24.1</v>
       </c>
       <c r="F11" t="n">
-        <v>49.6</v>
+        <v>48.6</v>
       </c>
       <c r="G11" t="n">
-        <v>32.3</v>
+        <v>36.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>27.2</v>
+        <v>15.11</v>
       </c>
       <c r="D12" t="n">
-        <v>2.61</v>
+        <v>2.32</v>
       </c>
       <c r="E12" t="n">
-        <v>22.1</v>
+        <v>14.9</v>
       </c>
       <c r="F12" t="n">
-        <v>41.8</v>
+        <v>51.8</v>
       </c>
       <c r="G12" t="n">
-        <v>32</v>
+        <v>33.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>19.4</v>
+        <v>52.56</v>
       </c>
       <c r="D13" t="n">
-        <v>1.62</v>
+        <v>7.8</v>
       </c>
       <c r="E13" t="n">
-        <v>31.1</v>
+        <v>10.6</v>
       </c>
       <c r="F13" t="n">
-        <v>30</v>
+        <v>51.1</v>
       </c>
       <c r="G13" t="n">
-        <v>30.5</v>
+        <v>30.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="14">
@@ -846,172 +846,172 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>32.45</v>
+        <v>32.36</v>
       </c>
       <c r="D14" t="n">
-        <v>1.95</v>
+        <v>1.94</v>
       </c>
       <c r="E14" t="n">
-        <v>85.7</v>
+        <v>83.7</v>
       </c>
       <c r="F14" t="n">
-        <v>6.4</v>
+        <v>5.7</v>
       </c>
       <c r="G14" t="n">
-        <v>30.2</v>
+        <v>29.1</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>29.09</v>
+        <v>12.52</v>
       </c>
       <c r="D15" t="n">
-        <v>2.79</v>
+        <v>1.32</v>
       </c>
       <c r="E15" t="n">
-        <v>19.6</v>
+        <v>12.8</v>
       </c>
       <c r="F15" t="n">
-        <v>29.6</v>
+        <v>44</v>
       </c>
       <c r="G15" t="n">
-        <v>26.6</v>
+        <v>28.4</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>21.13</v>
+        <v>14.35</v>
       </c>
       <c r="D16" t="n">
-        <v>1.8</v>
+        <v>1.21</v>
       </c>
       <c r="E16" t="n">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="F16" t="n">
-        <v>25.7</v>
+        <v>38.7</v>
       </c>
       <c r="G16" t="n">
-        <v>22.5</v>
+        <v>26.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>23.18</v>
+        <v>36.81</v>
       </c>
       <c r="D17" t="n">
-        <v>1.94</v>
+        <v>3.23</v>
       </c>
       <c r="E17" t="n">
-        <v>12.1</v>
+        <v>18.4</v>
       </c>
       <c r="F17" t="n">
-        <v>31.8</v>
+        <v>25.2</v>
       </c>
       <c r="G17" t="n">
-        <v>22</v>
+        <v>23.2</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>50.9</v>
+        <v>21.21</v>
       </c>
       <c r="D18" t="n">
-        <v>7.55</v>
+        <v>1.8</v>
       </c>
       <c r="E18" t="n">
-        <v>3.6</v>
+        <v>15.6</v>
       </c>
       <c r="F18" t="n">
-        <v>36.4</v>
+        <v>25.9</v>
       </c>
       <c r="G18" t="n">
-        <v>20</v>
+        <v>22.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>36.34</v>
+        <v>23.16</v>
       </c>
       <c r="D19" t="n">
-        <v>3.19</v>
+        <v>1.94</v>
       </c>
       <c r="E19" t="n">
-        <v>13.6</v>
+        <v>11.3</v>
       </c>
       <c r="F19" t="n">
-        <v>18.6</v>
+        <v>31.9</v>
       </c>
       <c r="G19" t="n">
-        <v>17.1</v>
+        <v>21.6</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="20">
@@ -1026,22 +1026,22 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>29.14</v>
+        <v>29.29</v>
       </c>
       <c r="D20" t="n">
-        <v>2.29</v>
+        <v>2.3</v>
       </c>
       <c r="E20" t="n">
-        <v>11.4</v>
+        <v>12.4</v>
       </c>
       <c r="F20" t="n">
-        <v>18.6</v>
+        <v>22.7</v>
       </c>
       <c r="G20" t="n">
-        <v>16.4</v>
+        <v>19.6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="21">
@@ -1056,22 +1056,22 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>51.55</v>
+        <v>51.71</v>
       </c>
       <c r="D21" t="n">
-        <v>3.53</v>
+        <v>3.54</v>
       </c>
       <c r="E21" t="n">
-        <v>5</v>
+        <v>8.5</v>
       </c>
       <c r="F21" t="n">
-        <v>19.3</v>
+        <v>21.3</v>
       </c>
       <c r="G21" t="n">
-        <v>15</v>
+        <v>17.4</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="22">
@@ -1086,292 +1086,292 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>66.87</v>
+        <v>67.95999999999999</v>
       </c>
       <c r="D22" t="n">
-        <v>3.55</v>
+        <v>3.61</v>
       </c>
       <c r="E22" t="n">
-        <v>4.3</v>
+        <v>5.7</v>
       </c>
       <c r="F22" t="n">
-        <v>16.4</v>
+        <v>20.6</v>
       </c>
       <c r="G22" t="n">
-        <v>12.8</v>
+        <v>16.1</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>10.5</v>
+        <v>22.27</v>
       </c>
       <c r="D23" t="n">
-        <v>0.62</v>
+        <v>2.32</v>
       </c>
       <c r="E23" t="n">
-        <v>37.9</v>
+        <v>4.3</v>
       </c>
       <c r="F23" t="n">
-        <v>0.7</v>
+        <v>18.1</v>
       </c>
       <c r="G23" t="n">
-        <v>11.9</v>
+        <v>13.9</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>22.08</v>
+        <v>10.52</v>
       </c>
       <c r="D24" t="n">
-        <v>2.3</v>
+        <v>0.62</v>
       </c>
       <c r="E24" t="n">
-        <v>2.9</v>
+        <v>38.3</v>
       </c>
       <c r="F24" t="n">
-        <v>14.3</v>
+        <v>1.1</v>
       </c>
       <c r="G24" t="n">
-        <v>10.9</v>
+        <v>12.2</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>8.300000000000001</v>
+        <v>25.64</v>
       </c>
       <c r="D25" t="n">
-        <v>0.92</v>
+        <v>2.3</v>
       </c>
       <c r="E25" t="n">
-        <v>2.9</v>
+        <v>1.4</v>
       </c>
       <c r="F25" t="n">
-        <v>10.7</v>
+        <v>15.6</v>
       </c>
       <c r="G25" t="n">
-        <v>8.4</v>
+        <v>11.3</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>7.68</v>
+        <v>17.3</v>
       </c>
       <c r="D26" t="n">
-        <v>1.19</v>
+        <v>3.24</v>
       </c>
       <c r="E26" t="n">
-        <v>0.7</v>
+        <v>4.3</v>
       </c>
       <c r="F26" t="n">
-        <v>10</v>
+        <v>13.8</v>
       </c>
       <c r="G26" t="n">
-        <v>7.2</v>
+        <v>11</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>25.4</v>
+        <v>18.64</v>
       </c>
       <c r="D27" t="n">
-        <v>2.27</v>
+        <v>1.43</v>
       </c>
       <c r="E27" t="n">
-        <v>0.7</v>
+        <v>5.7</v>
       </c>
       <c r="F27" t="n">
-        <v>7.9</v>
+        <v>12.4</v>
       </c>
       <c r="G27" t="n">
-        <v>5.7</v>
+        <v>10.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>17.01</v>
+        <v>40.21</v>
       </c>
       <c r="D28" t="n">
-        <v>3.18</v>
+        <v>3.75</v>
       </c>
       <c r="E28" t="n">
-        <v>0.7</v>
+        <v>4.3</v>
       </c>
       <c r="F28" t="n">
-        <v>7.1</v>
+        <v>12.4</v>
       </c>
       <c r="G28" t="n">
-        <v>5.2</v>
+        <v>10</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>39.89</v>
+        <v>8.34</v>
       </c>
       <c r="D29" t="n">
-        <v>3.72</v>
+        <v>0.92</v>
       </c>
       <c r="E29" t="n">
-        <v>0.7</v>
+        <v>3.5</v>
       </c>
       <c r="F29" t="n">
-        <v>7.1</v>
+        <v>11</v>
       </c>
       <c r="G29" t="n">
-        <v>5.2</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>22.19</v>
+        <v>7.67</v>
       </c>
       <c r="D30" t="n">
-        <v>1.99</v>
+        <v>1.19</v>
       </c>
       <c r="E30" t="n">
-        <v>12.1</v>
+        <v>0.7</v>
       </c>
       <c r="F30" t="n">
-        <v>1.4</v>
+        <v>10.3</v>
       </c>
       <c r="G30" t="n">
-        <v>4.6</v>
+        <v>7.4</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>18.47</v>
+        <v>22.1</v>
       </c>
       <c r="D31" t="n">
-        <v>1.41</v>
+        <v>1.98</v>
       </c>
       <c r="E31" t="n">
-        <v>0.7</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F31" t="n">
-        <v>4.6</v>
+        <v>1.4</v>
       </c>
       <c r="G31" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="32">
@@ -1386,7 +1386,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25.52</v>
+        <v>25.46</v>
       </c>
       <c r="D32" t="n">
         <v>2.87</v>
@@ -1395,13 +1395,13 @@
         <v>0.7</v>
       </c>
       <c r="F32" t="n">
-        <v>0.7</v>
+        <v>1.1</v>
       </c>
       <c r="G32" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu Sep 17 14:28:11 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.3</v>
+        <v>7.31</v>
       </c>
       <c r="D2" t="n">
         <v>0.6899999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>90.8</v>
+        <v>91.2</v>
       </c>
       <c r="F2" t="n">
-        <v>92.59999999999999</v>
+        <v>92.3</v>
       </c>
       <c r="G2" t="n">
         <v>91.7</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="3">
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.12</v>
+        <v>19.94</v>
       </c>
       <c r="D3" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="E3" t="n">
-        <v>69.5</v>
+        <v>68.7</v>
       </c>
       <c r="F3" t="n">
-        <v>54.6</v>
+        <v>49.6</v>
       </c>
       <c r="G3" t="n">
-        <v>62.1</v>
+        <v>59.2</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="4">
@@ -546,22 +546,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>33.66</v>
+        <v>33.87</v>
       </c>
       <c r="D4" t="n">
-        <v>2.1</v>
+        <v>2.12</v>
       </c>
       <c r="E4" t="n">
-        <v>34</v>
+        <v>37.3</v>
       </c>
       <c r="F4" t="n">
-        <v>74.5</v>
+        <v>76.8</v>
       </c>
       <c r="G4" t="n">
-        <v>54.3</v>
+        <v>57</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="5">
@@ -576,202 +576,202 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>29.81</v>
+        <v>29.89</v>
       </c>
       <c r="D5" t="n">
-        <v>2.86</v>
+        <v>2.87</v>
       </c>
       <c r="E5" t="n">
-        <v>44.7</v>
+        <v>46.5</v>
       </c>
       <c r="F5" t="n">
-        <v>49.3</v>
+        <v>50.7</v>
       </c>
       <c r="G5" t="n">
-        <v>47</v>
+        <v>48.6</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>16.8</v>
+        <v>21.84</v>
       </c>
       <c r="D6" t="n">
-        <v>1.81</v>
+        <v>2.03</v>
       </c>
       <c r="E6" t="n">
-        <v>12.4</v>
+        <v>37.3</v>
       </c>
       <c r="F6" t="n">
-        <v>77.7</v>
+        <v>47.5</v>
       </c>
       <c r="G6" t="n">
-        <v>45</v>
+        <v>42.4</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>21.85</v>
+        <v>19.66</v>
       </c>
       <c r="D7" t="n">
-        <v>2.03</v>
+        <v>3.52</v>
       </c>
       <c r="E7" t="n">
-        <v>37.6</v>
+        <v>31.3</v>
       </c>
       <c r="F7" t="n">
-        <v>47.5</v>
+        <v>48.9</v>
       </c>
       <c r="G7" t="n">
-        <v>42.6</v>
+        <v>40.1</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>20.34</v>
+        <v>16.64</v>
       </c>
       <c r="D8" t="n">
-        <v>1.72</v>
+        <v>1.8</v>
       </c>
       <c r="E8" t="n">
-        <v>78</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F8" t="n">
-        <v>25.2</v>
+        <v>70.8</v>
       </c>
       <c r="G8" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>19.56</v>
+        <v>27.49</v>
       </c>
       <c r="D9" t="n">
-        <v>1.63</v>
+        <v>2.64</v>
       </c>
       <c r="E9" t="n">
-        <v>43.3</v>
+        <v>26.1</v>
       </c>
       <c r="F9" t="n">
-        <v>37.9</v>
+        <v>52.8</v>
       </c>
       <c r="G9" t="n">
-        <v>40.6</v>
+        <v>39.4</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>19.61</v>
+        <v>14.48</v>
       </c>
       <c r="D10" t="n">
-        <v>3.52</v>
+        <v>1.22</v>
       </c>
       <c r="E10" t="n">
-        <v>30.5</v>
+        <v>26.1</v>
       </c>
       <c r="F10" t="n">
-        <v>48.9</v>
+        <v>51.1</v>
       </c>
       <c r="G10" t="n">
-        <v>39.7</v>
+        <v>38.6</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>27.34</v>
+        <v>19.49</v>
       </c>
       <c r="D11" t="n">
-        <v>2.63</v>
+        <v>1.63</v>
       </c>
       <c r="E11" t="n">
-        <v>24.1</v>
+        <v>36.3</v>
       </c>
       <c r="F11" t="n">
-        <v>48.6</v>
+        <v>38</v>
       </c>
       <c r="G11" t="n">
-        <v>36.3</v>
+        <v>37.1</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="12">
@@ -786,52 +786,52 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>15.11</v>
+        <v>15.15</v>
       </c>
       <c r="D12" t="n">
         <v>2.32</v>
       </c>
       <c r="E12" t="n">
-        <v>14.9</v>
+        <v>19</v>
       </c>
       <c r="F12" t="n">
         <v>51.8</v>
       </c>
       <c r="G12" t="n">
-        <v>33.3</v>
+        <v>35.4</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>52.56</v>
+        <v>37.12</v>
       </c>
       <c r="D13" t="n">
-        <v>7.8</v>
+        <v>3.26</v>
       </c>
       <c r="E13" t="n">
-        <v>10.6</v>
+        <v>25</v>
       </c>
       <c r="F13" t="n">
-        <v>51.1</v>
+        <v>37.3</v>
       </c>
       <c r="G13" t="n">
-        <v>30.9</v>
+        <v>31.2</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="14">
@@ -846,112 +846,112 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>32.36</v>
+        <v>32.59</v>
       </c>
       <c r="D14" t="n">
-        <v>1.94</v>
+        <v>1.95</v>
       </c>
       <c r="E14" t="n">
-        <v>83.7</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>5.7</v>
+        <v>7.4</v>
       </c>
       <c r="G14" t="n">
-        <v>29.1</v>
+        <v>31</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>12.52</v>
+        <v>51.86</v>
       </c>
       <c r="D15" t="n">
-        <v>1.32</v>
+        <v>7.69</v>
       </c>
       <c r="E15" t="n">
-        <v>12.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F15" t="n">
-        <v>44</v>
+        <v>48.2</v>
       </c>
       <c r="G15" t="n">
-        <v>28.4</v>
+        <v>28.7</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>14.35</v>
+        <v>20.09</v>
       </c>
       <c r="D16" t="n">
-        <v>1.21</v>
+        <v>1.7</v>
       </c>
       <c r="E16" t="n">
-        <v>14.9</v>
+        <v>64.8</v>
       </c>
       <c r="F16" t="n">
-        <v>38.7</v>
+        <v>12</v>
       </c>
       <c r="G16" t="n">
-        <v>26.8</v>
+        <v>27.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>36.81</v>
+        <v>23.27</v>
       </c>
       <c r="D17" t="n">
-        <v>3.23</v>
+        <v>1.95</v>
       </c>
       <c r="E17" t="n">
-        <v>18.4</v>
+        <v>16.2</v>
       </c>
       <c r="F17" t="n">
-        <v>25.2</v>
+        <v>35.9</v>
       </c>
       <c r="G17" t="n">
-        <v>23.2</v>
+        <v>26.1</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="18">
@@ -966,52 +966,52 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>21.21</v>
+        <v>21.27</v>
       </c>
       <c r="D18" t="n">
-        <v>1.8</v>
+        <v>1.81</v>
       </c>
       <c r="E18" t="n">
-        <v>15.6</v>
+        <v>16.9</v>
       </c>
       <c r="F18" t="n">
-        <v>25.9</v>
+        <v>31</v>
       </c>
       <c r="G18" t="n">
-        <v>22.8</v>
+        <v>23.9</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>23.16</v>
+        <v>12.33</v>
       </c>
       <c r="D19" t="n">
-        <v>1.94</v>
+        <v>1.3</v>
       </c>
       <c r="E19" t="n">
         <v>11.3</v>
       </c>
       <c r="F19" t="n">
-        <v>31.9</v>
+        <v>32</v>
       </c>
       <c r="G19" t="n">
-        <v>21.6</v>
+        <v>21.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="20">
@@ -1026,22 +1026,22 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>29.29</v>
+        <v>29.37</v>
       </c>
       <c r="D20" t="n">
         <v>2.3</v>
       </c>
       <c r="E20" t="n">
-        <v>12.4</v>
+        <v>15.5</v>
       </c>
       <c r="F20" t="n">
-        <v>22.7</v>
+        <v>22.9</v>
       </c>
       <c r="G20" t="n">
-        <v>19.6</v>
+        <v>20.7</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="21">
@@ -1056,7 +1056,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>51.71</v>
+        <v>51.69</v>
       </c>
       <c r="D21" t="n">
         <v>3.54</v>
@@ -1065,13 +1065,13 @@
         <v>8.5</v>
       </c>
       <c r="F21" t="n">
-        <v>21.3</v>
+        <v>21.5</v>
       </c>
       <c r="G21" t="n">
-        <v>17.4</v>
+        <v>17.6</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="22">
@@ -1086,22 +1086,22 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>67.95999999999999</v>
+        <v>67.79000000000001</v>
       </c>
       <c r="D22" t="n">
-        <v>3.61</v>
+        <v>3.6</v>
       </c>
       <c r="E22" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="F22" t="n">
-        <v>20.6</v>
+        <v>18.3</v>
       </c>
       <c r="G22" t="n">
-        <v>16.1</v>
+        <v>14.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="23">
@@ -1116,22 +1116,22 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>22.27</v>
+        <v>22.11</v>
       </c>
       <c r="D23" t="n">
-        <v>2.32</v>
+        <v>2.31</v>
       </c>
       <c r="E23" t="n">
-        <v>4.3</v>
+        <v>3.5</v>
       </c>
       <c r="F23" t="n">
-        <v>18.1</v>
+        <v>16.9</v>
       </c>
       <c r="G23" t="n">
-        <v>13.9</v>
+        <v>12.9</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="24">
@@ -1146,22 +1146,22 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>10.52</v>
+        <v>10.56</v>
       </c>
       <c r="D24" t="n">
         <v>0.62</v>
       </c>
       <c r="E24" t="n">
-        <v>38.3</v>
+        <v>39.1</v>
       </c>
       <c r="F24" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="G24" t="n">
-        <v>12.2</v>
+        <v>12.7</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="25">
@@ -1176,142 +1176,142 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>25.64</v>
+        <v>25.7</v>
       </c>
       <c r="D25" t="n">
         <v>2.3</v>
       </c>
       <c r="E25" t="n">
-        <v>1.4</v>
+        <v>2.1</v>
       </c>
       <c r="F25" t="n">
-        <v>15.6</v>
+        <v>15.8</v>
       </c>
       <c r="G25" t="n">
-        <v>11.3</v>
+        <v>11.7</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>17.3</v>
+        <v>22.43</v>
       </c>
       <c r="D26" t="n">
-        <v>3.24</v>
+        <v>2.01</v>
       </c>
       <c r="E26" t="n">
-        <v>4.3</v>
+        <v>17.6</v>
       </c>
       <c r="F26" t="n">
-        <v>13.8</v>
+        <v>6</v>
       </c>
       <c r="G26" t="n">
-        <v>11</v>
+        <v>9.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>18.64</v>
+        <v>8.33</v>
       </c>
       <c r="D27" t="n">
-        <v>1.43</v>
+        <v>0.92</v>
       </c>
       <c r="E27" t="n">
-        <v>5.7</v>
+        <v>3.5</v>
       </c>
       <c r="F27" t="n">
-        <v>12.4</v>
+        <v>11.3</v>
       </c>
       <c r="G27" t="n">
-        <v>10.4</v>
+        <v>8.9</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>40.21</v>
+        <v>18.54</v>
       </c>
       <c r="D28" t="n">
-        <v>3.75</v>
+        <v>1.42</v>
       </c>
       <c r="E28" t="n">
-        <v>4.3</v>
+        <v>1.4</v>
       </c>
       <c r="F28" t="n">
-        <v>12.4</v>
+        <v>8.1</v>
       </c>
       <c r="G28" t="n">
-        <v>10</v>
+        <v>6.1</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>8.34</v>
+        <v>39.94</v>
       </c>
       <c r="D29" t="n">
-        <v>0.92</v>
+        <v>3.72</v>
       </c>
       <c r="E29" t="n">
-        <v>3.5</v>
+        <v>1.4</v>
       </c>
       <c r="F29" t="n">
-        <v>11</v>
+        <v>7.4</v>
       </c>
       <c r="G29" t="n">
-        <v>8.800000000000001</v>
+        <v>5.6</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="30">
@@ -1326,52 +1326,52 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>7.67</v>
+        <v>7.62</v>
       </c>
       <c r="D30" t="n">
-        <v>1.19</v>
+        <v>1.18</v>
       </c>
       <c r="E30" t="n">
         <v>0.7</v>
       </c>
       <c r="F30" t="n">
-        <v>10.3</v>
+        <v>6.7</v>
       </c>
       <c r="G30" t="n">
-        <v>7.4</v>
+        <v>4.9</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>22.1</v>
+        <v>16.85</v>
       </c>
       <c r="D31" t="n">
-        <v>1.98</v>
+        <v>3.15</v>
       </c>
       <c r="E31" t="n">
-        <v>8.199999999999999</v>
+        <v>0.7</v>
       </c>
       <c r="F31" t="n">
-        <v>1.4</v>
+        <v>4.2</v>
       </c>
       <c r="G31" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25.46</v>
+        <v>25.36</v>
       </c>
       <c r="D32" t="n">
-        <v>2.87</v>
+        <v>2.86</v>
       </c>
       <c r="E32" t="n">
         <v>0.7</v>
       </c>
       <c r="F32" t="n">
-        <v>1.1</v>
+        <v>0.7</v>
       </c>
       <c r="G32" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri Sep 18 13:52:47 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.31</v>
+        <v>7.26</v>
       </c>
       <c r="D2" t="n">
         <v>0.6899999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>91.2</v>
+        <v>88.5</v>
       </c>
       <c r="F2" t="n">
-        <v>92.3</v>
+        <v>92</v>
       </c>
       <c r="G2" t="n">
-        <v>91.7</v>
+        <v>90.2</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="3">
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>19.94</v>
+        <v>20.13</v>
       </c>
       <c r="D3" t="n">
-        <v>0.97</v>
+        <v>0.99</v>
       </c>
       <c r="E3" t="n">
-        <v>68.7</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>49.6</v>
+        <v>60.8</v>
       </c>
       <c r="G3" t="n">
-        <v>59.2</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="4">
@@ -546,142 +546,142 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>33.87</v>
+        <v>33.79</v>
       </c>
       <c r="D4" t="n">
-        <v>2.12</v>
+        <v>2.11</v>
       </c>
       <c r="E4" t="n">
-        <v>37.3</v>
+        <v>37.1</v>
       </c>
       <c r="F4" t="n">
-        <v>76.8</v>
+        <v>75.2</v>
       </c>
       <c r="G4" t="n">
-        <v>57</v>
+        <v>56.1</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>29.89</v>
+        <v>38.76</v>
       </c>
       <c r="D5" t="n">
-        <v>2.87</v>
+        <v>3.41</v>
       </c>
       <c r="E5" t="n">
-        <v>46.5</v>
+        <v>51.7</v>
       </c>
       <c r="F5" t="n">
-        <v>50.7</v>
+        <v>55.6</v>
       </c>
       <c r="G5" t="n">
-        <v>48.6</v>
+        <v>53.7</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>21.84</v>
+        <v>19.71</v>
       </c>
       <c r="D6" t="n">
-        <v>2.03</v>
+        <v>1.65</v>
       </c>
       <c r="E6" t="n">
-        <v>37.3</v>
+        <v>54.5</v>
       </c>
       <c r="F6" t="n">
-        <v>47.5</v>
+        <v>48.6</v>
       </c>
       <c r="G6" t="n">
-        <v>42.4</v>
+        <v>51.6</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>19.66</v>
+        <v>30.29</v>
       </c>
       <c r="D7" t="n">
-        <v>3.52</v>
+        <v>2.9</v>
       </c>
       <c r="E7" t="n">
-        <v>31.3</v>
+        <v>49</v>
       </c>
       <c r="F7" t="n">
-        <v>48.9</v>
+        <v>51.7</v>
       </c>
       <c r="G7" t="n">
-        <v>40.1</v>
+        <v>50.3</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>16.64</v>
+        <v>22.1</v>
       </c>
       <c r="D8" t="n">
-        <v>1.8</v>
+        <v>2.06</v>
       </c>
       <c r="E8" t="n">
-        <v>9.199999999999999</v>
+        <v>44.8</v>
       </c>
       <c r="F8" t="n">
-        <v>70.8</v>
+        <v>53.1</v>
       </c>
       <c r="G8" t="n">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="9">
@@ -696,82 +696,82 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>27.49</v>
+        <v>27.75</v>
       </c>
       <c r="D9" t="n">
-        <v>2.64</v>
+        <v>2.67</v>
       </c>
       <c r="E9" t="n">
-        <v>26.1</v>
+        <v>29.4</v>
       </c>
       <c r="F9" t="n">
-        <v>52.8</v>
+        <v>58</v>
       </c>
       <c r="G9" t="n">
-        <v>39.4</v>
+        <v>43.7</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>14.48</v>
+        <v>19.67</v>
       </c>
       <c r="D10" t="n">
-        <v>1.22</v>
+        <v>3.53</v>
       </c>
       <c r="E10" t="n">
-        <v>26.1</v>
+        <v>32.2</v>
       </c>
       <c r="F10" t="n">
-        <v>51.1</v>
+        <v>52.8</v>
       </c>
       <c r="G10" t="n">
-        <v>38.6</v>
+        <v>42.5</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>19.49</v>
+        <v>14.47</v>
       </c>
       <c r="D11" t="n">
-        <v>1.63</v>
+        <v>1.22</v>
       </c>
       <c r="E11" t="n">
-        <v>36.3</v>
+        <v>24.1</v>
       </c>
       <c r="F11" t="n">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="G11" t="n">
-        <v>37.1</v>
+        <v>37.6</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="12">
@@ -786,82 +786,82 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>15.15</v>
+        <v>15.2</v>
       </c>
       <c r="D12" t="n">
-        <v>2.32</v>
+        <v>2.33</v>
       </c>
       <c r="E12" t="n">
-        <v>19</v>
+        <v>22.4</v>
       </c>
       <c r="F12" t="n">
-        <v>51.8</v>
+        <v>52.4</v>
       </c>
       <c r="G12" t="n">
-        <v>35.4</v>
+        <v>37.4</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>37.12</v>
+        <v>32.78</v>
       </c>
       <c r="D13" t="n">
-        <v>3.26</v>
+        <v>1.97</v>
       </c>
       <c r="E13" t="n">
-        <v>25</v>
+        <v>86</v>
       </c>
       <c r="F13" t="n">
-        <v>37.3</v>
+        <v>14.3</v>
       </c>
       <c r="G13" t="n">
-        <v>31.2</v>
+        <v>35.8</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>32.59</v>
+        <v>16.51</v>
       </c>
       <c r="D14" t="n">
-        <v>1.95</v>
+        <v>1.78</v>
       </c>
       <c r="E14" t="n">
-        <v>85.90000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="F14" t="n">
-        <v>7.4</v>
+        <v>62.9</v>
       </c>
       <c r="G14" t="n">
-        <v>31</v>
+        <v>35.7</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="15">
@@ -876,202 +876,202 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>51.86</v>
+        <v>53.46</v>
       </c>
       <c r="D15" t="n">
-        <v>7.69</v>
+        <v>7.93</v>
       </c>
       <c r="E15" t="n">
-        <v>9.199999999999999</v>
+        <v>12.6</v>
       </c>
       <c r="F15" t="n">
-        <v>48.2</v>
+        <v>55.9</v>
       </c>
       <c r="G15" t="n">
-        <v>28.7</v>
+        <v>34.3</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>20.09</v>
+        <v>21.65</v>
       </c>
       <c r="D16" t="n">
-        <v>1.7</v>
+        <v>1.84</v>
       </c>
       <c r="E16" t="n">
-        <v>64.8</v>
+        <v>28.7</v>
       </c>
       <c r="F16" t="n">
-        <v>12</v>
+        <v>38.5</v>
       </c>
       <c r="G16" t="n">
-        <v>27.8</v>
+        <v>33.6</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>23.27</v>
+        <v>20.19</v>
       </c>
       <c r="D17" t="n">
-        <v>1.95</v>
+        <v>1.71</v>
       </c>
       <c r="E17" t="n">
-        <v>16.2</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="F17" t="n">
-        <v>35.9</v>
+        <v>18.2</v>
       </c>
       <c r="G17" t="n">
-        <v>26.1</v>
+        <v>32.9</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>21.27</v>
+        <v>23.53</v>
       </c>
       <c r="D18" t="n">
-        <v>1.81</v>
+        <v>1.97</v>
       </c>
       <c r="E18" t="n">
-        <v>16.9</v>
+        <v>24.5</v>
       </c>
       <c r="F18" t="n">
-        <v>31</v>
+        <v>39.9</v>
       </c>
       <c r="G18" t="n">
-        <v>23.9</v>
+        <v>32.2</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>12.33</v>
+        <v>29.66</v>
       </c>
       <c r="D19" t="n">
-        <v>1.3</v>
+        <v>2.33</v>
       </c>
       <c r="E19" t="n">
-        <v>11.3</v>
+        <v>21.7</v>
       </c>
       <c r="F19" t="n">
-        <v>32</v>
+        <v>34.3</v>
       </c>
       <c r="G19" t="n">
-        <v>21.7</v>
+        <v>28</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>29.37</v>
+        <v>52.54</v>
       </c>
       <c r="D20" t="n">
-        <v>2.3</v>
+        <v>3.6</v>
       </c>
       <c r="E20" t="n">
-        <v>15.5</v>
+        <v>16.1</v>
       </c>
       <c r="F20" t="n">
-        <v>22.9</v>
+        <v>31.5</v>
       </c>
       <c r="G20" t="n">
-        <v>20.7</v>
+        <v>23.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>51.69</v>
+        <v>12.28</v>
       </c>
       <c r="D21" t="n">
-        <v>3.54</v>
+        <v>1.29</v>
       </c>
       <c r="E21" t="n">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="F21" t="n">
-        <v>21.5</v>
+        <v>27.3</v>
       </c>
       <c r="G21" t="n">
-        <v>17.6</v>
+        <v>21.6</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="22">
@@ -1086,52 +1086,52 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>67.79000000000001</v>
+        <v>68.48999999999999</v>
       </c>
       <c r="D22" t="n">
-        <v>3.6</v>
+        <v>3.63</v>
       </c>
       <c r="E22" t="n">
-        <v>5.6</v>
+        <v>12.6</v>
       </c>
       <c r="F22" t="n">
-        <v>18.3</v>
+        <v>25.2</v>
       </c>
       <c r="G22" t="n">
-        <v>14.5</v>
+        <v>21.4</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>22.11</v>
+        <v>8.58</v>
       </c>
       <c r="D23" t="n">
-        <v>2.31</v>
+        <v>0.95</v>
       </c>
       <c r="E23" t="n">
-        <v>3.5</v>
+        <v>9.1</v>
       </c>
       <c r="F23" t="n">
-        <v>16.9</v>
+        <v>31.5</v>
       </c>
       <c r="G23" t="n">
-        <v>12.9</v>
+        <v>20.3</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="24">
@@ -1146,22 +1146,22 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>10.56</v>
+        <v>10.64</v>
       </c>
       <c r="D24" t="n">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="E24" t="n">
-        <v>39.1</v>
+        <v>44.1</v>
       </c>
       <c r="F24" t="n">
-        <v>1.4</v>
+        <v>9.4</v>
       </c>
       <c r="G24" t="n">
-        <v>12.7</v>
+        <v>19.8</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="25">
@@ -1176,82 +1176,82 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>25.7</v>
+        <v>26.2</v>
       </c>
       <c r="D25" t="n">
-        <v>2.3</v>
+        <v>2.34</v>
       </c>
       <c r="E25" t="n">
-        <v>2.1</v>
+        <v>7.7</v>
       </c>
       <c r="F25" t="n">
-        <v>15.8</v>
+        <v>30.4</v>
       </c>
       <c r="G25" t="n">
-        <v>11.7</v>
+        <v>19.1</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>22.43</v>
+        <v>40.7</v>
       </c>
       <c r="D26" t="n">
-        <v>2.01</v>
+        <v>3.79</v>
       </c>
       <c r="E26" t="n">
-        <v>17.6</v>
+        <v>6.3</v>
       </c>
       <c r="F26" t="n">
-        <v>6</v>
+        <v>19.9</v>
       </c>
       <c r="G26" t="n">
-        <v>9.5</v>
+        <v>15.8</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>8.33</v>
+        <v>22.34</v>
       </c>
       <c r="D27" t="n">
-        <v>0.92</v>
+        <v>2.33</v>
       </c>
       <c r="E27" t="n">
-        <v>3.5</v>
+        <v>5.6</v>
       </c>
       <c r="F27" t="n">
-        <v>11.3</v>
+        <v>19.9</v>
       </c>
       <c r="G27" t="n">
-        <v>8.9</v>
+        <v>15.6</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="28">
@@ -1266,82 +1266,82 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>18.54</v>
+        <v>18.77</v>
       </c>
       <c r="D28" t="n">
-        <v>1.42</v>
+        <v>1.44</v>
       </c>
       <c r="E28" t="n">
-        <v>1.4</v>
+        <v>8.4</v>
       </c>
       <c r="F28" t="n">
-        <v>8.1</v>
+        <v>16.8</v>
       </c>
       <c r="G28" t="n">
-        <v>6.1</v>
+        <v>14.3</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>39.94</v>
+        <v>7.71</v>
       </c>
       <c r="D29" t="n">
-        <v>3.72</v>
+        <v>1.2</v>
       </c>
       <c r="E29" t="n">
-        <v>1.4</v>
+        <v>2.8</v>
       </c>
       <c r="F29" t="n">
-        <v>7.4</v>
+        <v>18.5</v>
       </c>
       <c r="G29" t="n">
-        <v>5.6</v>
+        <v>13.8</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>7.62</v>
+        <v>22.54</v>
       </c>
       <c r="D30" t="n">
-        <v>1.18</v>
+        <v>2.02</v>
       </c>
       <c r="E30" t="n">
-        <v>0.7</v>
+        <v>20.3</v>
       </c>
       <c r="F30" t="n">
-        <v>6.7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G30" t="n">
-        <v>4.9</v>
+        <v>12.2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="31">
@@ -1356,22 +1356,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>16.85</v>
+        <v>17.11</v>
       </c>
       <c r="D31" t="n">
-        <v>3.15</v>
+        <v>3.2</v>
       </c>
       <c r="E31" t="n">
-        <v>0.7</v>
+        <v>2.1</v>
       </c>
       <c r="F31" t="n">
-        <v>4.2</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G31" t="n">
-        <v>3.2</v>
+        <v>6.7</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25.36</v>
+        <v>25.79</v>
       </c>
       <c r="D32" t="n">
-        <v>2.86</v>
+        <v>2.9</v>
       </c>
       <c r="E32" t="n">
-        <v>0.7</v>
+        <v>4.9</v>
       </c>
       <c r="F32" t="n">
-        <v>0.7</v>
+        <v>3.8</v>
       </c>
       <c r="G32" t="n">
-        <v>0.7</v>
+        <v>4.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat Sep 19 13:26:44 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>88.5</v>
+        <v>88.2</v>
       </c>
       <c r="F2" t="n">
-        <v>92</v>
+        <v>91.7</v>
       </c>
       <c r="G2" t="n">
-        <v>90.2</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>0.99</v>
       </c>
       <c r="E3" t="n">
-        <v>69.90000000000001</v>
+        <v>69.8</v>
       </c>
       <c r="F3" t="n">
         <v>60.8</v>
       </c>
       <c r="G3" t="n">
-        <v>65.40000000000001</v>
+        <v>65.3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>2.11</v>
       </c>
       <c r="E4" t="n">
-        <v>37.1</v>
+        <v>37.2</v>
       </c>
       <c r="F4" t="n">
-        <v>75.2</v>
+        <v>75</v>
       </c>
       <c r="G4" t="n">
         <v>56.1</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="5">
@@ -588,10 +588,10 @@
         <v>55.6</v>
       </c>
       <c r="G5" t="n">
-        <v>53.7</v>
+        <v>53.6</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="6">
@@ -621,7 +621,7 @@
         <v>51.6</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="7">
@@ -651,7 +651,7 @@
         <v>50.3</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="8">
@@ -681,7 +681,7 @@
         <v>49</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>2.67</v>
       </c>
       <c r="E9" t="n">
-        <v>29.4</v>
+        <v>29.5</v>
       </c>
       <c r="F9" t="n">
         <v>58</v>
       </c>
       <c r="G9" t="n">
-        <v>43.7</v>
+        <v>43.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="10">
@@ -732,7 +732,7 @@
         <v>3.53</v>
       </c>
       <c r="E10" t="n">
-        <v>32.2</v>
+        <v>32.3</v>
       </c>
       <c r="F10" t="n">
         <v>52.8</v>
@@ -741,7 +741,7 @@
         <v>42.5</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.22</v>
       </c>
       <c r="E11" t="n">
-        <v>24.1</v>
+        <v>24.3</v>
       </c>
       <c r="F11" t="n">
         <v>51</v>
       </c>
       <c r="G11" t="n">
-        <v>37.6</v>
+        <v>37.7</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>2.33</v>
       </c>
       <c r="E12" t="n">
-        <v>22.4</v>
+        <v>22.6</v>
       </c>
       <c r="F12" t="n">
         <v>52.4</v>
       </c>
       <c r="G12" t="n">
-        <v>37.4</v>
+        <v>37.5</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.97</v>
       </c>
       <c r="E13" t="n">
-        <v>86</v>
+        <v>85.8</v>
       </c>
       <c r="F13" t="n">
-        <v>14.3</v>
+        <v>14.6</v>
       </c>
       <c r="G13" t="n">
-        <v>35.8</v>
+        <v>35.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.78</v>
       </c>
       <c r="E14" t="n">
-        <v>8.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F14" t="n">
-        <v>62.9</v>
+        <v>62.8</v>
       </c>
       <c r="G14" t="n">
-        <v>35.7</v>
+        <v>35.8</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>7.93</v>
       </c>
       <c r="E15" t="n">
-        <v>12.6</v>
+        <v>12.8</v>
       </c>
       <c r="F15" t="n">
         <v>55.9</v>
       </c>
       <c r="G15" t="n">
-        <v>34.3</v>
+        <v>34.4</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>1.84</v>
       </c>
       <c r="E16" t="n">
-        <v>28.7</v>
+        <v>28.8</v>
       </c>
       <c r="F16" t="n">
         <v>38.5</v>
       </c>
       <c r="G16" t="n">
-        <v>33.6</v>
+        <v>33.7</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.71</v>
       </c>
       <c r="E17" t="n">
-        <v>67.09999999999999</v>
+        <v>67</v>
       </c>
       <c r="F17" t="n">
-        <v>18.2</v>
+        <v>18.4</v>
       </c>
       <c r="G17" t="n">
-        <v>32.9</v>
+        <v>33</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>1.97</v>
       </c>
       <c r="E18" t="n">
-        <v>24.5</v>
+        <v>24.7</v>
       </c>
       <c r="F18" t="n">
         <v>39.9</v>
       </c>
       <c r="G18" t="n">
-        <v>32.2</v>
+        <v>32.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>2.33</v>
       </c>
       <c r="E19" t="n">
-        <v>21.7</v>
+        <v>21.9</v>
       </c>
       <c r="F19" t="n">
-        <v>34.3</v>
+        <v>34.4</v>
       </c>
       <c r="G19" t="n">
-        <v>28</v>
+        <v>28.1</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>3.6</v>
       </c>
       <c r="E20" t="n">
-        <v>16.1</v>
+        <v>16.3</v>
       </c>
       <c r="F20" t="n">
-        <v>31.5</v>
+        <v>31.6</v>
       </c>
       <c r="G20" t="n">
-        <v>23.8</v>
+        <v>24</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>1.29</v>
       </c>
       <c r="E21" t="n">
-        <v>8.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F21" t="n">
-        <v>27.3</v>
+        <v>27.4</v>
       </c>
       <c r="G21" t="n">
-        <v>21.6</v>
+        <v>21.8</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>3.63</v>
       </c>
       <c r="E22" t="n">
-        <v>12.6</v>
+        <v>12.8</v>
       </c>
       <c r="F22" t="n">
-        <v>25.2</v>
+        <v>25.3</v>
       </c>
       <c r="G22" t="n">
-        <v>21.4</v>
+        <v>21.6</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>0.95</v>
       </c>
       <c r="E23" t="n">
-        <v>9.1</v>
+        <v>9.4</v>
       </c>
       <c r="F23" t="n">
-        <v>31.5</v>
+        <v>31.6</v>
       </c>
       <c r="G23" t="n">
-        <v>20.3</v>
+        <v>20.5</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="24">
@@ -1155,13 +1155,13 @@
         <v>44.1</v>
       </c>
       <c r="F24" t="n">
-        <v>9.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G24" t="n">
-        <v>19.8</v>
+        <v>20</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.34</v>
       </c>
       <c r="E25" t="n">
-        <v>7.7</v>
+        <v>8</v>
       </c>
       <c r="F25" t="n">
-        <v>30.4</v>
+        <v>30.6</v>
       </c>
       <c r="G25" t="n">
-        <v>19.1</v>
+        <v>19.3</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>3.79</v>
       </c>
       <c r="E26" t="n">
-        <v>6.3</v>
+        <v>6.6</v>
       </c>
       <c r="F26" t="n">
-        <v>19.9</v>
+        <v>20.1</v>
       </c>
       <c r="G26" t="n">
-        <v>15.8</v>
+        <v>16.1</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.33</v>
       </c>
       <c r="E27" t="n">
-        <v>5.6</v>
+        <v>5.9</v>
       </c>
       <c r="F27" t="n">
-        <v>19.9</v>
+        <v>20.1</v>
       </c>
       <c r="G27" t="n">
-        <v>15.6</v>
+        <v>15.9</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>1.44</v>
       </c>
       <c r="E28" t="n">
-        <v>8.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F28" t="n">
-        <v>16.8</v>
+        <v>17</v>
       </c>
       <c r="G28" t="n">
-        <v>14.3</v>
+        <v>14.5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.2</v>
       </c>
       <c r="E29" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="F29" t="n">
-        <v>18.5</v>
+        <v>18.8</v>
       </c>
       <c r="G29" t="n">
-        <v>13.8</v>
+        <v>14.1</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>2.02</v>
       </c>
       <c r="E30" t="n">
-        <v>20.3</v>
+        <v>20.5</v>
       </c>
       <c r="F30" t="n">
-        <v>8.699999999999999</v>
+        <v>9</v>
       </c>
       <c r="G30" t="n">
-        <v>12.2</v>
+        <v>12.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.2</v>
       </c>
       <c r="E31" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="F31" t="n">
-        <v>8.699999999999999</v>
+        <v>9</v>
       </c>
       <c r="G31" t="n">
-        <v>6.7</v>
+        <v>7</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.9</v>
       </c>
       <c r="E32" t="n">
-        <v>4.9</v>
+        <v>5.2</v>
       </c>
       <c r="F32" t="n">
-        <v>3.8</v>
+        <v>4.2</v>
       </c>
       <c r="G32" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun Sep 20 13:43:04 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>88.2</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>91.7</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>89.90000000000001</v>
+        <v>89.7</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>0.99</v>
       </c>
       <c r="E3" t="n">
-        <v>69.8</v>
+        <v>69.7</v>
       </c>
       <c r="F3" t="n">
-        <v>60.8</v>
+        <v>60.7</v>
       </c>
       <c r="G3" t="n">
-        <v>65.3</v>
+        <v>65.2</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="4">
@@ -555,13 +555,13 @@
         <v>37.2</v>
       </c>
       <c r="F4" t="n">
-        <v>75</v>
+        <v>74.8</v>
       </c>
       <c r="G4" t="n">
-        <v>56.1</v>
+        <v>56</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="5">
@@ -585,13 +585,13 @@
         <v>51.7</v>
       </c>
       <c r="F5" t="n">
-        <v>55.6</v>
+        <v>55.5</v>
       </c>
       <c r="G5" t="n">
         <v>53.6</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="6">
@@ -621,7 +621,7 @@
         <v>51.6</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="7">
@@ -651,7 +651,7 @@
         <v>50.3</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="8">
@@ -681,7 +681,7 @@
         <v>49</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>2.67</v>
       </c>
       <c r="E9" t="n">
-        <v>29.5</v>
+        <v>29.7</v>
       </c>
       <c r="F9" t="n">
-        <v>58</v>
+        <v>57.9</v>
       </c>
       <c r="G9" t="n">
         <v>43.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>3.53</v>
       </c>
       <c r="E10" t="n">
-        <v>32.3</v>
+        <v>32.4</v>
       </c>
       <c r="F10" t="n">
         <v>52.8</v>
       </c>
       <c r="G10" t="n">
-        <v>42.5</v>
+        <v>42.6</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.22</v>
       </c>
       <c r="E11" t="n">
-        <v>24.3</v>
+        <v>24.5</v>
       </c>
       <c r="F11" t="n">
         <v>51</v>
       </c>
       <c r="G11" t="n">
-        <v>37.7</v>
+        <v>37.8</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>2.33</v>
       </c>
       <c r="E12" t="n">
-        <v>22.6</v>
+        <v>22.8</v>
       </c>
       <c r="F12" t="n">
         <v>52.4</v>
       </c>
       <c r="G12" t="n">
-        <v>37.5</v>
+        <v>37.6</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.97</v>
       </c>
       <c r="E13" t="n">
-        <v>85.8</v>
+        <v>85.5</v>
       </c>
       <c r="F13" t="n">
-        <v>14.6</v>
+        <v>14.8</v>
       </c>
       <c r="G13" t="n">
-        <v>35.9</v>
+        <v>36</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.78</v>
       </c>
       <c r="E14" t="n">
-        <v>8.699999999999999</v>
+        <v>9</v>
       </c>
       <c r="F14" t="n">
         <v>62.8</v>
       </c>
       <c r="G14" t="n">
-        <v>35.8</v>
+        <v>35.9</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>7.93</v>
       </c>
       <c r="E15" t="n">
-        <v>12.8</v>
+        <v>13.1</v>
       </c>
       <c r="F15" t="n">
         <v>55.9</v>
       </c>
       <c r="G15" t="n">
-        <v>34.4</v>
+        <v>34.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>1.84</v>
       </c>
       <c r="E16" t="n">
-        <v>28.8</v>
+        <v>29</v>
       </c>
       <c r="F16" t="n">
-        <v>38.5</v>
+        <v>38.6</v>
       </c>
       <c r="G16" t="n">
-        <v>33.7</v>
+        <v>33.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.71</v>
       </c>
       <c r="E17" t="n">
-        <v>67</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="F17" t="n">
-        <v>18.4</v>
+        <v>18.6</v>
       </c>
       <c r="G17" t="n">
-        <v>33</v>
+        <v>33.1</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>1.97</v>
       </c>
       <c r="E18" t="n">
-        <v>24.7</v>
+        <v>24.8</v>
       </c>
       <c r="F18" t="n">
-        <v>39.9</v>
+        <v>40</v>
       </c>
       <c r="G18" t="n">
-        <v>32.3</v>
+        <v>32.4</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>2.33</v>
       </c>
       <c r="E19" t="n">
-        <v>21.9</v>
+        <v>22.1</v>
       </c>
       <c r="F19" t="n">
-        <v>34.4</v>
+        <v>34.5</v>
       </c>
       <c r="G19" t="n">
-        <v>28.1</v>
+        <v>28.3</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>3.6</v>
       </c>
       <c r="E20" t="n">
-        <v>16.3</v>
+        <v>16.6</v>
       </c>
       <c r="F20" t="n">
-        <v>31.6</v>
+        <v>31.7</v>
       </c>
       <c r="G20" t="n">
-        <v>24</v>
+        <v>24.1</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>1.29</v>
       </c>
       <c r="E21" t="n">
-        <v>8.699999999999999</v>
+        <v>9</v>
       </c>
       <c r="F21" t="n">
-        <v>27.4</v>
+        <v>27.6</v>
       </c>
       <c r="G21" t="n">
-        <v>21.8</v>
+        <v>22</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>3.63</v>
       </c>
       <c r="E22" t="n">
-        <v>12.8</v>
+        <v>13.1</v>
       </c>
       <c r="F22" t="n">
-        <v>25.3</v>
+        <v>25.5</v>
       </c>
       <c r="G22" t="n">
-        <v>21.6</v>
+        <v>21.8</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>0.95</v>
       </c>
       <c r="E23" t="n">
-        <v>9.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F23" t="n">
-        <v>31.6</v>
+        <v>31.7</v>
       </c>
       <c r="G23" t="n">
-        <v>20.5</v>
+        <v>20.7</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="24">
@@ -1155,13 +1155,13 @@
         <v>44.1</v>
       </c>
       <c r="F24" t="n">
-        <v>9.699999999999999</v>
+        <v>10</v>
       </c>
       <c r="G24" t="n">
-        <v>20</v>
+        <v>20.2</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.34</v>
       </c>
       <c r="E25" t="n">
-        <v>8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F25" t="n">
-        <v>30.6</v>
+        <v>30.7</v>
       </c>
       <c r="G25" t="n">
-        <v>19.3</v>
+        <v>19.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>3.79</v>
       </c>
       <c r="E26" t="n">
-        <v>6.6</v>
+        <v>6.9</v>
       </c>
       <c r="F26" t="n">
-        <v>20.1</v>
+        <v>20.3</v>
       </c>
       <c r="G26" t="n">
-        <v>16.1</v>
+        <v>16.3</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.33</v>
       </c>
       <c r="E27" t="n">
-        <v>5.9</v>
+        <v>6.2</v>
       </c>
       <c r="F27" t="n">
-        <v>20.1</v>
+        <v>20.3</v>
       </c>
       <c r="G27" t="n">
-        <v>15.9</v>
+        <v>16.1</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>1.44</v>
       </c>
       <c r="E28" t="n">
-        <v>8.699999999999999</v>
+        <v>9</v>
       </c>
       <c r="F28" t="n">
-        <v>17</v>
+        <v>17.2</v>
       </c>
       <c r="G28" t="n">
-        <v>14.5</v>
+        <v>14.8</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.2</v>
       </c>
       <c r="E29" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="F29" t="n">
-        <v>18.8</v>
+        <v>19</v>
       </c>
       <c r="G29" t="n">
-        <v>14.1</v>
+        <v>14.3</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>2.02</v>
       </c>
       <c r="E30" t="n">
-        <v>20.5</v>
+        <v>20.7</v>
       </c>
       <c r="F30" t="n">
-        <v>9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G30" t="n">
-        <v>12.5</v>
+        <v>12.7</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.2</v>
       </c>
       <c r="E31" t="n">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
       <c r="F31" t="n">
-        <v>9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G31" t="n">
-        <v>7</v>
+        <v>7.3</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.9</v>
       </c>
       <c r="E32" t="n">
-        <v>5.2</v>
+        <v>5.5</v>
       </c>
       <c r="F32" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="G32" t="n">
-        <v>4.5</v>
+        <v>4.8</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon Sep 21 16:01:39 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,112 +486,112 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.26</v>
+        <v>7.32</v>
       </c>
       <c r="D2" t="n">
         <v>0.6899999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>87.90000000000001</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>91.40000000000001</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>89.7</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.13</v>
+        <v>28.72</v>
       </c>
       <c r="D3" t="n">
-        <v>0.99</v>
+        <v>2.76</v>
       </c>
       <c r="E3" t="n">
-        <v>69.7</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>60.7</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>65.2</v>
+        <v>76</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>33.79</v>
+        <v>20.34</v>
       </c>
       <c r="D4" t="n">
-        <v>2.11</v>
+        <v>0.99</v>
       </c>
       <c r="E4" t="n">
-        <v>37.2</v>
+        <v>81.8</v>
       </c>
       <c r="F4" t="n">
-        <v>74.8</v>
+        <v>60.6</v>
       </c>
       <c r="G4" t="n">
-        <v>56</v>
+        <v>71.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>38.76</v>
+        <v>34.58</v>
       </c>
       <c r="D5" t="n">
-        <v>3.41</v>
+        <v>2.16</v>
       </c>
       <c r="E5" t="n">
-        <v>51.7</v>
+        <v>43.2</v>
       </c>
       <c r="F5" t="n">
-        <v>55.5</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>53.6</v>
+        <v>61.6</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="6">
@@ -606,52 +606,52 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>19.71</v>
+        <v>19.98</v>
       </c>
       <c r="D6" t="n">
-        <v>1.65</v>
+        <v>1.67</v>
       </c>
       <c r="E6" t="n">
-        <v>54.5</v>
+        <v>64</v>
       </c>
       <c r="F6" t="n">
-        <v>48.6</v>
+        <v>57.2</v>
       </c>
       <c r="G6" t="n">
-        <v>51.6</v>
+        <v>60.6</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>30.29</v>
+        <v>14.65</v>
       </c>
       <c r="D7" t="n">
-        <v>2.9</v>
+        <v>1.24</v>
       </c>
       <c r="E7" t="n">
-        <v>49</v>
+        <v>43.2</v>
       </c>
       <c r="F7" t="n">
-        <v>51.7</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>50.3</v>
+        <v>58</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="8">
@@ -666,682 +666,682 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>22.1</v>
+        <v>22.4</v>
       </c>
       <c r="D8" t="n">
-        <v>2.06</v>
+        <v>2.08</v>
       </c>
       <c r="E8" t="n">
-        <v>44.8</v>
+        <v>52.1</v>
       </c>
       <c r="F8" t="n">
-        <v>53.1</v>
+        <v>57.9</v>
       </c>
       <c r="G8" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>27.75</v>
+        <v>30.42</v>
       </c>
       <c r="D9" t="n">
-        <v>2.67</v>
+        <v>2.92</v>
       </c>
       <c r="E9" t="n">
-        <v>29.7</v>
+        <v>50</v>
       </c>
       <c r="F9" t="n">
-        <v>57.9</v>
+        <v>55.1</v>
       </c>
       <c r="G9" t="n">
-        <v>43.8</v>
+        <v>52.6</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>19.67</v>
+        <v>16.81</v>
       </c>
       <c r="D10" t="n">
-        <v>3.53</v>
+        <v>1.81</v>
       </c>
       <c r="E10" t="n">
-        <v>32.4</v>
+        <v>15.8</v>
       </c>
       <c r="F10" t="n">
-        <v>52.8</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="G10" t="n">
-        <v>42.6</v>
+        <v>46.9</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>14.47</v>
+        <v>38.25</v>
       </c>
       <c r="D11" t="n">
-        <v>1.22</v>
+        <v>3.36</v>
       </c>
       <c r="E11" t="n">
-        <v>24.5</v>
+        <v>43.8</v>
       </c>
       <c r="F11" t="n">
-        <v>51</v>
+        <v>49.7</v>
       </c>
       <c r="G11" t="n">
-        <v>37.8</v>
+        <v>46.7</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>15.2</v>
+        <v>19.74</v>
       </c>
       <c r="D12" t="n">
-        <v>2.33</v>
+        <v>3.54</v>
       </c>
       <c r="E12" t="n">
-        <v>22.8</v>
+        <v>35.6</v>
       </c>
       <c r="F12" t="n">
-        <v>52.4</v>
+        <v>55.8</v>
       </c>
       <c r="G12" t="n">
-        <v>37.6</v>
+        <v>45.7</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>32.78</v>
+        <v>23.83</v>
       </c>
       <c r="D13" t="n">
-        <v>1.97</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>85.5</v>
+        <v>40.4</v>
       </c>
       <c r="F13" t="n">
-        <v>14.8</v>
+        <v>50</v>
       </c>
       <c r="G13" t="n">
-        <v>36</v>
+        <v>45.2</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>16.51</v>
+        <v>21.92</v>
       </c>
       <c r="D14" t="n">
-        <v>1.78</v>
+        <v>1.86</v>
       </c>
       <c r="E14" t="n">
-        <v>9</v>
+        <v>34.9</v>
       </c>
       <c r="F14" t="n">
-        <v>62.8</v>
+        <v>52.4</v>
       </c>
       <c r="G14" t="n">
-        <v>35.9</v>
+        <v>43.7</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>53.46</v>
+        <v>30.18</v>
       </c>
       <c r="D15" t="n">
-        <v>7.93</v>
+        <v>2.37</v>
       </c>
       <c r="E15" t="n">
-        <v>13.1</v>
+        <v>36.6</v>
       </c>
       <c r="F15" t="n">
-        <v>55.9</v>
+        <v>50</v>
       </c>
       <c r="G15" t="n">
-        <v>34.5</v>
+        <v>43.3</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>21.65</v>
+        <v>33.25</v>
       </c>
       <c r="D16" t="n">
-        <v>1.84</v>
+        <v>1.99</v>
       </c>
       <c r="E16" t="n">
-        <v>29</v>
+        <v>89</v>
       </c>
       <c r="F16" t="n">
-        <v>38.6</v>
+        <v>18.2</v>
       </c>
       <c r="G16" t="n">
-        <v>33.8</v>
+        <v>39.4</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>20.19</v>
+        <v>54.03</v>
       </c>
       <c r="D17" t="n">
-        <v>1.71</v>
+        <v>8.02</v>
       </c>
       <c r="E17" t="n">
-        <v>66.90000000000001</v>
+        <v>15.1</v>
       </c>
       <c r="F17" t="n">
-        <v>18.6</v>
+        <v>62.3</v>
       </c>
       <c r="G17" t="n">
-        <v>33.1</v>
+        <v>38.7</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>23.53</v>
+        <v>26.96</v>
       </c>
       <c r="D18" t="n">
-        <v>1.97</v>
+        <v>2.41</v>
       </c>
       <c r="E18" t="n">
-        <v>24.8</v>
+        <v>20.5</v>
       </c>
       <c r="F18" t="n">
-        <v>40</v>
+        <v>54.1</v>
       </c>
       <c r="G18" t="n">
-        <v>32.4</v>
+        <v>37.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>29.66</v>
+        <v>53.59</v>
       </c>
       <c r="D19" t="n">
-        <v>2.33</v>
+        <v>3.67</v>
       </c>
       <c r="E19" t="n">
-        <v>22.1</v>
+        <v>28.8</v>
       </c>
       <c r="F19" t="n">
-        <v>34.5</v>
+        <v>39</v>
       </c>
       <c r="G19" t="n">
-        <v>28.3</v>
+        <v>33.9</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>52.54</v>
+        <v>20.18</v>
       </c>
       <c r="D20" t="n">
-        <v>3.6</v>
+        <v>1.71</v>
       </c>
       <c r="E20" t="n">
-        <v>16.6</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="F20" t="n">
-        <v>31.7</v>
+        <v>18.8</v>
       </c>
       <c r="G20" t="n">
-        <v>24.1</v>
+        <v>32.7</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>12.28</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="D21" t="n">
-        <v>1.29</v>
+        <v>0.97</v>
       </c>
       <c r="E21" t="n">
-        <v>9</v>
+        <v>19.9</v>
       </c>
       <c r="F21" t="n">
-        <v>27.6</v>
+        <v>44.5</v>
       </c>
       <c r="G21" t="n">
-        <v>22</v>
+        <v>32.2</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>68.48999999999999</v>
+        <v>12.55</v>
       </c>
       <c r="D22" t="n">
-        <v>3.63</v>
+        <v>1.32</v>
       </c>
       <c r="E22" t="n">
-        <v>13.1</v>
+        <v>15.8</v>
       </c>
       <c r="F22" t="n">
-        <v>25.5</v>
+        <v>45.5</v>
       </c>
       <c r="G22" t="n">
-        <v>21.8</v>
+        <v>30.7</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>8.58</v>
+        <v>14.97</v>
       </c>
       <c r="D23" t="n">
-        <v>0.95</v>
+        <v>2.3</v>
       </c>
       <c r="E23" t="n">
-        <v>9.699999999999999</v>
+        <v>6.5</v>
       </c>
       <c r="F23" t="n">
-        <v>31.7</v>
+        <v>45.5</v>
       </c>
       <c r="G23" t="n">
-        <v>20.7</v>
+        <v>26</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>10.64</v>
+        <v>22.67</v>
       </c>
       <c r="D24" t="n">
-        <v>0.63</v>
+        <v>2.37</v>
       </c>
       <c r="E24" t="n">
-        <v>44.1</v>
+        <v>10.3</v>
       </c>
       <c r="F24" t="n">
-        <v>10</v>
+        <v>29.8</v>
       </c>
       <c r="G24" t="n">
-        <v>20.2</v>
+        <v>23.9</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>26.2</v>
+        <v>22.79</v>
       </c>
       <c r="D25" t="n">
-        <v>2.34</v>
+        <v>2.05</v>
       </c>
       <c r="E25" t="n">
-        <v>8.300000000000001</v>
+        <v>32.5</v>
       </c>
       <c r="F25" t="n">
-        <v>30.7</v>
+        <v>18.8</v>
       </c>
       <c r="G25" t="n">
-        <v>19.5</v>
+        <v>22.9</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>40.7</v>
+        <v>10.71</v>
       </c>
       <c r="D26" t="n">
-        <v>3.79</v>
+        <v>0.63</v>
       </c>
       <c r="E26" t="n">
-        <v>6.9</v>
+        <v>51.4</v>
       </c>
       <c r="F26" t="n">
-        <v>20.3</v>
+        <v>10.3</v>
       </c>
       <c r="G26" t="n">
-        <v>16.3</v>
+        <v>22.6</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>22.34</v>
+        <v>7.79</v>
       </c>
       <c r="D27" t="n">
-        <v>2.33</v>
+        <v>1.21</v>
       </c>
       <c r="E27" t="n">
-        <v>6.2</v>
+        <v>7.5</v>
       </c>
       <c r="F27" t="n">
-        <v>20.3</v>
+        <v>28.8</v>
       </c>
       <c r="G27" t="n">
-        <v>16.1</v>
+        <v>22.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>18.77</v>
+        <v>40.98</v>
       </c>
       <c r="D28" t="n">
-        <v>1.44</v>
+        <v>3.82</v>
       </c>
       <c r="E28" t="n">
-        <v>9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F28" t="n">
-        <v>17.2</v>
+        <v>27.1</v>
       </c>
       <c r="G28" t="n">
-        <v>14.8</v>
+        <v>21.4</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>7.71</v>
+        <v>18.95</v>
       </c>
       <c r="D29" t="n">
-        <v>1.2</v>
+        <v>1.45</v>
       </c>
       <c r="E29" t="n">
-        <v>3.4</v>
+        <v>16.1</v>
       </c>
       <c r="F29" t="n">
-        <v>19</v>
+        <v>23.6</v>
       </c>
       <c r="G29" t="n">
-        <v>14.3</v>
+        <v>21.4</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>22.54</v>
+        <v>68.14</v>
       </c>
       <c r="D30" t="n">
-        <v>2.02</v>
+        <v>3.61</v>
       </c>
       <c r="E30" t="n">
-        <v>20.7</v>
+        <v>9.6</v>
       </c>
       <c r="F30" t="n">
-        <v>9.300000000000001</v>
+        <v>20.9</v>
       </c>
       <c r="G30" t="n">
-        <v>12.7</v>
+        <v>17.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="31">
@@ -1356,22 +1356,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>17.11</v>
+        <v>17.08</v>
       </c>
       <c r="D31" t="n">
         <v>3.2</v>
       </c>
       <c r="E31" t="n">
-        <v>2.8</v>
+        <v>2.1</v>
       </c>
       <c r="F31" t="n">
-        <v>9.300000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="G31" t="n">
         <v>7.3</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25.79</v>
+        <v>25.69</v>
       </c>
       <c r="D32" t="n">
-        <v>2.9</v>
+        <v>2.89</v>
       </c>
       <c r="E32" t="n">
-        <v>5.5</v>
+        <v>2.7</v>
       </c>
       <c r="F32" t="n">
-        <v>4.5</v>
+        <v>2.7</v>
       </c>
       <c r="G32" t="n">
-        <v>4.8</v>
+        <v>2.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue Sep 22 14:12:24 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>92.09999999999999</v>
+        <v>91.8</v>
       </c>
       <c r="F2" t="n">
-        <v>91.09999999999999</v>
+        <v>90.8</v>
       </c>
       <c r="G2" t="n">
-        <v>91.59999999999999</v>
+        <v>91.3</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="3">
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28.72</v>
+        <v>28.76</v>
       </c>
       <c r="D3" t="n">
         <v>2.76</v>
       </c>
       <c r="E3" t="n">
-        <v>66.40000000000001</v>
+        <v>68</v>
       </c>
       <c r="F3" t="n">
-        <v>85.59999999999999</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>76</v>
+        <v>76.7</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="4">
@@ -546,22 +546,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>20.34</v>
+        <v>20.16</v>
       </c>
       <c r="D4" t="n">
         <v>0.99</v>
       </c>
       <c r="E4" t="n">
-        <v>81.8</v>
+        <v>74.5</v>
       </c>
       <c r="F4" t="n">
-        <v>60.6</v>
+        <v>60.5</v>
       </c>
       <c r="G4" t="n">
-        <v>71.2</v>
+        <v>67.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="5">
@@ -576,772 +576,772 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>34.58</v>
+        <v>34.41</v>
       </c>
       <c r="D5" t="n">
-        <v>2.16</v>
+        <v>2.14</v>
       </c>
       <c r="E5" t="n">
-        <v>43.2</v>
+        <v>41.5</v>
       </c>
       <c r="F5" t="n">
-        <v>80.09999999999999</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>61.6</v>
+        <v>59.2</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>19.98</v>
+        <v>22.49</v>
       </c>
       <c r="D6" t="n">
-        <v>1.67</v>
+        <v>2.09</v>
       </c>
       <c r="E6" t="n">
-        <v>64</v>
+        <v>57.5</v>
       </c>
       <c r="F6" t="n">
-        <v>57.2</v>
+        <v>60.5</v>
       </c>
       <c r="G6" t="n">
-        <v>60.6</v>
+        <v>59</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>14.65</v>
+        <v>24.34</v>
       </c>
       <c r="D7" t="n">
-        <v>1.24</v>
+        <v>2.04</v>
       </c>
       <c r="E7" t="n">
-        <v>43.2</v>
+        <v>53.1</v>
       </c>
       <c r="F7" t="n">
-        <v>72.90000000000001</v>
+        <v>63.3</v>
       </c>
       <c r="G7" t="n">
-        <v>58</v>
+        <v>58.2</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>22.4</v>
+        <v>19.91</v>
       </c>
       <c r="D8" t="n">
-        <v>2.08</v>
+        <v>1.66</v>
       </c>
       <c r="E8" t="n">
-        <v>52.1</v>
+        <v>61.2</v>
       </c>
       <c r="F8" t="n">
-        <v>57.9</v>
+        <v>53.1</v>
       </c>
       <c r="G8" t="n">
-        <v>55</v>
+        <v>57.1</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>30.42</v>
+        <v>16.99</v>
       </c>
       <c r="D9" t="n">
-        <v>2.92</v>
+        <v>1.84</v>
       </c>
       <c r="E9" t="n">
-        <v>50</v>
+        <v>19.7</v>
       </c>
       <c r="F9" t="n">
-        <v>55.1</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>52.6</v>
+        <v>53.1</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>16.81</v>
+        <v>30.29</v>
       </c>
       <c r="D10" t="n">
-        <v>1.81</v>
+        <v>2.91</v>
       </c>
       <c r="E10" t="n">
-        <v>15.8</v>
+        <v>48.6</v>
       </c>
       <c r="F10" t="n">
-        <v>78.09999999999999</v>
+        <v>53.4</v>
       </c>
       <c r="G10" t="n">
-        <v>46.9</v>
+        <v>51</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>38.25</v>
+        <v>19.8</v>
       </c>
       <c r="D11" t="n">
-        <v>3.36</v>
+        <v>3.55</v>
       </c>
       <c r="E11" t="n">
-        <v>43.8</v>
+        <v>41.2</v>
       </c>
       <c r="F11" t="n">
-        <v>49.7</v>
+        <v>59.5</v>
       </c>
       <c r="G11" t="n">
-        <v>46.7</v>
+        <v>50.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>19.74</v>
+        <v>38.01</v>
       </c>
       <c r="D12" t="n">
-        <v>3.54</v>
+        <v>3.34</v>
       </c>
       <c r="E12" t="n">
-        <v>35.6</v>
+        <v>40.8</v>
       </c>
       <c r="F12" t="n">
-        <v>55.8</v>
+        <v>47.3</v>
       </c>
       <c r="G12" t="n">
-        <v>45.7</v>
+        <v>44</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>23.83</v>
+        <v>21.89</v>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>1.86</v>
       </c>
       <c r="E13" t="n">
-        <v>40.4</v>
+        <v>34.7</v>
       </c>
       <c r="F13" t="n">
-        <v>50</v>
+        <v>52.4</v>
       </c>
       <c r="G13" t="n">
-        <v>45.2</v>
+        <v>43.5</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>21.92</v>
+        <v>30.1</v>
       </c>
       <c r="D14" t="n">
-        <v>1.86</v>
+        <v>2.36</v>
       </c>
       <c r="E14" t="n">
-        <v>34.9</v>
+        <v>34.7</v>
       </c>
       <c r="F14" t="n">
-        <v>52.4</v>
+        <v>47.6</v>
       </c>
       <c r="G14" t="n">
-        <v>43.7</v>
+        <v>41.2</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>30.18</v>
+        <v>26.99</v>
       </c>
       <c r="D15" t="n">
-        <v>2.37</v>
+        <v>2.42</v>
       </c>
       <c r="E15" t="n">
-        <v>36.6</v>
+        <v>22.8</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>56.1</v>
       </c>
       <c r="G15" t="n">
-        <v>43.3</v>
+        <v>39.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>33.25</v>
+        <v>54.2</v>
       </c>
       <c r="D16" t="n">
-        <v>1.99</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="E16" t="n">
-        <v>89</v>
+        <v>15.6</v>
       </c>
       <c r="F16" t="n">
-        <v>18.2</v>
+        <v>63.3</v>
       </c>
       <c r="G16" t="n">
-        <v>39.4</v>
+        <v>39.5</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>54.03</v>
+        <v>32.98</v>
       </c>
       <c r="D17" t="n">
-        <v>8.02</v>
+        <v>1.98</v>
       </c>
       <c r="E17" t="n">
-        <v>15.1</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="F17" t="n">
-        <v>62.3</v>
+        <v>16.7</v>
       </c>
       <c r="G17" t="n">
-        <v>38.7</v>
+        <v>37.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>26.96</v>
+        <v>15.15</v>
       </c>
       <c r="D18" t="n">
-        <v>2.41</v>
+        <v>2.32</v>
       </c>
       <c r="E18" t="n">
-        <v>20.5</v>
+        <v>19.4</v>
       </c>
       <c r="F18" t="n">
-        <v>54.1</v>
+        <v>51</v>
       </c>
       <c r="G18" t="n">
-        <v>37.3</v>
+        <v>35.2</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>53.59</v>
+        <v>14.42</v>
       </c>
       <c r="D19" t="n">
-        <v>3.67</v>
+        <v>1.22</v>
       </c>
       <c r="E19" t="n">
-        <v>28.8</v>
+        <v>19.4</v>
       </c>
       <c r="F19" t="n">
-        <v>39</v>
+        <v>50.7</v>
       </c>
       <c r="G19" t="n">
-        <v>33.9</v>
+        <v>35</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>20.18</v>
+        <v>8.73</v>
       </c>
       <c r="D20" t="n">
-        <v>1.71</v>
+        <v>0.97</v>
       </c>
       <c r="E20" t="n">
-        <v>65.09999999999999</v>
+        <v>19</v>
       </c>
       <c r="F20" t="n">
-        <v>18.8</v>
+        <v>44.6</v>
       </c>
       <c r="G20" t="n">
-        <v>32.7</v>
+        <v>31.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>8.789999999999999</v>
+        <v>12.54</v>
       </c>
       <c r="D21" t="n">
-        <v>0.97</v>
+        <v>1.32</v>
       </c>
       <c r="E21" t="n">
-        <v>19.9</v>
+        <v>15.6</v>
       </c>
       <c r="F21" t="n">
-        <v>44.5</v>
+        <v>45.6</v>
       </c>
       <c r="G21" t="n">
-        <v>32.2</v>
+        <v>30.6</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>12.55</v>
+        <v>53.07</v>
       </c>
       <c r="D22" t="n">
-        <v>1.32</v>
+        <v>3.63</v>
       </c>
       <c r="E22" t="n">
-        <v>15.8</v>
+        <v>23.8</v>
       </c>
       <c r="F22" t="n">
-        <v>45.5</v>
+        <v>35</v>
       </c>
       <c r="G22" t="n">
-        <v>30.7</v>
+        <v>29.4</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>14.97</v>
+        <v>20.08</v>
       </c>
       <c r="D23" t="n">
-        <v>2.3</v>
+        <v>1.7</v>
       </c>
       <c r="E23" t="n">
-        <v>6.5</v>
+        <v>61.9</v>
       </c>
       <c r="F23" t="n">
-        <v>45.5</v>
+        <v>11.9</v>
       </c>
       <c r="G23" t="n">
-        <v>26</v>
+        <v>26.9</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>22.67</v>
+        <v>69.05</v>
       </c>
       <c r="D24" t="n">
-        <v>2.37</v>
+        <v>3.66</v>
       </c>
       <c r="E24" t="n">
-        <v>10.3</v>
+        <v>18.4</v>
       </c>
       <c r="F24" t="n">
-        <v>29.8</v>
+        <v>31</v>
       </c>
       <c r="G24" t="n">
-        <v>23.9</v>
+        <v>24.7</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>22.79</v>
+        <v>41.51</v>
       </c>
       <c r="D25" t="n">
-        <v>2.05</v>
+        <v>3.87</v>
       </c>
       <c r="E25" t="n">
-        <v>32.5</v>
+        <v>10.2</v>
       </c>
       <c r="F25" t="n">
-        <v>18.8</v>
+        <v>38.8</v>
       </c>
       <c r="G25" t="n">
-        <v>22.9</v>
+        <v>24.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>10.71</v>
+        <v>22.71</v>
       </c>
       <c r="D26" t="n">
-        <v>0.63</v>
+        <v>2.37</v>
       </c>
       <c r="E26" t="n">
-        <v>51.4</v>
+        <v>10.9</v>
       </c>
       <c r="F26" t="n">
-        <v>10.3</v>
+        <v>29.9</v>
       </c>
       <c r="G26" t="n">
-        <v>22.6</v>
+        <v>24.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>7.79</v>
+        <v>22.8</v>
       </c>
       <c r="D27" t="n">
-        <v>1.21</v>
+        <v>2.05</v>
       </c>
       <c r="E27" t="n">
-        <v>7.5</v>
+        <v>33.7</v>
       </c>
       <c r="F27" t="n">
-        <v>28.8</v>
+        <v>19</v>
       </c>
       <c r="G27" t="n">
-        <v>22.4</v>
+        <v>23.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>40.98</v>
+        <v>7.84</v>
       </c>
       <c r="D28" t="n">
-        <v>3.82</v>
+        <v>1.22</v>
       </c>
       <c r="E28" t="n">
         <v>8.199999999999999</v>
       </c>
       <c r="F28" t="n">
-        <v>27.1</v>
+        <v>35.4</v>
       </c>
       <c r="G28" t="n">
-        <v>21.4</v>
+        <v>21.8</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>18.95</v>
+        <v>10.66</v>
       </c>
       <c r="D29" t="n">
-        <v>1.45</v>
+        <v>0.63</v>
       </c>
       <c r="E29" t="n">
-        <v>16.1</v>
+        <v>45.6</v>
       </c>
       <c r="F29" t="n">
-        <v>23.6</v>
+        <v>10.5</v>
       </c>
       <c r="G29" t="n">
-        <v>21.4</v>
+        <v>21.1</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>68.14</v>
+        <v>18.9</v>
       </c>
       <c r="D30" t="n">
-        <v>3.61</v>
+        <v>1.45</v>
       </c>
       <c r="E30" t="n">
-        <v>9.6</v>
+        <v>13.9</v>
       </c>
       <c r="F30" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="G30" t="n">
         <v>20.9</v>
       </c>
-      <c r="G30" t="n">
-        <v>17.5</v>
-      </c>
       <c r="H30" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="31">
@@ -1356,22 +1356,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>17.08</v>
+        <v>17.11</v>
       </c>
       <c r="D31" t="n">
         <v>3.2</v>
       </c>
       <c r="E31" t="n">
-        <v>2.1</v>
+        <v>3.7</v>
       </c>
       <c r="F31" t="n">
-        <v>9.6</v>
+        <v>9.9</v>
       </c>
       <c r="G31" t="n">
-        <v>7.3</v>
+        <v>8</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25.69</v>
+        <v>25.75</v>
       </c>
       <c r="D32" t="n">
-        <v>2.89</v>
+        <v>2.9</v>
       </c>
       <c r="E32" t="n">
-        <v>2.7</v>
+        <v>5.4</v>
       </c>
       <c r="F32" t="n">
-        <v>2.7</v>
+        <v>5.4</v>
       </c>
       <c r="G32" t="n">
-        <v>2.7</v>
+        <v>5.4</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Wed Sep 23 14:27:41 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.32</v>
+        <v>7.27</v>
       </c>
       <c r="D2" t="n">
         <v>0.6899999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>91.8</v>
+        <v>88.2</v>
       </c>
       <c r="F2" t="n">
-        <v>90.8</v>
+        <v>90.5</v>
       </c>
       <c r="G2" t="n">
-        <v>91.3</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="3">
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28.76</v>
+        <v>28.82</v>
       </c>
       <c r="D3" t="n">
-        <v>2.76</v>
+        <v>2.77</v>
       </c>
       <c r="E3" t="n">
-        <v>68</v>
+        <v>68.2</v>
       </c>
       <c r="F3" t="n">
-        <v>85.40000000000001</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>76.7</v>
+        <v>78.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="4">
@@ -546,22 +546,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>20.16</v>
+        <v>20.02</v>
       </c>
       <c r="D4" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="E4" t="n">
-        <v>74.5</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>60.5</v>
+        <v>53</v>
       </c>
       <c r="G4" t="n">
-        <v>67.5</v>
+        <v>60</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="5">
@@ -576,22 +576,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>34.41</v>
+        <v>34.14</v>
       </c>
       <c r="D5" t="n">
-        <v>2.14</v>
+        <v>2.13</v>
       </c>
       <c r="E5" t="n">
-        <v>41.5</v>
+        <v>40.5</v>
       </c>
       <c r="F5" t="n">
-        <v>76.90000000000001</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>59.2</v>
+        <v>58.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="6">
@@ -606,262 +606,262 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>22.49</v>
+        <v>22.45</v>
       </c>
       <c r="D6" t="n">
         <v>2.09</v>
       </c>
       <c r="E6" t="n">
-        <v>57.5</v>
+        <v>53.4</v>
       </c>
       <c r="F6" t="n">
         <v>60.5</v>
       </c>
       <c r="G6" t="n">
-        <v>59</v>
+        <v>56.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>24.34</v>
+        <v>19.76</v>
       </c>
       <c r="D7" t="n">
-        <v>2.04</v>
+        <v>1.65</v>
       </c>
       <c r="E7" t="n">
-        <v>53.1</v>
+        <v>55.1</v>
       </c>
       <c r="F7" t="n">
-        <v>63.3</v>
+        <v>48</v>
       </c>
       <c r="G7" t="n">
-        <v>58.2</v>
+        <v>51.5</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19.91</v>
+        <v>19.78</v>
       </c>
       <c r="D8" t="n">
-        <v>1.66</v>
+        <v>3.55</v>
       </c>
       <c r="E8" t="n">
-        <v>61.2</v>
+        <v>38.5</v>
       </c>
       <c r="F8" t="n">
-        <v>53.1</v>
+        <v>59.5</v>
       </c>
       <c r="G8" t="n">
-        <v>57.1</v>
+        <v>49</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>16.99</v>
+        <v>30.15</v>
       </c>
       <c r="D9" t="n">
-        <v>1.84</v>
+        <v>2.89</v>
       </c>
       <c r="E9" t="n">
-        <v>19.7</v>
+        <v>45.3</v>
       </c>
       <c r="F9" t="n">
-        <v>86.40000000000001</v>
+        <v>49.7</v>
       </c>
       <c r="G9" t="n">
-        <v>53.1</v>
+        <v>47.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>30.29</v>
+        <v>30.34</v>
       </c>
       <c r="D10" t="n">
-        <v>2.91</v>
+        <v>2.38</v>
       </c>
       <c r="E10" t="n">
-        <v>48.6</v>
+        <v>43.2</v>
       </c>
       <c r="F10" t="n">
-        <v>53.4</v>
+        <v>51.7</v>
       </c>
       <c r="G10" t="n">
-        <v>51</v>
+        <v>47.5</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>19.8</v>
+        <v>23.84</v>
       </c>
       <c r="D11" t="n">
-        <v>3.55</v>
+        <v>2</v>
       </c>
       <c r="E11" t="n">
-        <v>41.2</v>
+        <v>41.9</v>
       </c>
       <c r="F11" t="n">
-        <v>59.5</v>
+        <v>49.7</v>
       </c>
       <c r="G11" t="n">
-        <v>50.3</v>
+        <v>45.8</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>38.01</v>
+        <v>16.78</v>
       </c>
       <c r="D12" t="n">
-        <v>3.34</v>
+        <v>1.81</v>
       </c>
       <c r="E12" t="n">
-        <v>40.8</v>
+        <v>13.2</v>
       </c>
       <c r="F12" t="n">
-        <v>47.3</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>44</v>
+        <v>45.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>21.89</v>
+        <v>37.96</v>
       </c>
       <c r="D13" t="n">
-        <v>1.86</v>
+        <v>3.34</v>
       </c>
       <c r="E13" t="n">
-        <v>34.7</v>
+        <v>40.5</v>
       </c>
       <c r="F13" t="n">
-        <v>52.4</v>
+        <v>47.3</v>
       </c>
       <c r="G13" t="n">
-        <v>43.5</v>
+        <v>43.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>30.1</v>
+        <v>54.33</v>
       </c>
       <c r="D14" t="n">
-        <v>2.36</v>
+        <v>8.06</v>
       </c>
       <c r="E14" t="n">
-        <v>34.7</v>
+        <v>16.2</v>
       </c>
       <c r="F14" t="n">
-        <v>47.6</v>
+        <v>63.5</v>
       </c>
       <c r="G14" t="n">
-        <v>41.2</v>
+        <v>39.9</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="15">
@@ -876,442 +876,442 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>26.99</v>
+        <v>26.78</v>
       </c>
       <c r="D15" t="n">
-        <v>2.42</v>
+        <v>2.4</v>
       </c>
       <c r="E15" t="n">
-        <v>22.8</v>
+        <v>16.2</v>
       </c>
       <c r="F15" t="n">
-        <v>56.1</v>
+        <v>51.4</v>
       </c>
       <c r="G15" t="n">
-        <v>39.5</v>
+        <v>33.8</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>54.2</v>
+        <v>15.13</v>
       </c>
       <c r="D16" t="n">
-        <v>8.039999999999999</v>
+        <v>2.32</v>
       </c>
       <c r="E16" t="n">
-        <v>15.6</v>
+        <v>16.6</v>
       </c>
       <c r="F16" t="n">
-        <v>63.3</v>
+        <v>51</v>
       </c>
       <c r="G16" t="n">
-        <v>39.5</v>
+        <v>33.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>32.98</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="D17" t="n">
-        <v>1.98</v>
+        <v>0.97</v>
       </c>
       <c r="E17" t="n">
-        <v>86.40000000000001</v>
+        <v>17.9</v>
       </c>
       <c r="F17" t="n">
-        <v>16.7</v>
+        <v>44.6</v>
       </c>
       <c r="G17" t="n">
-        <v>37.6</v>
+        <v>31.2</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>15.15</v>
+        <v>32.58</v>
       </c>
       <c r="D18" t="n">
-        <v>2.32</v>
+        <v>1.95</v>
       </c>
       <c r="E18" t="n">
-        <v>19.4</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="F18" t="n">
-        <v>51</v>
+        <v>7.4</v>
       </c>
       <c r="G18" t="n">
-        <v>35.2</v>
+        <v>29.9</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>14.42</v>
+        <v>21.4</v>
       </c>
       <c r="D19" t="n">
-        <v>1.22</v>
+        <v>1.82</v>
       </c>
       <c r="E19" t="n">
-        <v>19.4</v>
+        <v>18.9</v>
       </c>
       <c r="F19" t="n">
-        <v>50.7</v>
+        <v>32.4</v>
       </c>
       <c r="G19" t="n">
-        <v>35</v>
+        <v>25.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>8.73</v>
+        <v>52.35</v>
       </c>
       <c r="D20" t="n">
-        <v>0.97</v>
+        <v>3.59</v>
       </c>
       <c r="E20" t="n">
-        <v>19</v>
+        <v>13.5</v>
       </c>
       <c r="F20" t="n">
-        <v>44.6</v>
+        <v>29.7</v>
       </c>
       <c r="G20" t="n">
-        <v>31.8</v>
+        <v>24.9</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>12.54</v>
+        <v>68.52</v>
       </c>
       <c r="D21" t="n">
-        <v>1.32</v>
+        <v>3.64</v>
       </c>
       <c r="E21" t="n">
-        <v>15.6</v>
+        <v>15.5</v>
       </c>
       <c r="F21" t="n">
-        <v>45.6</v>
+        <v>28.7</v>
       </c>
       <c r="G21" t="n">
-        <v>30.6</v>
+        <v>24.8</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>53.07</v>
+        <v>14.31</v>
       </c>
       <c r="D22" t="n">
-        <v>3.63</v>
+        <v>1.21</v>
       </c>
       <c r="E22" t="n">
-        <v>23.8</v>
+        <v>11.5</v>
       </c>
       <c r="F22" t="n">
-        <v>35</v>
+        <v>37.2</v>
       </c>
       <c r="G22" t="n">
-        <v>29.4</v>
+        <v>24.3</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>20.08</v>
+        <v>12.41</v>
       </c>
       <c r="D23" t="n">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
       <c r="E23" t="n">
-        <v>61.9</v>
+        <v>13.9</v>
       </c>
       <c r="F23" t="n">
-        <v>11.9</v>
+        <v>33.1</v>
       </c>
       <c r="G23" t="n">
-        <v>26.9</v>
+        <v>23.5</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>69.05</v>
+        <v>41.03</v>
       </c>
       <c r="D24" t="n">
-        <v>3.66</v>
+        <v>3.83</v>
       </c>
       <c r="E24" t="n">
-        <v>18.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F24" t="n">
-        <v>31</v>
+        <v>29.4</v>
       </c>
       <c r="G24" t="n">
-        <v>24.7</v>
+        <v>23.2</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>41.51</v>
+        <v>7.79</v>
       </c>
       <c r="D25" t="n">
-        <v>3.87</v>
+        <v>1.21</v>
       </c>
       <c r="E25" t="n">
-        <v>10.2</v>
+        <v>7.8</v>
       </c>
       <c r="F25" t="n">
-        <v>38.8</v>
+        <v>28.7</v>
       </c>
       <c r="G25" t="n">
-        <v>24.5</v>
+        <v>22.4</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>22.71</v>
+        <v>10.65</v>
       </c>
       <c r="D26" t="n">
-        <v>2.37</v>
+        <v>0.63</v>
       </c>
       <c r="E26" t="n">
-        <v>10.9</v>
+        <v>45.3</v>
       </c>
       <c r="F26" t="n">
-        <v>29.9</v>
+        <v>10.8</v>
       </c>
       <c r="G26" t="n">
-        <v>24.2</v>
+        <v>21.1</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="D27" t="n">
-        <v>2.05</v>
+        <v>2.37</v>
       </c>
       <c r="E27" t="n">
-        <v>33.7</v>
+        <v>10.8</v>
       </c>
       <c r="F27" t="n">
-        <v>19</v>
+        <v>30.1</v>
       </c>
       <c r="G27" t="n">
-        <v>23.4</v>
+        <v>20.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>7.84</v>
+        <v>19.9</v>
       </c>
       <c r="D28" t="n">
-        <v>1.22</v>
+        <v>1.69</v>
       </c>
       <c r="E28" t="n">
-        <v>8.199999999999999</v>
+        <v>56.1</v>
       </c>
       <c r="F28" t="n">
-        <v>35.4</v>
+        <v>4.7</v>
       </c>
       <c r="G28" t="n">
-        <v>21.8</v>
+        <v>20.1</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>10.66</v>
+        <v>22.66</v>
       </c>
       <c r="D29" t="n">
-        <v>0.63</v>
+        <v>2.03</v>
       </c>
       <c r="E29" t="n">
-        <v>45.6</v>
+        <v>24.3</v>
       </c>
       <c r="F29" t="n">
-        <v>10.5</v>
+        <v>12.8</v>
       </c>
       <c r="G29" t="n">
-        <v>21.1</v>
+        <v>16.3</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="30">
@@ -1326,22 +1326,22 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>18.9</v>
+        <v>18.83</v>
       </c>
       <c r="D30" t="n">
-        <v>1.45</v>
+        <v>1.44</v>
       </c>
       <c r="E30" t="n">
-        <v>13.9</v>
+        <v>10.8</v>
       </c>
       <c r="F30" t="n">
-        <v>23.8</v>
+        <v>17.2</v>
       </c>
       <c r="G30" t="n">
-        <v>20.9</v>
+        <v>15.3</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="31">
@@ -1356,22 +1356,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>17.11</v>
+        <v>16.96</v>
       </c>
       <c r="D31" t="n">
-        <v>3.2</v>
+        <v>3.17</v>
       </c>
       <c r="E31" t="n">
-        <v>3.7</v>
+        <v>1.4</v>
       </c>
       <c r="F31" t="n">
-        <v>9.9</v>
+        <v>6.1</v>
       </c>
       <c r="G31" t="n">
-        <v>8</v>
+        <v>4.7</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25.75</v>
+        <v>25.62</v>
       </c>
       <c r="D32" t="n">
-        <v>2.9</v>
+        <v>2.88</v>
       </c>
       <c r="E32" t="n">
-        <v>5.4</v>
+        <v>2.7</v>
       </c>
       <c r="F32" t="n">
-        <v>5.4</v>
+        <v>2.7</v>
       </c>
       <c r="G32" t="n">
-        <v>5.4</v>
+        <v>2.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu Sep 24 14:27:43 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,112 +486,112 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.27</v>
+        <v>7.31</v>
       </c>
       <c r="D2" t="n">
         <v>0.6899999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>88.2</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>90.5</v>
+        <v>90.3</v>
       </c>
       <c r="G2" t="n">
-        <v>89.40000000000001</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28.82</v>
+        <v>19.89</v>
       </c>
       <c r="D3" t="n">
-        <v>2.77</v>
+        <v>0.97</v>
       </c>
       <c r="E3" t="n">
-        <v>68.2</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>88.90000000000001</v>
+        <v>47.7</v>
       </c>
       <c r="G3" t="n">
-        <v>78.5</v>
+        <v>56.4</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>20.02</v>
+        <v>19.86</v>
       </c>
       <c r="D4" t="n">
-        <v>0.98</v>
+        <v>1.66</v>
       </c>
       <c r="E4" t="n">
-        <v>66.90000000000001</v>
+        <v>57</v>
       </c>
       <c r="F4" t="n">
-        <v>53</v>
+        <v>53.4</v>
       </c>
       <c r="G4" t="n">
-        <v>60</v>
+        <v>55.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>34.14</v>
+        <v>28.05</v>
       </c>
       <c r="D5" t="n">
-        <v>2.13</v>
+        <v>2.7</v>
       </c>
       <c r="E5" t="n">
-        <v>40.5</v>
+        <v>38.9</v>
       </c>
       <c r="F5" t="n">
-        <v>76.40000000000001</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>58.4</v>
+        <v>52.5</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="6">
@@ -606,82 +606,82 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>22.45</v>
+        <v>22.25</v>
       </c>
       <c r="D6" t="n">
-        <v>2.09</v>
+        <v>2.07</v>
       </c>
       <c r="E6" t="n">
-        <v>53.4</v>
+        <v>47.7</v>
       </c>
       <c r="F6" t="n">
-        <v>60.5</v>
+        <v>54.7</v>
       </c>
       <c r="G6" t="n">
-        <v>56.9</v>
+        <v>51.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>19.76</v>
+        <v>16.93</v>
       </c>
       <c r="D7" t="n">
-        <v>1.65</v>
+        <v>1.83</v>
       </c>
       <c r="E7" t="n">
-        <v>55.1</v>
+        <v>19.5</v>
       </c>
       <c r="F7" t="n">
-        <v>48</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>51.5</v>
+        <v>50.7</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19.78</v>
+        <v>33.07</v>
       </c>
       <c r="D8" t="n">
-        <v>3.55</v>
+        <v>2.07</v>
       </c>
       <c r="E8" t="n">
-        <v>38.5</v>
+        <v>24.8</v>
       </c>
       <c r="F8" t="n">
-        <v>59.5</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>49</v>
+        <v>45.5</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="9">
@@ -696,22 +696,22 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>30.15</v>
+        <v>29.7</v>
       </c>
       <c r="D9" t="n">
-        <v>2.89</v>
+        <v>2.85</v>
       </c>
       <c r="E9" t="n">
-        <v>45.3</v>
+        <v>38.6</v>
       </c>
       <c r="F9" t="n">
-        <v>49.7</v>
+        <v>44</v>
       </c>
       <c r="G9" t="n">
-        <v>47.5</v>
+        <v>41.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="10">
@@ -726,22 +726,22 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>30.34</v>
+        <v>30.08</v>
       </c>
       <c r="D10" t="n">
-        <v>2.38</v>
+        <v>2.36</v>
       </c>
       <c r="E10" t="n">
-        <v>43.2</v>
+        <v>34.2</v>
       </c>
       <c r="F10" t="n">
-        <v>51.7</v>
+        <v>47.3</v>
       </c>
       <c r="G10" t="n">
-        <v>47.5</v>
+        <v>40.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="11">
@@ -756,112 +756,112 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>23.84</v>
+        <v>23.63</v>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>1.98</v>
       </c>
       <c r="E11" t="n">
-        <v>41.9</v>
+        <v>31.5</v>
       </c>
       <c r="F11" t="n">
-        <v>49.7</v>
+        <v>42.6</v>
       </c>
       <c r="G11" t="n">
-        <v>45.8</v>
+        <v>37.1</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>16.78</v>
+        <v>37.32</v>
       </c>
       <c r="D12" t="n">
-        <v>1.81</v>
+        <v>3.28</v>
       </c>
       <c r="E12" t="n">
-        <v>13.2</v>
+        <v>31.2</v>
       </c>
       <c r="F12" t="n">
-        <v>77.40000000000001</v>
+        <v>38.9</v>
       </c>
       <c r="G12" t="n">
-        <v>45.3</v>
+        <v>35.1</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>37.96</v>
+        <v>19.51</v>
       </c>
       <c r="D13" t="n">
-        <v>3.34</v>
+        <v>3.5</v>
       </c>
       <c r="E13" t="n">
-        <v>40.5</v>
+        <v>28.2</v>
       </c>
       <c r="F13" t="n">
-        <v>47.3</v>
+        <v>40.3</v>
       </c>
       <c r="G13" t="n">
-        <v>43.9</v>
+        <v>34.2</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>54.33</v>
+        <v>15.11</v>
       </c>
       <c r="D14" t="n">
-        <v>8.06</v>
+        <v>2.32</v>
       </c>
       <c r="E14" t="n">
-        <v>16.2</v>
+        <v>15.1</v>
       </c>
       <c r="F14" t="n">
-        <v>63.5</v>
+        <v>51</v>
       </c>
       <c r="G14" t="n">
-        <v>39.9</v>
+        <v>33.1</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="15">
@@ -876,82 +876,82 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>26.78</v>
+        <v>26.73</v>
       </c>
       <c r="D15" t="n">
-        <v>2.4</v>
+        <v>2.39</v>
       </c>
       <c r="E15" t="n">
-        <v>16.2</v>
+        <v>14.8</v>
       </c>
       <c r="F15" t="n">
-        <v>51.4</v>
+        <v>48</v>
       </c>
       <c r="G15" t="n">
-        <v>33.8</v>
+        <v>31.4</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>15.13</v>
+        <v>52.64</v>
       </c>
       <c r="D16" t="n">
-        <v>2.32</v>
+        <v>7.81</v>
       </c>
       <c r="E16" t="n">
-        <v>16.6</v>
+        <v>11.7</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G16" t="n">
-        <v>33.8</v>
+        <v>30.9</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>8.699999999999999</v>
+        <v>12.55</v>
       </c>
       <c r="D17" t="n">
-        <v>0.97</v>
+        <v>1.31</v>
       </c>
       <c r="E17" t="n">
-        <v>17.9</v>
+        <v>17.1</v>
       </c>
       <c r="F17" t="n">
-        <v>44.6</v>
+        <v>40.9</v>
       </c>
       <c r="G17" t="n">
-        <v>31.2</v>
+        <v>29</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="18">
@@ -966,232 +966,232 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>32.58</v>
+        <v>31.96</v>
       </c>
       <c r="D18" t="n">
-        <v>1.95</v>
+        <v>1.92</v>
       </c>
       <c r="E18" t="n">
-        <v>82.40000000000001</v>
+        <v>71.8</v>
       </c>
       <c r="F18" t="n">
-        <v>7.4</v>
+        <v>4.7</v>
       </c>
       <c r="G18" t="n">
-        <v>29.9</v>
+        <v>24.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>21.4</v>
+        <v>14.3</v>
       </c>
       <c r="D19" t="n">
-        <v>1.82</v>
+        <v>1.21</v>
       </c>
       <c r="E19" t="n">
-        <v>18.9</v>
+        <v>11.4</v>
       </c>
       <c r="F19" t="n">
-        <v>32.4</v>
+        <v>37.2</v>
       </c>
       <c r="G19" t="n">
-        <v>25.7</v>
+        <v>24.3</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>52.35</v>
+        <v>19.91</v>
       </c>
       <c r="D20" t="n">
-        <v>3.59</v>
+        <v>1.69</v>
       </c>
       <c r="E20" t="n">
-        <v>13.5</v>
+        <v>56.4</v>
       </c>
       <c r="F20" t="n">
-        <v>29.7</v>
+        <v>5</v>
       </c>
       <c r="G20" t="n">
-        <v>24.9</v>
+        <v>20.4</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>68.52</v>
+        <v>8.49</v>
       </c>
       <c r="D21" t="n">
-        <v>3.64</v>
+        <v>0.95</v>
       </c>
       <c r="E21" t="n">
-        <v>15.5</v>
+        <v>7.4</v>
       </c>
       <c r="F21" t="n">
-        <v>28.7</v>
+        <v>31.2</v>
       </c>
       <c r="G21" t="n">
-        <v>24.8</v>
+        <v>19.3</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>14.31</v>
+        <v>21.06</v>
       </c>
       <c r="D22" t="n">
-        <v>1.21</v>
+        <v>1.79</v>
       </c>
       <c r="E22" t="n">
-        <v>11.5</v>
+        <v>10.7</v>
       </c>
       <c r="F22" t="n">
-        <v>37.2</v>
+        <v>21.8</v>
       </c>
       <c r="G22" t="n">
-        <v>24.3</v>
+        <v>18.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>12.41</v>
+        <v>51.56</v>
       </c>
       <c r="D23" t="n">
-        <v>1.3</v>
+        <v>3.53</v>
       </c>
       <c r="E23" t="n">
-        <v>13.9</v>
+        <v>5.4</v>
       </c>
       <c r="F23" t="n">
-        <v>33.1</v>
+        <v>18.5</v>
       </c>
       <c r="G23" t="n">
-        <v>23.5</v>
+        <v>14.5</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>41.03</v>
+        <v>22.21</v>
       </c>
       <c r="D24" t="n">
-        <v>3.83</v>
+        <v>2.32</v>
       </c>
       <c r="E24" t="n">
-        <v>8.800000000000001</v>
+        <v>4.7</v>
       </c>
       <c r="F24" t="n">
-        <v>29.4</v>
+        <v>18.1</v>
       </c>
       <c r="G24" t="n">
-        <v>23.2</v>
+        <v>14.1</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>7.79</v>
+        <v>67.78</v>
       </c>
       <c r="D25" t="n">
-        <v>1.21</v>
+        <v>3.59</v>
       </c>
       <c r="E25" t="n">
-        <v>7.8</v>
+        <v>5.4</v>
       </c>
       <c r="F25" t="n">
-        <v>28.7</v>
+        <v>16.8</v>
       </c>
       <c r="G25" t="n">
-        <v>22.4</v>
+        <v>13.4</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="26">
@@ -1206,142 +1206,142 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>10.65</v>
+        <v>10.51</v>
       </c>
       <c r="D26" t="n">
-        <v>0.63</v>
+        <v>0.62</v>
       </c>
       <c r="E26" t="n">
-        <v>45.3</v>
+        <v>36.2</v>
       </c>
       <c r="F26" t="n">
-        <v>10.8</v>
+        <v>1.7</v>
       </c>
       <c r="G26" t="n">
-        <v>21.1</v>
+        <v>12</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>22.7</v>
+        <v>40.38</v>
       </c>
       <c r="D27" t="n">
-        <v>2.37</v>
+        <v>3.76</v>
       </c>
       <c r="E27" t="n">
-        <v>10.8</v>
+        <v>5.4</v>
       </c>
       <c r="F27" t="n">
-        <v>30.1</v>
+        <v>13.8</v>
       </c>
       <c r="G27" t="n">
-        <v>20.4</v>
+        <v>11.2</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>19.9</v>
+        <v>22.4</v>
       </c>
       <c r="D28" t="n">
-        <v>1.69</v>
+        <v>2.01</v>
       </c>
       <c r="E28" t="n">
-        <v>56.1</v>
+        <v>15.4</v>
       </c>
       <c r="F28" t="n">
-        <v>4.7</v>
+        <v>6</v>
       </c>
       <c r="G28" t="n">
-        <v>20.1</v>
+        <v>8.9</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>22.66</v>
+        <v>18.62</v>
       </c>
       <c r="D29" t="n">
-        <v>2.03</v>
+        <v>1.42</v>
       </c>
       <c r="E29" t="n">
-        <v>24.3</v>
+        <v>6</v>
       </c>
       <c r="F29" t="n">
-        <v>12.8</v>
+        <v>8.1</v>
       </c>
       <c r="G29" t="n">
-        <v>16.3</v>
+        <v>7.4</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>18.83</v>
+        <v>7.64</v>
       </c>
       <c r="D30" t="n">
-        <v>1.44</v>
+        <v>1.18</v>
       </c>
       <c r="E30" t="n">
-        <v>10.8</v>
+        <v>1.3</v>
       </c>
       <c r="F30" t="n">
-        <v>17.2</v>
+        <v>6.7</v>
       </c>
       <c r="G30" t="n">
-        <v>15.3</v>
+        <v>5.1</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="31">
@@ -1356,22 +1356,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>16.96</v>
+        <v>16.37</v>
       </c>
       <c r="D31" t="n">
-        <v>3.17</v>
+        <v>3.06</v>
       </c>
       <c r="E31" t="n">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="F31" t="n">
-        <v>6.1</v>
+        <v>2.3</v>
       </c>
       <c r="G31" t="n">
-        <v>4.7</v>
+        <v>1.8</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25.62</v>
+        <v>25.13</v>
       </c>
       <c r="D32" t="n">
-        <v>2.88</v>
+        <v>2.83</v>
       </c>
       <c r="E32" t="n">
-        <v>2.7</v>
+        <v>0.7</v>
       </c>
       <c r="F32" t="n">
-        <v>2.7</v>
+        <v>0.7</v>
       </c>
       <c r="G32" t="n">
-        <v>2.7</v>
+        <v>0.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri Sep 25 14:45:11 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>89.90000000000001</v>
+        <v>89.7</v>
       </c>
       <c r="F2" t="n">
-        <v>90.3</v>
+        <v>90</v>
       </c>
       <c r="G2" t="n">
-        <v>90.09999999999999</v>
+        <v>89.8</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>0.97</v>
       </c>
       <c r="E3" t="n">
-        <v>65.09999999999999</v>
+        <v>65</v>
       </c>
       <c r="F3" t="n">
         <v>47.7</v>
       </c>
       <c r="G3" t="n">
-        <v>56.4</v>
+        <v>56.3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="4">
@@ -555,13 +555,13 @@
         <v>57</v>
       </c>
       <c r="F4" t="n">
-        <v>53.4</v>
+        <v>53.3</v>
       </c>
       <c r="G4" t="n">
         <v>55.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.7</v>
       </c>
       <c r="E5" t="n">
-        <v>38.9</v>
+        <v>39</v>
       </c>
       <c r="F5" t="n">
-        <v>66.09999999999999</v>
+        <v>66</v>
       </c>
       <c r="G5" t="n">
         <v>52.5</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="6">
@@ -621,7 +621,7 @@
         <v>51.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.83</v>
       </c>
       <c r="E7" t="n">
-        <v>19.5</v>
+        <v>19.7</v>
       </c>
       <c r="F7" t="n">
-        <v>81.90000000000001</v>
+        <v>81.7</v>
       </c>
       <c r="G7" t="n">
         <v>50.7</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>2.07</v>
       </c>
       <c r="E8" t="n">
-        <v>24.8</v>
+        <v>25</v>
       </c>
       <c r="F8" t="n">
-        <v>66.09999999999999</v>
+        <v>66</v>
       </c>
       <c r="G8" t="n">
         <v>45.5</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="9">
@@ -702,7 +702,7 @@
         <v>2.85</v>
       </c>
       <c r="E9" t="n">
-        <v>38.6</v>
+        <v>38.7</v>
       </c>
       <c r="F9" t="n">
         <v>44</v>
@@ -711,7 +711,7 @@
         <v>41.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="10">
@@ -732,7 +732,7 @@
         <v>2.36</v>
       </c>
       <c r="E10" t="n">
-        <v>34.2</v>
+        <v>34.3</v>
       </c>
       <c r="F10" t="n">
         <v>47.3</v>
@@ -741,7 +741,7 @@
         <v>40.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.98</v>
       </c>
       <c r="E11" t="n">
-        <v>31.5</v>
+        <v>31.7</v>
       </c>
       <c r="F11" t="n">
-        <v>42.6</v>
+        <v>42.7</v>
       </c>
       <c r="G11" t="n">
-        <v>37.1</v>
+        <v>37.2</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>3.28</v>
       </c>
       <c r="E12" t="n">
-        <v>31.2</v>
+        <v>31.3</v>
       </c>
       <c r="F12" t="n">
-        <v>38.9</v>
+        <v>39</v>
       </c>
       <c r="G12" t="n">
-        <v>35.1</v>
+        <v>35.2</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>3.5</v>
       </c>
       <c r="E13" t="n">
-        <v>28.2</v>
+        <v>28.3</v>
       </c>
       <c r="F13" t="n">
         <v>40.3</v>
       </c>
       <c r="G13" t="n">
-        <v>34.2</v>
+        <v>34.3</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2.32</v>
       </c>
       <c r="E14" t="n">
-        <v>15.1</v>
+        <v>15.3</v>
       </c>
       <c r="F14" t="n">
         <v>51</v>
       </c>
       <c r="G14" t="n">
-        <v>33.1</v>
+        <v>33.2</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>2.39</v>
       </c>
       <c r="E15" t="n">
-        <v>14.8</v>
+        <v>15</v>
       </c>
       <c r="F15" t="n">
         <v>48</v>
       </c>
       <c r="G15" t="n">
-        <v>31.4</v>
+        <v>31.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>7.81</v>
       </c>
       <c r="E16" t="n">
-        <v>11.7</v>
+        <v>12</v>
       </c>
       <c r="F16" t="n">
         <v>50</v>
       </c>
       <c r="G16" t="n">
-        <v>30.9</v>
+        <v>31</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.31</v>
       </c>
       <c r="E17" t="n">
-        <v>17.1</v>
+        <v>17.3</v>
       </c>
       <c r="F17" t="n">
-        <v>40.9</v>
+        <v>41</v>
       </c>
       <c r="G17" t="n">
-        <v>29</v>
+        <v>29.2</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>1.92</v>
       </c>
       <c r="E18" t="n">
-        <v>71.8</v>
+        <v>71.7</v>
       </c>
       <c r="F18" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="G18" t="n">
-        <v>24.8</v>
+        <v>25</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.21</v>
       </c>
       <c r="E19" t="n">
-        <v>11.4</v>
+        <v>11.7</v>
       </c>
       <c r="F19" t="n">
-        <v>37.2</v>
+        <v>37.3</v>
       </c>
       <c r="G19" t="n">
-        <v>24.3</v>
+        <v>24.5</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>1.69</v>
       </c>
       <c r="E20" t="n">
-        <v>56.4</v>
+        <v>56.3</v>
       </c>
       <c r="F20" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="G20" t="n">
-        <v>20.4</v>
+        <v>20.6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>0.95</v>
       </c>
       <c r="E21" t="n">
-        <v>7.4</v>
+        <v>7.7</v>
       </c>
       <c r="F21" t="n">
-        <v>31.2</v>
+        <v>31.3</v>
       </c>
       <c r="G21" t="n">
-        <v>19.3</v>
+        <v>19.5</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.79</v>
       </c>
       <c r="E22" t="n">
-        <v>10.7</v>
+        <v>11</v>
       </c>
       <c r="F22" t="n">
-        <v>21.8</v>
+        <v>22</v>
       </c>
       <c r="G22" t="n">
-        <v>18.5</v>
+        <v>18.7</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>3.53</v>
       </c>
       <c r="E23" t="n">
-        <v>5.4</v>
+        <v>5.7</v>
       </c>
       <c r="F23" t="n">
-        <v>18.5</v>
+        <v>18.7</v>
       </c>
       <c r="G23" t="n">
-        <v>14.5</v>
+        <v>14.8</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.32</v>
       </c>
       <c r="E24" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="F24" t="n">
-        <v>18.1</v>
+        <v>18.3</v>
       </c>
       <c r="G24" t="n">
-        <v>14.1</v>
+        <v>14.3</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>3.59</v>
       </c>
       <c r="E25" t="n">
-        <v>5.4</v>
+        <v>5.7</v>
       </c>
       <c r="F25" t="n">
-        <v>16.8</v>
+        <v>17</v>
       </c>
       <c r="G25" t="n">
-        <v>13.4</v>
+        <v>13.6</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>0.62</v>
       </c>
       <c r="E26" t="n">
-        <v>36.2</v>
+        <v>36.3</v>
       </c>
       <c r="F26" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="G26" t="n">
-        <v>12</v>
+        <v>12.3</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>3.76</v>
       </c>
       <c r="E27" t="n">
-        <v>5.4</v>
+        <v>5.7</v>
       </c>
       <c r="F27" t="n">
-        <v>13.8</v>
+        <v>14</v>
       </c>
       <c r="G27" t="n">
-        <v>11.2</v>
+        <v>11.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.01</v>
       </c>
       <c r="E28" t="n">
-        <v>15.4</v>
+        <v>15.7</v>
       </c>
       <c r="F28" t="n">
-        <v>6</v>
+        <v>6.3</v>
       </c>
       <c r="G28" t="n">
-        <v>8.9</v>
+        <v>9.1</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.42</v>
       </c>
       <c r="E29" t="n">
-        <v>6</v>
+        <v>6.3</v>
       </c>
       <c r="F29" t="n">
-        <v>8.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G29" t="n">
-        <v>7.4</v>
+        <v>7.7</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.18</v>
       </c>
       <c r="E30" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="F30" t="n">
-        <v>6.7</v>
+        <v>7</v>
       </c>
       <c r="G30" t="n">
-        <v>5.1</v>
+        <v>5.4</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.06</v>
       </c>
       <c r="E31" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>2.3</v>
+        <v>2.7</v>
       </c>
       <c r="G31" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.83</v>
       </c>
       <c r="E32" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat Sep 26 13:54:10 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E2" t="n">
+        <v>89.40000000000001</v>
+      </c>
+      <c r="F2" t="n">
         <v>89.7</v>
       </c>
-      <c r="F2" t="n">
-        <v>90</v>
-      </c>
       <c r="G2" t="n">
-        <v>89.8</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="3">
@@ -522,7 +522,7 @@
         <v>0.97</v>
       </c>
       <c r="E3" t="n">
-        <v>65</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="F3" t="n">
         <v>47.7</v>
@@ -531,7 +531,7 @@
         <v>56.3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="4">
@@ -558,10 +558,10 @@
         <v>53.3</v>
       </c>
       <c r="G4" t="n">
-        <v>55.2</v>
+        <v>55.1</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>2.7</v>
       </c>
       <c r="E5" t="n">
-        <v>39</v>
+        <v>39.1</v>
       </c>
       <c r="F5" t="n">
-        <v>66</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="G5" t="n">
         <v>52.5</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="6">
@@ -615,13 +615,13 @@
         <v>47.7</v>
       </c>
       <c r="F6" t="n">
-        <v>54.7</v>
+        <v>54.6</v>
       </c>
       <c r="G6" t="n">
         <v>51.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.83</v>
       </c>
       <c r="E7" t="n">
-        <v>19.7</v>
+        <v>19.9</v>
       </c>
       <c r="F7" t="n">
-        <v>81.7</v>
+        <v>81.5</v>
       </c>
       <c r="G7" t="n">
         <v>50.7</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>2.07</v>
       </c>
       <c r="E8" t="n">
-        <v>25</v>
+        <v>25.2</v>
       </c>
       <c r="F8" t="n">
-        <v>66</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="G8" t="n">
         <v>45.5</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="9">
@@ -708,10 +708,10 @@
         <v>44</v>
       </c>
       <c r="G9" t="n">
-        <v>41.3</v>
+        <v>41.4</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.36</v>
       </c>
       <c r="E10" t="n">
-        <v>34.3</v>
+        <v>34.4</v>
       </c>
       <c r="F10" t="n">
-        <v>47.3</v>
+        <v>47.4</v>
       </c>
       <c r="G10" t="n">
-        <v>40.8</v>
+        <v>40.9</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.98</v>
       </c>
       <c r="E11" t="n">
-        <v>31.7</v>
+        <v>31.8</v>
       </c>
       <c r="F11" t="n">
         <v>42.7</v>
       </c>
       <c r="G11" t="n">
-        <v>37.2</v>
+        <v>37.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>3.28</v>
       </c>
       <c r="E12" t="n">
-        <v>31.3</v>
+        <v>31.5</v>
       </c>
       <c r="F12" t="n">
-        <v>39</v>
+        <v>39.1</v>
       </c>
       <c r="G12" t="n">
-        <v>35.2</v>
+        <v>35.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>3.5</v>
       </c>
       <c r="E13" t="n">
-        <v>28.3</v>
+        <v>28.5</v>
       </c>
       <c r="F13" t="n">
-        <v>40.3</v>
+        <v>40.4</v>
       </c>
       <c r="G13" t="n">
-        <v>34.3</v>
+        <v>34.4</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2.32</v>
       </c>
       <c r="E14" t="n">
-        <v>15.3</v>
+        <v>15.6</v>
       </c>
       <c r="F14" t="n">
         <v>51</v>
       </c>
       <c r="G14" t="n">
-        <v>33.2</v>
+        <v>33.3</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>2.39</v>
       </c>
       <c r="E15" t="n">
-        <v>15</v>
+        <v>15.2</v>
       </c>
       <c r="F15" t="n">
         <v>48</v>
       </c>
       <c r="G15" t="n">
-        <v>31.5</v>
+        <v>31.6</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>7.81</v>
       </c>
       <c r="E16" t="n">
-        <v>12</v>
+        <v>12.3</v>
       </c>
       <c r="F16" t="n">
         <v>50</v>
       </c>
       <c r="G16" t="n">
-        <v>31</v>
+        <v>31.1</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.31</v>
       </c>
       <c r="E17" t="n">
-        <v>17.3</v>
+        <v>17.5</v>
       </c>
       <c r="F17" t="n">
-        <v>41</v>
+        <v>41.1</v>
       </c>
       <c r="G17" t="n">
-        <v>29.2</v>
+        <v>29.3</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>1.92</v>
       </c>
       <c r="E18" t="n">
-        <v>71.7</v>
+        <v>71.5</v>
       </c>
       <c r="F18" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="G18" t="n">
-        <v>25</v>
+        <v>25.2</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.21</v>
       </c>
       <c r="E19" t="n">
-        <v>11.7</v>
+        <v>11.9</v>
       </c>
       <c r="F19" t="n">
-        <v>37.3</v>
+        <v>37.4</v>
       </c>
       <c r="G19" t="n">
-        <v>24.5</v>
+        <v>24.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="20">
@@ -1035,13 +1035,13 @@
         <v>56.3</v>
       </c>
       <c r="F20" t="n">
-        <v>5.3</v>
+        <v>5.6</v>
       </c>
       <c r="G20" t="n">
-        <v>20.6</v>
+        <v>20.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>0.95</v>
       </c>
       <c r="E21" t="n">
-        <v>7.7</v>
+        <v>7.9</v>
       </c>
       <c r="F21" t="n">
-        <v>31.3</v>
+        <v>31.5</v>
       </c>
       <c r="G21" t="n">
-        <v>19.5</v>
+        <v>19.7</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.79</v>
       </c>
       <c r="E22" t="n">
-        <v>11</v>
+        <v>11.3</v>
       </c>
       <c r="F22" t="n">
-        <v>22</v>
+        <v>22.2</v>
       </c>
       <c r="G22" t="n">
-        <v>18.7</v>
+        <v>18.9</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>3.53</v>
       </c>
       <c r="E23" t="n">
-        <v>5.7</v>
+        <v>6</v>
       </c>
       <c r="F23" t="n">
-        <v>18.7</v>
+        <v>18.9</v>
       </c>
       <c r="G23" t="n">
-        <v>14.8</v>
+        <v>15</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.32</v>
       </c>
       <c r="E24" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="F24" t="n">
-        <v>18.3</v>
+        <v>18.5</v>
       </c>
       <c r="G24" t="n">
-        <v>14.3</v>
+        <v>14.6</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>3.59</v>
       </c>
       <c r="E25" t="n">
-        <v>5.7</v>
+        <v>6</v>
       </c>
       <c r="F25" t="n">
-        <v>17</v>
+        <v>17.2</v>
       </c>
       <c r="G25" t="n">
-        <v>13.6</v>
+        <v>13.8</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>0.62</v>
       </c>
       <c r="E26" t="n">
-        <v>36.3</v>
+        <v>36.4</v>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="G26" t="n">
-        <v>12.3</v>
+        <v>12.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>3.76</v>
       </c>
       <c r="E27" t="n">
-        <v>5.7</v>
+        <v>6</v>
       </c>
       <c r="F27" t="n">
-        <v>14</v>
+        <v>14.2</v>
       </c>
       <c r="G27" t="n">
-        <v>11.5</v>
+        <v>11.8</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.01</v>
       </c>
       <c r="E28" t="n">
-        <v>15.7</v>
+        <v>15.9</v>
       </c>
       <c r="F28" t="n">
-        <v>6.3</v>
+        <v>6.6</v>
       </c>
       <c r="G28" t="n">
-        <v>9.1</v>
+        <v>9.4</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.42</v>
       </c>
       <c r="E29" t="n">
-        <v>6.3</v>
+        <v>6.6</v>
       </c>
       <c r="F29" t="n">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="G29" t="n">
-        <v>7.7</v>
+        <v>8</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.18</v>
       </c>
       <c r="E30" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="F30" t="n">
-        <v>7</v>
+        <v>7.3</v>
       </c>
       <c r="G30" t="n">
-        <v>5.4</v>
+        <v>5.7</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.06</v>
       </c>
       <c r="E31" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="F31" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="G31" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.83</v>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="F32" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="G32" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun Sep 27 14:50:33 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>89.40000000000001</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>89.7</v>
+        <v>89.5</v>
       </c>
       <c r="G2" t="n">
-        <v>89.59999999999999</v>
+        <v>89.3</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>0.97</v>
       </c>
       <c r="E3" t="n">
-        <v>64.90000000000001</v>
+        <v>64.8</v>
       </c>
       <c r="F3" t="n">
         <v>47.7</v>
       </c>
       <c r="G3" t="n">
-        <v>56.3</v>
+        <v>56.2</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="4">
@@ -552,7 +552,7 @@
         <v>1.66</v>
       </c>
       <c r="E4" t="n">
-        <v>57</v>
+        <v>56.9</v>
       </c>
       <c r="F4" t="n">
         <v>53.3</v>
@@ -561,7 +561,7 @@
         <v>55.1</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="5">
@@ -585,13 +585,13 @@
         <v>39.1</v>
       </c>
       <c r="F5" t="n">
-        <v>65.90000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="G5" t="n">
         <v>52.5</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="6">
@@ -621,7 +621,7 @@
         <v>51.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.83</v>
       </c>
       <c r="E7" t="n">
-        <v>19.9</v>
+        <v>20.1</v>
       </c>
       <c r="F7" t="n">
-        <v>81.5</v>
+        <v>81.2</v>
       </c>
       <c r="G7" t="n">
         <v>50.7</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>2.07</v>
       </c>
       <c r="E8" t="n">
-        <v>25.2</v>
+        <v>25.3</v>
       </c>
       <c r="F8" t="n">
-        <v>65.90000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="G8" t="n">
-        <v>45.5</v>
+        <v>45.6</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>2.85</v>
       </c>
       <c r="E9" t="n">
-        <v>38.7</v>
+        <v>38.8</v>
       </c>
       <c r="F9" t="n">
-        <v>44</v>
+        <v>44.1</v>
       </c>
       <c r="G9" t="n">
         <v>41.4</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.36</v>
       </c>
       <c r="E10" t="n">
-        <v>34.4</v>
+        <v>34.5</v>
       </c>
       <c r="F10" t="n">
         <v>47.4</v>
       </c>
       <c r="G10" t="n">
-        <v>40.9</v>
+        <v>41</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.98</v>
       </c>
       <c r="E11" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="F11" t="n">
-        <v>42.7</v>
+        <v>42.8</v>
       </c>
       <c r="G11" t="n">
         <v>37.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>3.28</v>
       </c>
       <c r="E12" t="n">
-        <v>31.5</v>
+        <v>31.6</v>
       </c>
       <c r="F12" t="n">
         <v>39.1</v>
       </c>
       <c r="G12" t="n">
-        <v>35.3</v>
+        <v>35.4</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>3.5</v>
       </c>
       <c r="E13" t="n">
-        <v>28.5</v>
+        <v>28.6</v>
       </c>
       <c r="F13" t="n">
-        <v>40.4</v>
+        <v>40.5</v>
       </c>
       <c r="G13" t="n">
-        <v>34.4</v>
+        <v>34.5</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2.32</v>
       </c>
       <c r="E14" t="n">
-        <v>15.6</v>
+        <v>15.8</v>
       </c>
       <c r="F14" t="n">
         <v>51</v>
       </c>
       <c r="G14" t="n">
-        <v>33.3</v>
+        <v>33.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>2.39</v>
       </c>
       <c r="E15" t="n">
-        <v>15.2</v>
+        <v>15.5</v>
       </c>
       <c r="F15" t="n">
         <v>48</v>
       </c>
       <c r="G15" t="n">
-        <v>31.6</v>
+        <v>31.7</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>7.81</v>
       </c>
       <c r="E16" t="n">
-        <v>12.3</v>
+        <v>12.5</v>
       </c>
       <c r="F16" t="n">
         <v>50</v>
       </c>
       <c r="G16" t="n">
-        <v>31.1</v>
+        <v>31.2</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.31</v>
       </c>
       <c r="E17" t="n">
-        <v>17.5</v>
+        <v>17.8</v>
       </c>
       <c r="F17" t="n">
         <v>41.1</v>
       </c>
       <c r="G17" t="n">
-        <v>29.3</v>
+        <v>29.4</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>1.92</v>
       </c>
       <c r="E18" t="n">
-        <v>71.5</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="F18" t="n">
-        <v>5.3</v>
+        <v>5.6</v>
       </c>
       <c r="G18" t="n">
-        <v>25.2</v>
+        <v>25.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.21</v>
       </c>
       <c r="E19" t="n">
-        <v>11.9</v>
+        <v>12.2</v>
       </c>
       <c r="F19" t="n">
-        <v>37.4</v>
+        <v>37.5</v>
       </c>
       <c r="G19" t="n">
-        <v>24.7</v>
+        <v>24.8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>1.69</v>
       </c>
       <c r="E20" t="n">
-        <v>56.3</v>
+        <v>56.2</v>
       </c>
       <c r="F20" t="n">
-        <v>5.6</v>
+        <v>5.9</v>
       </c>
       <c r="G20" t="n">
-        <v>20.8</v>
+        <v>21</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>0.95</v>
       </c>
       <c r="E21" t="n">
-        <v>7.9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F21" t="n">
-        <v>31.5</v>
+        <v>31.6</v>
       </c>
       <c r="G21" t="n">
-        <v>19.7</v>
+        <v>19.9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.79</v>
       </c>
       <c r="E22" t="n">
-        <v>11.3</v>
+        <v>11.5</v>
       </c>
       <c r="F22" t="n">
-        <v>22.2</v>
+        <v>22.4</v>
       </c>
       <c r="G22" t="n">
-        <v>18.9</v>
+        <v>19.1</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>3.53</v>
       </c>
       <c r="E23" t="n">
-        <v>6</v>
+        <v>6.2</v>
       </c>
       <c r="F23" t="n">
-        <v>18.9</v>
+        <v>19.1</v>
       </c>
       <c r="G23" t="n">
-        <v>15</v>
+        <v>15.2</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>2.32</v>
       </c>
       <c r="E24" t="n">
-        <v>5.3</v>
+        <v>5.6</v>
       </c>
       <c r="F24" t="n">
-        <v>18.5</v>
+        <v>18.8</v>
       </c>
       <c r="G24" t="n">
-        <v>14.6</v>
+        <v>14.8</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>3.59</v>
       </c>
       <c r="E25" t="n">
-        <v>6</v>
+        <v>6.2</v>
       </c>
       <c r="F25" t="n">
-        <v>17.2</v>
+        <v>17.4</v>
       </c>
       <c r="G25" t="n">
-        <v>13.8</v>
+        <v>14.1</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>0.62</v>
       </c>
       <c r="E26" t="n">
-        <v>36.4</v>
+        <v>36.5</v>
       </c>
       <c r="F26" t="n">
-        <v>2.3</v>
+        <v>2.6</v>
       </c>
       <c r="G26" t="n">
-        <v>12.5</v>
+        <v>12.8</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>3.76</v>
       </c>
       <c r="E27" t="n">
-        <v>6</v>
+        <v>6.2</v>
       </c>
       <c r="F27" t="n">
-        <v>14.2</v>
+        <v>14.5</v>
       </c>
       <c r="G27" t="n">
-        <v>11.8</v>
+        <v>12</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.01</v>
       </c>
       <c r="E28" t="n">
-        <v>15.9</v>
+        <v>16.1</v>
       </c>
       <c r="F28" t="n">
-        <v>6.6</v>
+        <v>6.9</v>
       </c>
       <c r="G28" t="n">
-        <v>9.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.42</v>
       </c>
       <c r="E29" t="n">
-        <v>6.6</v>
+        <v>6.9</v>
       </c>
       <c r="F29" t="n">
-        <v>8.6</v>
+        <v>8.9</v>
       </c>
       <c r="G29" t="n">
-        <v>8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>1.18</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="F30" t="n">
-        <v>7.3</v>
+        <v>7.6</v>
       </c>
       <c r="G30" t="n">
-        <v>5.7</v>
+        <v>6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.06</v>
       </c>
       <c r="E31" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="F31" t="n">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="G31" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.83</v>
       </c>
       <c r="E32" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="F32" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="G32" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon Sep 28 17:49:33 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,802 +486,802 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.31</v>
+        <v>7.32</v>
       </c>
       <c r="D2" t="n">
         <v>0.6899999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>89.09999999999999</v>
+        <v>91.8</v>
       </c>
       <c r="F2" t="n">
-        <v>89.5</v>
+        <v>89.2</v>
       </c>
       <c r="G2" t="n">
-        <v>89.3</v>
+        <v>90.5</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>19.89</v>
+        <v>28.06</v>
       </c>
       <c r="D3" t="n">
-        <v>0.97</v>
+        <v>2.7</v>
       </c>
       <c r="E3" t="n">
-        <v>64.8</v>
+        <v>40.5</v>
       </c>
       <c r="F3" t="n">
-        <v>47.7</v>
+        <v>65.7</v>
       </c>
       <c r="G3" t="n">
-        <v>56.2</v>
+        <v>53.1</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>19.86</v>
+        <v>19.61</v>
       </c>
       <c r="D4" t="n">
-        <v>1.66</v>
+        <v>0.96</v>
       </c>
       <c r="E4" t="n">
-        <v>56.9</v>
+        <v>62.7</v>
       </c>
       <c r="F4" t="n">
-        <v>53.3</v>
+        <v>42.8</v>
       </c>
       <c r="G4" t="n">
-        <v>55.1</v>
+        <v>52.8</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>28.05</v>
+        <v>16.99</v>
       </c>
       <c r="D5" t="n">
-        <v>2.7</v>
+        <v>1.83</v>
       </c>
       <c r="E5" t="n">
-        <v>39.1</v>
+        <v>22.5</v>
       </c>
       <c r="F5" t="n">
-        <v>65.8</v>
+        <v>81</v>
       </c>
       <c r="G5" t="n">
-        <v>52.5</v>
+        <v>51.8</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>22.25</v>
+        <v>12.79</v>
       </c>
       <c r="D6" t="n">
-        <v>2.07</v>
+        <v>1.34</v>
       </c>
       <c r="E6" t="n">
-        <v>47.7</v>
+        <v>23.5</v>
       </c>
       <c r="F6" t="n">
-        <v>54.6</v>
+        <v>59.8</v>
       </c>
       <c r="G6" t="n">
-        <v>51.2</v>
+        <v>41.7</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>16.93</v>
+        <v>21.86</v>
       </c>
       <c r="D7" t="n">
-        <v>1.83</v>
+        <v>2.03</v>
       </c>
       <c r="E7" t="n">
-        <v>20.1</v>
+        <v>35.9</v>
       </c>
       <c r="F7" t="n">
-        <v>81.2</v>
+        <v>44.4</v>
       </c>
       <c r="G7" t="n">
-        <v>50.7</v>
+        <v>40.2</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>33.07</v>
+        <v>19.51</v>
       </c>
       <c r="D8" t="n">
-        <v>2.07</v>
+        <v>1.63</v>
       </c>
       <c r="E8" t="n">
-        <v>25.3</v>
+        <v>36.3</v>
       </c>
       <c r="F8" t="n">
-        <v>65.8</v>
+        <v>35.6</v>
       </c>
       <c r="G8" t="n">
-        <v>45.6</v>
+        <v>35.9</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>29.7</v>
+        <v>19.48</v>
       </c>
       <c r="D9" t="n">
-        <v>2.85</v>
+        <v>3.49</v>
       </c>
       <c r="E9" t="n">
-        <v>38.8</v>
+        <v>26.8</v>
       </c>
       <c r="F9" t="n">
-        <v>44.1</v>
+        <v>36.3</v>
       </c>
       <c r="G9" t="n">
-        <v>41.4</v>
+        <v>31.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>30.08</v>
+        <v>14.3</v>
       </c>
       <c r="D10" t="n">
-        <v>2.36</v>
+        <v>1.21</v>
       </c>
       <c r="E10" t="n">
-        <v>34.5</v>
+        <v>12.4</v>
       </c>
       <c r="F10" t="n">
-        <v>47.4</v>
+        <v>37.6</v>
       </c>
       <c r="G10" t="n">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>23.63</v>
+        <v>14.96</v>
       </c>
       <c r="D11" t="n">
-        <v>1.98</v>
+        <v>2.3</v>
       </c>
       <c r="E11" t="n">
-        <v>31.9</v>
+        <v>5.9</v>
       </c>
       <c r="F11" t="n">
-        <v>42.8</v>
+        <v>43.8</v>
       </c>
       <c r="G11" t="n">
-        <v>37.3</v>
+        <v>24.8</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>37.32</v>
+        <v>29.4</v>
       </c>
       <c r="D12" t="n">
-        <v>3.28</v>
+        <v>2.31</v>
       </c>
       <c r="E12" t="n">
-        <v>31.6</v>
+        <v>15.7</v>
       </c>
       <c r="F12" t="n">
-        <v>39.1</v>
+        <v>26.5</v>
       </c>
       <c r="G12" t="n">
-        <v>35.4</v>
+        <v>23.2</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>19.51</v>
+        <v>31.5</v>
       </c>
       <c r="D13" t="n">
-        <v>3.5</v>
+        <v>1.89</v>
       </c>
       <c r="E13" t="n">
-        <v>28.6</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="F13" t="n">
-        <v>40.5</v>
+        <v>3.6</v>
       </c>
       <c r="G13" t="n">
-        <v>34.5</v>
+        <v>23.1</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>15.11</v>
+        <v>26.37</v>
       </c>
       <c r="D14" t="n">
-        <v>2.32</v>
+        <v>2.36</v>
       </c>
       <c r="E14" t="n">
-        <v>15.8</v>
+        <v>10.5</v>
       </c>
       <c r="F14" t="n">
-        <v>51</v>
+        <v>34.3</v>
       </c>
       <c r="G14" t="n">
-        <v>33.4</v>
+        <v>22.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>26.73</v>
+        <v>19.96</v>
       </c>
       <c r="D15" t="n">
-        <v>2.39</v>
+        <v>1.69</v>
       </c>
       <c r="E15" t="n">
-        <v>15.5</v>
+        <v>58.8</v>
       </c>
       <c r="F15" t="n">
-        <v>48</v>
+        <v>6.2</v>
       </c>
       <c r="G15" t="n">
-        <v>31.7</v>
+        <v>22</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>52.64</v>
+        <v>8.56</v>
       </c>
       <c r="D16" t="n">
-        <v>7.81</v>
+        <v>0.95</v>
       </c>
       <c r="E16" t="n">
-        <v>12.5</v>
+        <v>11.1</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>31.7</v>
       </c>
       <c r="G16" t="n">
-        <v>31.2</v>
+        <v>21.4</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>12.55</v>
+        <v>23.06</v>
       </c>
       <c r="D17" t="n">
-        <v>1.31</v>
+        <v>1.93</v>
       </c>
       <c r="E17" t="n">
-        <v>17.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F17" t="n">
-        <v>41.1</v>
+        <v>24.5</v>
       </c>
       <c r="G17" t="n">
-        <v>29.4</v>
+        <v>19.9</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>31.96</v>
+        <v>31.43</v>
       </c>
       <c r="D18" t="n">
-        <v>1.92</v>
+        <v>1.95</v>
       </c>
       <c r="E18" t="n">
-        <v>71.40000000000001</v>
+        <v>5.9</v>
       </c>
       <c r="F18" t="n">
-        <v>5.6</v>
+        <v>33</v>
       </c>
       <c r="G18" t="n">
-        <v>25.3</v>
+        <v>19.4</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>14.3</v>
+        <v>50.2</v>
       </c>
       <c r="D19" t="n">
-        <v>1.21</v>
+        <v>7.45</v>
       </c>
       <c r="E19" t="n">
-        <v>12.2</v>
+        <v>0.7</v>
       </c>
       <c r="F19" t="n">
-        <v>37.5</v>
+        <v>24.8</v>
       </c>
       <c r="G19" t="n">
-        <v>24.8</v>
+        <v>17.6</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>19.91</v>
+        <v>36.03</v>
       </c>
       <c r="D20" t="n">
-        <v>1.69</v>
+        <v>3.17</v>
       </c>
       <c r="E20" t="n">
-        <v>56.2</v>
+        <v>11.8</v>
       </c>
       <c r="F20" t="n">
-        <v>5.9</v>
+        <v>16.7</v>
       </c>
       <c r="G20" t="n">
-        <v>21</v>
+        <v>15.2</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>8.49</v>
+        <v>20.8</v>
       </c>
       <c r="D21" t="n">
-        <v>0.95</v>
+        <v>1.77</v>
       </c>
       <c r="E21" t="n">
-        <v>8.199999999999999</v>
+        <v>3.9</v>
       </c>
       <c r="F21" t="n">
-        <v>31.6</v>
+        <v>17.6</v>
       </c>
       <c r="G21" t="n">
-        <v>19.9</v>
+        <v>13.5</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>21.06</v>
+        <v>10.33</v>
       </c>
       <c r="D22" t="n">
-        <v>1.79</v>
+        <v>0.61</v>
       </c>
       <c r="E22" t="n">
-        <v>11.5</v>
+        <v>30.7</v>
       </c>
       <c r="F22" t="n">
-        <v>22.4</v>
+        <v>0.7</v>
       </c>
       <c r="G22" t="n">
-        <v>19.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>51.56</v>
+        <v>65.56999999999999</v>
       </c>
       <c r="D23" t="n">
-        <v>3.53</v>
+        <v>3.48</v>
       </c>
       <c r="E23" t="n">
-        <v>6.2</v>
+        <v>1.3</v>
       </c>
       <c r="F23" t="n">
-        <v>19.1</v>
+        <v>12.4</v>
       </c>
       <c r="G23" t="n">
-        <v>15.2</v>
+        <v>9.1</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>22.21</v>
+        <v>50.43</v>
       </c>
       <c r="D24" t="n">
-        <v>2.32</v>
+        <v>3.45</v>
       </c>
       <c r="E24" t="n">
-        <v>5.6</v>
+        <v>0.7</v>
       </c>
       <c r="F24" t="n">
-        <v>18.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G24" t="n">
-        <v>14.8</v>
+        <v>6.6</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>67.78</v>
+        <v>28.27</v>
       </c>
       <c r="D25" t="n">
-        <v>3.59</v>
+        <v>2.71</v>
       </c>
       <c r="E25" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="F25" t="n">
         <v>6.2</v>
       </c>
-      <c r="F25" t="n">
-        <v>17.4</v>
-      </c>
       <c r="G25" t="n">
-        <v>14.1</v>
+        <v>6.1</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>10.51</v>
+        <v>21.57</v>
       </c>
       <c r="D26" t="n">
-        <v>0.62</v>
+        <v>2.25</v>
       </c>
       <c r="E26" t="n">
-        <v>36.5</v>
+        <v>0.7</v>
       </c>
       <c r="F26" t="n">
-        <v>2.6</v>
+        <v>5.6</v>
       </c>
       <c r="G26" t="n">
-        <v>12.8</v>
+        <v>4.1</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>40.38</v>
+        <v>22.07</v>
       </c>
       <c r="D27" t="n">
-        <v>3.76</v>
+        <v>1.98</v>
       </c>
       <c r="E27" t="n">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
       <c r="F27" t="n">
-        <v>14.5</v>
+        <v>1.6</v>
       </c>
       <c r="G27" t="n">
-        <v>12</v>
+        <v>3.1</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>22.4</v>
+        <v>39.37</v>
       </c>
       <c r="D28" t="n">
-        <v>2.01</v>
+        <v>3.67</v>
       </c>
       <c r="E28" t="n">
-        <v>16.1</v>
+        <v>0.7</v>
       </c>
       <c r="F28" t="n">
-        <v>6.9</v>
+        <v>3.9</v>
       </c>
       <c r="G28" t="n">
-        <v>9.699999999999999</v>
+        <v>2.9</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="29">
@@ -1296,22 +1296,22 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>18.62</v>
+        <v>18.24</v>
       </c>
       <c r="D29" t="n">
-        <v>1.42</v>
+        <v>1.4</v>
       </c>
       <c r="E29" t="n">
-        <v>6.9</v>
+        <v>0.7</v>
       </c>
       <c r="F29" t="n">
-        <v>8.9</v>
+        <v>3.3</v>
       </c>
       <c r="G29" t="n">
-        <v>8.300000000000001</v>
+        <v>2.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="30">
@@ -1326,22 +1326,22 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>7.64</v>
+        <v>7.52</v>
       </c>
       <c r="D30" t="n">
-        <v>1.18</v>
+        <v>1.16</v>
       </c>
       <c r="E30" t="n">
-        <v>2.3</v>
+        <v>0.7</v>
       </c>
       <c r="F30" t="n">
-        <v>7.6</v>
+        <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>6</v>
+        <v>0.9</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="31">
@@ -1356,22 +1356,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>16.37</v>
+        <v>15.77</v>
       </c>
       <c r="D31" t="n">
-        <v>3.06</v>
+        <v>2.95</v>
       </c>
       <c r="E31" t="n">
-        <v>1.6</v>
+        <v>0.7</v>
       </c>
       <c r="F31" t="n">
-        <v>3.3</v>
+        <v>0.7</v>
       </c>
       <c r="G31" t="n">
-        <v>2.8</v>
+        <v>0.7</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="32">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25.13</v>
+        <v>24.55</v>
       </c>
       <c r="D32" t="n">
-        <v>2.83</v>
+        <v>2.76</v>
       </c>
       <c r="E32" t="n">
-        <v>1.6</v>
+        <v>0.7</v>
       </c>
       <c r="F32" t="n">
-        <v>1.6</v>
+        <v>0.7</v>
       </c>
       <c r="G32" t="n">
-        <v>1.6</v>
+        <v>0.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue Sep 29 16:08:15 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.32</v>
+        <v>7.34</v>
       </c>
       <c r="D2" t="n">
         <v>0.6899999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>91.8</v>
+        <v>93.2</v>
       </c>
       <c r="F2" t="n">
-        <v>89.2</v>
+        <v>89</v>
       </c>
       <c r="G2" t="n">
-        <v>90.5</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="3">
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28.06</v>
+        <v>28.07</v>
       </c>
       <c r="D3" t="n">
         <v>2.7</v>
       </c>
       <c r="E3" t="n">
-        <v>40.5</v>
+        <v>40.9</v>
       </c>
       <c r="F3" t="n">
-        <v>65.7</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>53.1</v>
+        <v>53.2</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="4">
@@ -546,232 +546,232 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>19.61</v>
+        <v>19.7</v>
       </c>
       <c r="D4" t="n">
         <v>0.96</v>
       </c>
       <c r="E4" t="n">
-        <v>62.7</v>
+        <v>63</v>
       </c>
       <c r="F4" t="n">
-        <v>42.8</v>
+        <v>42.9</v>
       </c>
       <c r="G4" t="n">
-        <v>52.8</v>
+        <v>52.9</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>16.99</v>
+        <v>21.94</v>
       </c>
       <c r="D5" t="n">
-        <v>1.83</v>
+        <v>2.04</v>
       </c>
       <c r="E5" t="n">
-        <v>22.5</v>
+        <v>39.9</v>
       </c>
       <c r="F5" t="n">
-        <v>81</v>
+        <v>48.1</v>
       </c>
       <c r="G5" t="n">
-        <v>51.8</v>
+        <v>44</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>12.79</v>
+        <v>16.69</v>
       </c>
       <c r="D6" t="n">
-        <v>1.34</v>
+        <v>1.8</v>
       </c>
       <c r="E6" t="n">
-        <v>23.5</v>
+        <v>11</v>
       </c>
       <c r="F6" t="n">
-        <v>59.8</v>
+        <v>67.5</v>
       </c>
       <c r="G6" t="n">
-        <v>41.7</v>
+        <v>39.3</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>21.86</v>
+        <v>8.81</v>
       </c>
       <c r="D7" t="n">
-        <v>2.03</v>
+        <v>0.98</v>
       </c>
       <c r="E7" t="n">
-        <v>35.9</v>
+        <v>24</v>
       </c>
       <c r="F7" t="n">
-        <v>44.4</v>
+        <v>53.2</v>
       </c>
       <c r="G7" t="n">
-        <v>40.2</v>
+        <v>38.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19.51</v>
+        <v>12.65</v>
       </c>
       <c r="D8" t="n">
-        <v>1.63</v>
+        <v>1.33</v>
       </c>
       <c r="E8" t="n">
-        <v>36.3</v>
+        <v>21.1</v>
       </c>
       <c r="F8" t="n">
-        <v>35.6</v>
+        <v>53.2</v>
       </c>
       <c r="G8" t="n">
-        <v>35.9</v>
+        <v>37.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>19.48</v>
+        <v>19.5</v>
       </c>
       <c r="D9" t="n">
-        <v>3.49</v>
+        <v>1.63</v>
       </c>
       <c r="E9" t="n">
-        <v>26.8</v>
+        <v>34.7</v>
       </c>
       <c r="F9" t="n">
-        <v>36.3</v>
+        <v>35.7</v>
       </c>
       <c r="G9" t="n">
-        <v>31.5</v>
+        <v>35.2</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>14.3</v>
+        <v>23.51</v>
       </c>
       <c r="D10" t="n">
-        <v>1.21</v>
+        <v>1.97</v>
       </c>
       <c r="E10" t="n">
-        <v>12.4</v>
+        <v>22.4</v>
       </c>
       <c r="F10" t="n">
-        <v>37.6</v>
+        <v>38.6</v>
       </c>
       <c r="G10" t="n">
-        <v>25</v>
+        <v>30.5</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>14.96</v>
+        <v>19.41</v>
       </c>
       <c r="D11" t="n">
-        <v>2.3</v>
+        <v>3.48</v>
       </c>
       <c r="E11" t="n">
-        <v>5.9</v>
+        <v>23.4</v>
       </c>
       <c r="F11" t="n">
-        <v>43.8</v>
+        <v>34.7</v>
       </c>
       <c r="G11" t="n">
-        <v>24.8</v>
+        <v>29.1</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="12">
@@ -786,232 +786,232 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>29.4</v>
+        <v>29.41</v>
       </c>
       <c r="D12" t="n">
         <v>2.31</v>
       </c>
       <c r="E12" t="n">
-        <v>15.7</v>
+        <v>16.2</v>
       </c>
       <c r="F12" t="n">
-        <v>26.5</v>
+        <v>26.6</v>
       </c>
       <c r="G12" t="n">
-        <v>23.2</v>
+        <v>23.5</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>31.5</v>
+        <v>14.23</v>
       </c>
       <c r="D13" t="n">
-        <v>1.89</v>
+        <v>1.2</v>
       </c>
       <c r="E13" t="n">
-        <v>68.59999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="F13" t="n">
-        <v>3.6</v>
+        <v>29.5</v>
       </c>
       <c r="G13" t="n">
-        <v>23.1</v>
+        <v>23</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>26.37</v>
+        <v>31.7</v>
       </c>
       <c r="D14" t="n">
-        <v>2.36</v>
+        <v>1.98</v>
       </c>
       <c r="E14" t="n">
-        <v>10.5</v>
+        <v>7.8</v>
       </c>
       <c r="F14" t="n">
-        <v>34.3</v>
+        <v>37.3</v>
       </c>
       <c r="G14" t="n">
-        <v>22.4</v>
+        <v>22.6</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>19.96</v>
+        <v>14.94</v>
       </c>
       <c r="D15" t="n">
-        <v>1.69</v>
+        <v>2.29</v>
       </c>
       <c r="E15" t="n">
-        <v>58.8</v>
+        <v>5.8</v>
       </c>
       <c r="F15" t="n">
-        <v>6.2</v>
+        <v>39</v>
       </c>
       <c r="G15" t="n">
-        <v>22</v>
+        <v>22.4</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>8.56</v>
+        <v>26.33</v>
       </c>
       <c r="D16" t="n">
-        <v>0.95</v>
+        <v>2.36</v>
       </c>
       <c r="E16" t="n">
-        <v>11.1</v>
+        <v>10.4</v>
       </c>
       <c r="F16" t="n">
-        <v>31.7</v>
+        <v>34.4</v>
       </c>
       <c r="G16" t="n">
-        <v>21.4</v>
+        <v>22.4</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>23.06</v>
+        <v>31.38</v>
       </c>
       <c r="D17" t="n">
-        <v>1.93</v>
+        <v>1.88</v>
       </c>
       <c r="E17" t="n">
-        <v>9.199999999999999</v>
+        <v>68.2</v>
       </c>
       <c r="F17" t="n">
-        <v>24.5</v>
+        <v>1.9</v>
       </c>
       <c r="G17" t="n">
-        <v>19.9</v>
+        <v>21.8</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>31.43</v>
+        <v>50.85</v>
       </c>
       <c r="D18" t="n">
-        <v>1.95</v>
+        <v>7.55</v>
       </c>
       <c r="E18" t="n">
-        <v>5.9</v>
+        <v>3.9</v>
       </c>
       <c r="F18" t="n">
-        <v>33</v>
+        <v>34.1</v>
       </c>
       <c r="G18" t="n">
-        <v>19.4</v>
+        <v>19</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>50.2</v>
+        <v>19.88</v>
       </c>
       <c r="D19" t="n">
-        <v>7.45</v>
+        <v>1.68</v>
       </c>
       <c r="E19" t="n">
-        <v>0.7</v>
+        <v>53.2</v>
       </c>
       <c r="F19" t="n">
-        <v>24.8</v>
+        <v>1.3</v>
       </c>
       <c r="G19" t="n">
-        <v>17.6</v>
+        <v>16.9</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="20">
@@ -1026,22 +1026,22 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>36.03</v>
+        <v>35.99</v>
       </c>
       <c r="D20" t="n">
         <v>3.17</v>
       </c>
       <c r="E20" t="n">
-        <v>11.8</v>
+        <v>11.7</v>
       </c>
       <c r="F20" t="n">
-        <v>16.7</v>
+        <v>16.9</v>
       </c>
       <c r="G20" t="n">
-        <v>15.2</v>
+        <v>15.3</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="21">
@@ -1056,22 +1056,22 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>20.8</v>
+        <v>20.76</v>
       </c>
       <c r="D21" t="n">
-        <v>1.77</v>
+        <v>1.76</v>
       </c>
       <c r="E21" t="n">
         <v>3.9</v>
       </c>
       <c r="F21" t="n">
-        <v>17.6</v>
+        <v>14.9</v>
       </c>
       <c r="G21" t="n">
-        <v>13.5</v>
+        <v>11.6</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="22">
@@ -1086,22 +1086,22 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>10.33</v>
+        <v>10.41</v>
       </c>
       <c r="D22" t="n">
         <v>0.61</v>
       </c>
       <c r="E22" t="n">
-        <v>30.7</v>
+        <v>33.1</v>
       </c>
       <c r="F22" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>9.699999999999999</v>
+        <v>10.6</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="23">
@@ -1116,112 +1116,112 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>65.56999999999999</v>
+        <v>66.03</v>
       </c>
       <c r="D23" t="n">
-        <v>3.48</v>
+        <v>3.5</v>
       </c>
       <c r="E23" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="F23" t="n">
-        <v>12.4</v>
+        <v>13</v>
       </c>
       <c r="G23" t="n">
-        <v>9.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>50.43</v>
+        <v>28.34</v>
       </c>
       <c r="D24" t="n">
-        <v>3.45</v>
+        <v>2.72</v>
       </c>
       <c r="E24" t="n">
-        <v>0.7</v>
+        <v>6.5</v>
       </c>
       <c r="F24" t="n">
-        <v>9.199999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="G24" t="n">
-        <v>6.6</v>
+        <v>8.5</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>28.27</v>
+        <v>50.31</v>
       </c>
       <c r="D25" t="n">
-        <v>2.71</v>
+        <v>3.44</v>
       </c>
       <c r="E25" t="n">
-        <v>5.9</v>
+        <v>0.6</v>
       </c>
       <c r="F25" t="n">
-        <v>6.2</v>
+        <v>7.8</v>
       </c>
       <c r="G25" t="n">
-        <v>6.1</v>
+        <v>5.6</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>21.57</v>
+        <v>39.55</v>
       </c>
       <c r="D26" t="n">
-        <v>2.25</v>
+        <v>3.69</v>
       </c>
       <c r="E26" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="F26" t="n">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="G26" t="n">
-        <v>4.1</v>
+        <v>4.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="27">
@@ -1236,7 +1236,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>22.07</v>
+        <v>22.05</v>
       </c>
       <c r="D27" t="n">
         <v>1.98</v>
@@ -1245,43 +1245,43 @@
         <v>6.5</v>
       </c>
       <c r="F27" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="G27" t="n">
-        <v>3.1</v>
+        <v>3.3</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>39.37</v>
+        <v>21.49</v>
       </c>
       <c r="D28" t="n">
-        <v>3.67</v>
+        <v>2.24</v>
       </c>
       <c r="E28" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="F28" t="n">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
       <c r="G28" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="29">
@@ -1296,112 +1296,112 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>18.24</v>
+        <v>18.36</v>
       </c>
       <c r="D29" t="n">
         <v>1.4</v>
       </c>
       <c r="E29" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="F29" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="G29" t="n">
-        <v>2.5</v>
+        <v>2.9</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>7.52</v>
+        <v>15.97</v>
       </c>
       <c r="D30" t="n">
-        <v>1.16</v>
+        <v>2.99</v>
       </c>
       <c r="E30" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="G30" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>15.77</v>
+        <v>24.62</v>
       </c>
       <c r="D31" t="n">
-        <v>2.95</v>
+        <v>2.77</v>
       </c>
       <c r="E31" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="F31" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="G31" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>24.55</v>
+        <v>7.52</v>
       </c>
       <c r="D32" t="n">
-        <v>2.76</v>
+        <v>1.16</v>
       </c>
       <c r="E32" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="G32" t="n">
-        <v>0.7</v>
+        <v>1.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Wed Sep 30 16:06:28 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.34</v>
+        <v>7.43</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.7</v>
       </c>
       <c r="E2" t="n">
-        <v>93.2</v>
+        <v>99.7</v>
       </c>
       <c r="F2" t="n">
-        <v>89</v>
+        <v>97.7</v>
       </c>
       <c r="G2" t="n">
-        <v>91.09999999999999</v>
+        <v>98.7</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="3">
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28.07</v>
+        <v>28.81</v>
       </c>
       <c r="D3" t="n">
-        <v>2.7</v>
+        <v>2.77</v>
       </c>
       <c r="E3" t="n">
-        <v>40.9</v>
+        <v>69</v>
       </c>
       <c r="F3" t="n">
-        <v>65.59999999999999</v>
+        <v>89</v>
       </c>
       <c r="G3" t="n">
-        <v>53.2</v>
+        <v>79</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="4">
@@ -546,532 +546,532 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>19.7</v>
+        <v>19.97</v>
       </c>
       <c r="D4" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="E4" t="n">
-        <v>63</v>
+        <v>67.7</v>
       </c>
       <c r="F4" t="n">
-        <v>42.9</v>
+        <v>54.8</v>
       </c>
       <c r="G4" t="n">
-        <v>52.9</v>
+        <v>61.3</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>21.94</v>
+        <v>19.76</v>
       </c>
       <c r="D5" t="n">
-        <v>2.04</v>
+        <v>3.54</v>
       </c>
       <c r="E5" t="n">
-        <v>39.9</v>
+        <v>38.4</v>
       </c>
       <c r="F5" t="n">
-        <v>48.1</v>
+        <v>56.8</v>
       </c>
       <c r="G5" t="n">
-        <v>44</v>
+        <v>47.6</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>16.69</v>
+        <v>22.01</v>
       </c>
       <c r="D6" t="n">
-        <v>1.8</v>
+        <v>2.05</v>
       </c>
       <c r="E6" t="n">
-        <v>11</v>
+        <v>41.9</v>
       </c>
       <c r="F6" t="n">
-        <v>67.5</v>
+        <v>49.7</v>
       </c>
       <c r="G6" t="n">
-        <v>39.3</v>
+        <v>45.8</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>8.81</v>
+        <v>16.83</v>
       </c>
       <c r="D7" t="n">
-        <v>0.98</v>
+        <v>1.81</v>
       </c>
       <c r="E7" t="n">
-        <v>24</v>
+        <v>16.8</v>
       </c>
       <c r="F7" t="n">
-        <v>53.2</v>
+        <v>74.8</v>
       </c>
       <c r="G7" t="n">
-        <v>38.6</v>
+        <v>45.8</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>12.65</v>
+        <v>9.07</v>
       </c>
       <c r="D8" t="n">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>21.1</v>
+        <v>24.5</v>
       </c>
       <c r="F8" t="n">
-        <v>53.2</v>
+        <v>63.9</v>
       </c>
       <c r="G8" t="n">
-        <v>37.2</v>
+        <v>44.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>19.5</v>
+        <v>12.71</v>
       </c>
       <c r="D9" t="n">
-        <v>1.63</v>
+        <v>1.33</v>
       </c>
       <c r="E9" t="n">
-        <v>34.7</v>
+        <v>22.3</v>
       </c>
       <c r="F9" t="n">
-        <v>35.7</v>
+        <v>53.2</v>
       </c>
       <c r="G9" t="n">
-        <v>35.2</v>
+        <v>37.7</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>23.51</v>
+        <v>26.83</v>
       </c>
       <c r="D10" t="n">
-        <v>1.97</v>
+        <v>2.4</v>
       </c>
       <c r="E10" t="n">
-        <v>22.4</v>
+        <v>21.3</v>
       </c>
       <c r="F10" t="n">
-        <v>38.6</v>
+        <v>53.2</v>
       </c>
       <c r="G10" t="n">
-        <v>30.5</v>
+        <v>37.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>19.41</v>
+        <v>19.5</v>
       </c>
       <c r="D11" t="n">
-        <v>3.48</v>
+        <v>1.63</v>
       </c>
       <c r="E11" t="n">
-        <v>23.4</v>
+        <v>34.8</v>
       </c>
       <c r="F11" t="n">
-        <v>34.7</v>
+        <v>35.8</v>
       </c>
       <c r="G11" t="n">
-        <v>29.1</v>
+        <v>35.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>29.41</v>
+        <v>23.53</v>
       </c>
       <c r="D12" t="n">
-        <v>2.31</v>
+        <v>1.97</v>
       </c>
       <c r="E12" t="n">
-        <v>16.2</v>
+        <v>24.8</v>
       </c>
       <c r="F12" t="n">
-        <v>26.6</v>
+        <v>38.7</v>
       </c>
       <c r="G12" t="n">
-        <v>23.5</v>
+        <v>31.8</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>14.23</v>
+        <v>20.03</v>
       </c>
       <c r="D13" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="E13" t="n">
-        <v>7.8</v>
+        <v>60</v>
       </c>
       <c r="F13" t="n">
-        <v>29.5</v>
+        <v>16.1</v>
       </c>
       <c r="G13" t="n">
-        <v>23</v>
+        <v>29.3</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>31.7</v>
+        <v>14.35</v>
       </c>
       <c r="D14" t="n">
-        <v>1.98</v>
+        <v>1.21</v>
       </c>
       <c r="E14" t="n">
-        <v>7.8</v>
+        <v>18.4</v>
       </c>
       <c r="F14" t="n">
-        <v>37.3</v>
+        <v>38.1</v>
       </c>
       <c r="G14" t="n">
-        <v>22.6</v>
+        <v>28.2</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>14.94</v>
+        <v>31.87</v>
       </c>
       <c r="D15" t="n">
-        <v>2.29</v>
+        <v>1.91</v>
       </c>
       <c r="E15" t="n">
-        <v>5.8</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>39</v>
+        <v>5.5</v>
       </c>
       <c r="G15" t="n">
-        <v>22.4</v>
+        <v>24.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>26.33</v>
+        <v>14.87</v>
       </c>
       <c r="D16" t="n">
-        <v>2.36</v>
+        <v>2.28</v>
       </c>
       <c r="E16" t="n">
-        <v>10.4</v>
+        <v>3.9</v>
       </c>
       <c r="F16" t="n">
-        <v>34.4</v>
+        <v>34.8</v>
       </c>
       <c r="G16" t="n">
-        <v>22.4</v>
+        <v>19.4</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>31.38</v>
+        <v>31.41</v>
       </c>
       <c r="D17" t="n">
-        <v>1.88</v>
+        <v>1.95</v>
       </c>
       <c r="E17" t="n">
-        <v>68.2</v>
+        <v>5.8</v>
       </c>
       <c r="F17" t="n">
-        <v>1.9</v>
+        <v>32.9</v>
       </c>
       <c r="G17" t="n">
-        <v>21.8</v>
+        <v>19.4</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>50.85</v>
+        <v>29.33</v>
       </c>
       <c r="D18" t="n">
-        <v>7.55</v>
+        <v>2.3</v>
       </c>
       <c r="E18" t="n">
-        <v>3.9</v>
+        <v>12.3</v>
       </c>
       <c r="F18" t="n">
-        <v>34.1</v>
+        <v>21.3</v>
       </c>
       <c r="G18" t="n">
-        <v>19</v>
+        <v>18.6</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>19.88</v>
+        <v>20.92</v>
       </c>
       <c r="D19" t="n">
-        <v>1.68</v>
+        <v>1.78</v>
       </c>
       <c r="E19" t="n">
-        <v>53.2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F19" t="n">
-        <v>1.3</v>
+        <v>21.3</v>
       </c>
       <c r="G19" t="n">
-        <v>16.9</v>
+        <v>17.8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>35.99</v>
+        <v>49.74</v>
       </c>
       <c r="D20" t="n">
-        <v>3.17</v>
+        <v>7.38</v>
       </c>
       <c r="E20" t="n">
-        <v>11.7</v>
+        <v>0.6</v>
       </c>
       <c r="F20" t="n">
-        <v>16.9</v>
+        <v>24.5</v>
       </c>
       <c r="G20" t="n">
-        <v>15.3</v>
+        <v>17.4</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>20.76</v>
+        <v>35.69</v>
       </c>
       <c r="D21" t="n">
-        <v>1.76</v>
+        <v>3.14</v>
       </c>
       <c r="E21" t="n">
-        <v>3.9</v>
+        <v>9</v>
       </c>
       <c r="F21" t="n">
-        <v>14.9</v>
+        <v>14.8</v>
       </c>
       <c r="G21" t="n">
-        <v>11.6</v>
+        <v>13.1</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="22">
@@ -1086,22 +1086,22 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>10.41</v>
+        <v>10.49</v>
       </c>
       <c r="D22" t="n">
         <v>0.61</v>
       </c>
       <c r="E22" t="n">
-        <v>33.1</v>
+        <v>35.5</v>
       </c>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="G22" t="n">
-        <v>10.6</v>
+        <v>11.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="23">
@@ -1116,172 +1116,172 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>66.03</v>
+        <v>66.34999999999999</v>
       </c>
       <c r="D23" t="n">
-        <v>3.5</v>
+        <v>3.52</v>
       </c>
       <c r="E23" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="F23" t="n">
-        <v>13</v>
+        <v>14.5</v>
       </c>
       <c r="G23" t="n">
-        <v>9.699999999999999</v>
+        <v>10.9</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>28.34</v>
+        <v>50.37</v>
       </c>
       <c r="D24" t="n">
-        <v>2.72</v>
+        <v>3.45</v>
       </c>
       <c r="E24" t="n">
-        <v>6.5</v>
+        <v>1.3</v>
       </c>
       <c r="F24" t="n">
-        <v>9.4</v>
+        <v>10</v>
       </c>
       <c r="G24" t="n">
-        <v>8.5</v>
+        <v>7.4</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>50.31</v>
+        <v>22.19</v>
       </c>
       <c r="D25" t="n">
-        <v>3.44</v>
+        <v>1.99</v>
       </c>
       <c r="E25" t="n">
-        <v>0.6</v>
+        <v>13.2</v>
       </c>
       <c r="F25" t="n">
-        <v>7.8</v>
+        <v>3.5</v>
       </c>
       <c r="G25" t="n">
-        <v>5.6</v>
+        <v>6.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>39.55</v>
+        <v>21.6</v>
       </c>
       <c r="D26" t="n">
-        <v>3.69</v>
+        <v>2.26</v>
       </c>
       <c r="E26" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="F26" t="n">
-        <v>5.8</v>
+        <v>7.7</v>
       </c>
       <c r="G26" t="n">
-        <v>4.5</v>
+        <v>6</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>22.05</v>
+        <v>28.13</v>
       </c>
       <c r="D27" t="n">
-        <v>1.98</v>
+        <v>2.7</v>
       </c>
       <c r="E27" t="n">
-        <v>6.5</v>
+        <v>5.8</v>
       </c>
       <c r="F27" t="n">
-        <v>1.9</v>
+        <v>5.8</v>
       </c>
       <c r="G27" t="n">
-        <v>3.3</v>
+        <v>5.8</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>21.49</v>
+        <v>7.56</v>
       </c>
       <c r="D28" t="n">
-        <v>2.24</v>
+        <v>1.17</v>
       </c>
       <c r="E28" t="n">
-        <v>0.6</v>
+        <v>1.9</v>
       </c>
       <c r="F28" t="n">
-        <v>4.2</v>
+        <v>3.9</v>
       </c>
       <c r="G28" t="n">
-        <v>3.1</v>
+        <v>3.3</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="29">
@@ -1296,7 +1296,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>18.36</v>
+        <v>18.35</v>
       </c>
       <c r="D29" t="n">
         <v>1.4</v>
@@ -1305,103 +1305,103 @@
         <v>1.3</v>
       </c>
       <c r="F29" t="n">
-        <v>3.6</v>
+        <v>3.9</v>
       </c>
       <c r="G29" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>15.97</v>
+        <v>39.28</v>
       </c>
       <c r="D30" t="n">
-        <v>2.99</v>
+        <v>3.66</v>
       </c>
       <c r="E30" t="n">
-        <v>1.3</v>
+        <v>0.6</v>
       </c>
       <c r="F30" t="n">
-        <v>1.3</v>
+        <v>2.6</v>
       </c>
       <c r="G30" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>24.62</v>
+        <v>16.15</v>
       </c>
       <c r="D31" t="n">
-        <v>2.77</v>
+        <v>3.04</v>
       </c>
       <c r="E31" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="F31" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="G31" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>7.52</v>
+        <v>24.73</v>
       </c>
       <c r="D32" t="n">
-        <v>1.16</v>
+        <v>2.79</v>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>1.9</v>
       </c>
       <c r="F32" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="G32" t="n">
-        <v>1.2</v>
+        <v>1.9</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu Oct  1 16:42:42 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.7</v>
       </c>
       <c r="E2" t="n">
-        <v>99.7</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>97.7</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>98.7</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>2.77</v>
       </c>
       <c r="E3" t="n">
-        <v>69</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>89</v>
+        <v>88.8</v>
       </c>
       <c r="G3" t="n">
-        <v>79</v>
+        <v>78.8</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>0.98</v>
       </c>
       <c r="E4" t="n">
-        <v>67.7</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="F4" t="n">
         <v>54.8</v>
       </c>
       <c r="G4" t="n">
-        <v>61.3</v>
+        <v>61.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>3.54</v>
       </c>
       <c r="E5" t="n">
-        <v>38.4</v>
+        <v>38.5</v>
       </c>
       <c r="F5" t="n">
-        <v>56.8</v>
+        <v>56.7</v>
       </c>
       <c r="G5" t="n">
         <v>47.6</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="6">
@@ -612,7 +612,7 @@
         <v>2.05</v>
       </c>
       <c r="E6" t="n">
-        <v>41.9</v>
+        <v>42</v>
       </c>
       <c r="F6" t="n">
         <v>49.7</v>
@@ -621,7 +621,7 @@
         <v>45.8</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.81</v>
       </c>
       <c r="E7" t="n">
-        <v>16.8</v>
+        <v>17</v>
       </c>
       <c r="F7" t="n">
-        <v>74.8</v>
+        <v>74.7</v>
       </c>
       <c r="G7" t="n">
         <v>45.8</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>24.5</v>
+        <v>24.7</v>
       </c>
       <c r="F8" t="n">
-        <v>63.9</v>
+        <v>63.8</v>
       </c>
       <c r="G8" t="n">
         <v>44.2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.33</v>
       </c>
       <c r="E9" t="n">
-        <v>22.3</v>
+        <v>22.4</v>
       </c>
       <c r="F9" t="n">
         <v>53.2</v>
       </c>
       <c r="G9" t="n">
-        <v>37.7</v>
+        <v>37.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="10">
@@ -732,7 +732,7 @@
         <v>2.4</v>
       </c>
       <c r="E10" t="n">
-        <v>21.3</v>
+        <v>21.5</v>
       </c>
       <c r="F10" t="n">
         <v>53.2</v>
@@ -741,7 +741,7 @@
         <v>37.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.63</v>
       </c>
       <c r="E11" t="n">
-        <v>34.8</v>
+        <v>34.9</v>
       </c>
       <c r="F11" t="n">
-        <v>35.8</v>
+        <v>35.9</v>
       </c>
       <c r="G11" t="n">
-        <v>35.3</v>
+        <v>35.4</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>1.97</v>
       </c>
       <c r="E12" t="n">
-        <v>24.8</v>
+        <v>25</v>
       </c>
       <c r="F12" t="n">
-        <v>38.7</v>
+        <v>38.8</v>
       </c>
       <c r="G12" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.7</v>
       </c>
       <c r="E13" t="n">
-        <v>60</v>
+        <v>59.9</v>
       </c>
       <c r="F13" t="n">
-        <v>16.1</v>
+        <v>16.3</v>
       </c>
       <c r="G13" t="n">
-        <v>29.3</v>
+        <v>29.4</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.21</v>
       </c>
       <c r="E14" t="n">
-        <v>18.4</v>
+        <v>18.6</v>
       </c>
       <c r="F14" t="n">
         <v>38.1</v>
       </c>
       <c r="G14" t="n">
-        <v>28.2</v>
+        <v>28.4</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.91</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>5.5</v>
+        <v>5.8</v>
       </c>
       <c r="G15" t="n">
-        <v>24.5</v>
+        <v>24.7</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>2.28</v>
       </c>
       <c r="E16" t="n">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
       <c r="F16" t="n">
-        <v>34.8</v>
+        <v>34.9</v>
       </c>
       <c r="G16" t="n">
-        <v>19.4</v>
+        <v>19.6</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.95</v>
       </c>
       <c r="E17" t="n">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
       <c r="F17" t="n">
-        <v>32.9</v>
+        <v>33</v>
       </c>
       <c r="G17" t="n">
-        <v>19.4</v>
+        <v>19.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.3</v>
       </c>
       <c r="E18" t="n">
-        <v>12.3</v>
+        <v>12.5</v>
       </c>
       <c r="F18" t="n">
-        <v>21.3</v>
+        <v>21.5</v>
       </c>
       <c r="G18" t="n">
-        <v>18.6</v>
+        <v>18.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.78</v>
       </c>
       <c r="E19" t="n">
-        <v>9.699999999999999</v>
+        <v>9.9</v>
       </c>
       <c r="F19" t="n">
-        <v>21.3</v>
+        <v>21.5</v>
       </c>
       <c r="G19" t="n">
-        <v>17.8</v>
+        <v>18</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>7.38</v>
       </c>
       <c r="E20" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>24.5</v>
+        <v>24.7</v>
       </c>
       <c r="G20" t="n">
-        <v>17.4</v>
+        <v>17.6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>3.14</v>
       </c>
       <c r="E21" t="n">
-        <v>9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F21" t="n">
-        <v>14.8</v>
+        <v>15.1</v>
       </c>
       <c r="G21" t="n">
-        <v>13.1</v>
+        <v>13.3</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>0.61</v>
       </c>
       <c r="E22" t="n">
-        <v>35.5</v>
+        <v>35.6</v>
       </c>
       <c r="F22" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="G22" t="n">
-        <v>11.5</v>
+        <v>11.8</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>3.52</v>
       </c>
       <c r="E23" t="n">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="F23" t="n">
-        <v>14.5</v>
+        <v>14.7</v>
       </c>
       <c r="G23" t="n">
-        <v>10.9</v>
+        <v>11.2</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>3.45</v>
       </c>
       <c r="E24" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="F24" t="n">
-        <v>10</v>
+        <v>10.3</v>
       </c>
       <c r="G24" t="n">
-        <v>7.4</v>
+        <v>7.7</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.99</v>
       </c>
       <c r="E25" t="n">
-        <v>13.2</v>
+        <v>13.5</v>
       </c>
       <c r="F25" t="n">
-        <v>3.5</v>
+        <v>3.8</v>
       </c>
       <c r="G25" t="n">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.26</v>
       </c>
       <c r="E26" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="F26" t="n">
-        <v>7.7</v>
+        <v>8</v>
       </c>
       <c r="G26" t="n">
-        <v>6</v>
+        <v>6.3</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.7</v>
       </c>
       <c r="E27" t="n">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
       <c r="F27" t="n">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
       <c r="G27" t="n">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>1.17</v>
       </c>
       <c r="E28" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="F28" t="n">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
       <c r="G28" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.4</v>
       </c>
       <c r="E29" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="F29" t="n">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
       <c r="G29" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>3.66</v>
       </c>
       <c r="E30" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="G30" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.04</v>
       </c>
       <c r="E31" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="F31" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="G31" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.79</v>
       </c>
       <c r="E32" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="F32" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="G32" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri Oct  2 15:58:55 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.7</v>
       </c>
       <c r="E2" t="n">
-        <v>99.40000000000001</v>
+        <v>99</v>
       </c>
       <c r="F2" t="n">
-        <v>97.40000000000001</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>98.40000000000001</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>2.77</v>
       </c>
       <c r="E3" t="n">
-        <v>68.90000000000001</v>
+        <v>68.8</v>
       </c>
       <c r="F3" t="n">
-        <v>88.8</v>
+        <v>88.5</v>
       </c>
       <c r="G3" t="n">
-        <v>78.8</v>
+        <v>78.7</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>0.98</v>
       </c>
       <c r="E4" t="n">
-        <v>67.59999999999999</v>
+        <v>67.5</v>
       </c>
       <c r="F4" t="n">
         <v>54.8</v>
       </c>
       <c r="G4" t="n">
-        <v>61.2</v>
+        <v>61.1</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="5">
@@ -591,7 +591,7 @@
         <v>47.6</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="6">
@@ -618,10 +618,10 @@
         <v>49.7</v>
       </c>
       <c r="G6" t="n">
-        <v>45.8</v>
+        <v>45.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.81</v>
       </c>
       <c r="E7" t="n">
-        <v>17</v>
+        <v>17.2</v>
       </c>
       <c r="F7" t="n">
-        <v>74.7</v>
+        <v>74.5</v>
       </c>
       <c r="G7" t="n">
-        <v>45.8</v>
+        <v>45.9</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>24.7</v>
+        <v>24.8</v>
       </c>
       <c r="F8" t="n">
-        <v>63.8</v>
+        <v>63.7</v>
       </c>
       <c r="G8" t="n">
-        <v>44.2</v>
+        <v>44.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.33</v>
       </c>
       <c r="E9" t="n">
-        <v>22.4</v>
+        <v>22.6</v>
       </c>
       <c r="F9" t="n">
         <v>53.2</v>
       </c>
       <c r="G9" t="n">
-        <v>37.8</v>
+        <v>37.9</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.4</v>
       </c>
       <c r="E10" t="n">
-        <v>21.5</v>
+        <v>21.7</v>
       </c>
       <c r="F10" t="n">
         <v>53.2</v>
       </c>
       <c r="G10" t="n">
-        <v>37.3</v>
+        <v>37.4</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.63</v>
       </c>
       <c r="E11" t="n">
-        <v>34.9</v>
+        <v>35</v>
       </c>
       <c r="F11" t="n">
-        <v>35.9</v>
+        <v>36</v>
       </c>
       <c r="G11" t="n">
-        <v>35.4</v>
+        <v>35.5</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>1.97</v>
       </c>
       <c r="E12" t="n">
-        <v>25</v>
+        <v>25.2</v>
       </c>
       <c r="F12" t="n">
-        <v>38.8</v>
+        <v>38.9</v>
       </c>
       <c r="G12" t="n">
-        <v>31.9</v>
+        <v>32</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="13">
@@ -825,13 +825,13 @@
         <v>59.9</v>
       </c>
       <c r="F13" t="n">
-        <v>16.3</v>
+        <v>16.6</v>
       </c>
       <c r="G13" t="n">
-        <v>29.4</v>
+        <v>29.6</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.21</v>
       </c>
       <c r="E14" t="n">
-        <v>18.6</v>
+        <v>18.8</v>
       </c>
       <c r="F14" t="n">
-        <v>38.1</v>
+        <v>38.2</v>
       </c>
       <c r="G14" t="n">
-        <v>28.4</v>
+        <v>28.5</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.91</v>
       </c>
       <c r="E15" t="n">
-        <v>68.90000000000001</v>
+        <v>68.8</v>
       </c>
       <c r="F15" t="n">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
       <c r="G15" t="n">
-        <v>24.7</v>
+        <v>24.9</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>2.28</v>
       </c>
       <c r="E16" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="F16" t="n">
-        <v>34.9</v>
+        <v>35</v>
       </c>
       <c r="G16" t="n">
-        <v>19.6</v>
+        <v>19.7</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.95</v>
       </c>
       <c r="E17" t="n">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
       <c r="F17" t="n">
-        <v>33</v>
+        <v>33.1</v>
       </c>
       <c r="G17" t="n">
-        <v>19.6</v>
+        <v>19.7</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.3</v>
       </c>
       <c r="E18" t="n">
-        <v>12.5</v>
+        <v>12.7</v>
       </c>
       <c r="F18" t="n">
-        <v>21.5</v>
+        <v>21.7</v>
       </c>
       <c r="G18" t="n">
-        <v>18.8</v>
+        <v>19</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.78</v>
       </c>
       <c r="E19" t="n">
-        <v>9.9</v>
+        <v>10.2</v>
       </c>
       <c r="F19" t="n">
-        <v>21.5</v>
+        <v>21.7</v>
       </c>
       <c r="G19" t="n">
-        <v>18</v>
+        <v>18.2</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>7.38</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="F20" t="n">
-        <v>24.7</v>
+        <v>24.8</v>
       </c>
       <c r="G20" t="n">
-        <v>17.6</v>
+        <v>17.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>3.14</v>
       </c>
       <c r="E21" t="n">
-        <v>9.300000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="F21" t="n">
-        <v>15.1</v>
+        <v>15.3</v>
       </c>
       <c r="G21" t="n">
-        <v>13.3</v>
+        <v>13.6</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>0.61</v>
       </c>
       <c r="E22" t="n">
-        <v>35.6</v>
+        <v>35.7</v>
       </c>
       <c r="F22" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="G22" t="n">
-        <v>11.8</v>
+        <v>12</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>3.52</v>
       </c>
       <c r="E23" t="n">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
       <c r="F23" t="n">
-        <v>14.7</v>
+        <v>15</v>
       </c>
       <c r="G23" t="n">
-        <v>11.2</v>
+        <v>11.4</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>3.45</v>
       </c>
       <c r="E24" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="F24" t="n">
-        <v>10.3</v>
+        <v>10.5</v>
       </c>
       <c r="G24" t="n">
-        <v>7.7</v>
+        <v>7.9</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.99</v>
       </c>
       <c r="E25" t="n">
-        <v>13.5</v>
+        <v>13.7</v>
       </c>
       <c r="F25" t="n">
-        <v>3.8</v>
+        <v>4.1</v>
       </c>
       <c r="G25" t="n">
-        <v>6.7</v>
+        <v>7</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.26</v>
       </c>
       <c r="E26" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="F26" t="n">
-        <v>8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G26" t="n">
-        <v>6.3</v>
+        <v>6.6</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.7</v>
       </c>
       <c r="E27" t="n">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
       <c r="F27" t="n">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
       <c r="G27" t="n">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>1.17</v>
       </c>
       <c r="E28" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="F28" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="G28" t="n">
-        <v>3.6</v>
+        <v>3.9</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.4</v>
       </c>
       <c r="E29" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="F29" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="G29" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>3.66</v>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="F30" t="n">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
       <c r="G30" t="n">
-        <v>2.3</v>
+        <v>2.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.04</v>
       </c>
       <c r="E31" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="F31" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="G31" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.79</v>
       </c>
       <c r="E32" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="F32" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="G32" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat Oct  3 14:26:08 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.7</v>
       </c>
       <c r="E2" t="n">
-        <v>99</v>
+        <v>98.7</v>
       </c>
       <c r="F2" t="n">
-        <v>97.09999999999999</v>
+        <v>96.8</v>
       </c>
       <c r="G2" t="n">
-        <v>98.09999999999999</v>
+        <v>97.8</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>2.77</v>
       </c>
       <c r="E3" t="n">
-        <v>68.8</v>
+        <v>68.7</v>
       </c>
       <c r="F3" t="n">
-        <v>88.5</v>
+        <v>88.3</v>
       </c>
       <c r="G3" t="n">
-        <v>78.7</v>
+        <v>78.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>0.98</v>
       </c>
       <c r="E4" t="n">
-        <v>67.5</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>54.8</v>
+        <v>54.7</v>
       </c>
       <c r="G4" t="n">
         <v>61.1</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>3.54</v>
       </c>
       <c r="E5" t="n">
-        <v>38.5</v>
+        <v>38.6</v>
       </c>
       <c r="F5" t="n">
-        <v>56.7</v>
+        <v>56.6</v>
       </c>
       <c r="G5" t="n">
         <v>47.6</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="6">
@@ -612,7 +612,7 @@
         <v>2.05</v>
       </c>
       <c r="E6" t="n">
-        <v>42</v>
+        <v>42.1</v>
       </c>
       <c r="F6" t="n">
         <v>49.7</v>
@@ -621,7 +621,7 @@
         <v>45.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.81</v>
       </c>
       <c r="E7" t="n">
-        <v>17.2</v>
+        <v>17.4</v>
       </c>
       <c r="F7" t="n">
-        <v>74.5</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="G7" t="n">
         <v>45.9</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>24.8</v>
+        <v>25</v>
       </c>
       <c r="F8" t="n">
-        <v>63.7</v>
+        <v>63.6</v>
       </c>
       <c r="G8" t="n">
         <v>44.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.33</v>
       </c>
       <c r="E9" t="n">
-        <v>22.6</v>
+        <v>22.8</v>
       </c>
       <c r="F9" t="n">
         <v>53.2</v>
       </c>
       <c r="G9" t="n">
-        <v>37.9</v>
+        <v>38</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.4</v>
       </c>
       <c r="E10" t="n">
-        <v>21.7</v>
+        <v>21.8</v>
       </c>
       <c r="F10" t="n">
         <v>53.2</v>
       </c>
       <c r="G10" t="n">
-        <v>37.4</v>
+        <v>37.5</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.63</v>
       </c>
       <c r="E11" t="n">
-        <v>35</v>
+        <v>35.1</v>
       </c>
       <c r="F11" t="n">
-        <v>36</v>
+        <v>36.1</v>
       </c>
       <c r="G11" t="n">
-        <v>35.5</v>
+        <v>35.6</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>1.97</v>
       </c>
       <c r="E12" t="n">
-        <v>25.2</v>
+        <v>25.3</v>
       </c>
       <c r="F12" t="n">
         <v>38.9</v>
       </c>
       <c r="G12" t="n">
-        <v>32</v>
+        <v>32.1</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.7</v>
       </c>
       <c r="E13" t="n">
-        <v>59.9</v>
+        <v>59.8</v>
       </c>
       <c r="F13" t="n">
-        <v>16.6</v>
+        <v>16.8</v>
       </c>
       <c r="G13" t="n">
-        <v>29.6</v>
+        <v>29.7</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.21</v>
       </c>
       <c r="E14" t="n">
-        <v>18.8</v>
+        <v>19</v>
       </c>
       <c r="F14" t="n">
-        <v>38.2</v>
+        <v>38.3</v>
       </c>
       <c r="G14" t="n">
-        <v>28.5</v>
+        <v>28.6</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.91</v>
       </c>
       <c r="E15" t="n">
-        <v>68.8</v>
+        <v>68.7</v>
       </c>
       <c r="F15" t="n">
-        <v>6.1</v>
+        <v>6.3</v>
       </c>
       <c r="G15" t="n">
-        <v>24.9</v>
+        <v>25</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>2.28</v>
       </c>
       <c r="E16" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="F16" t="n">
-        <v>35</v>
+        <v>35.1</v>
       </c>
       <c r="G16" t="n">
-        <v>19.7</v>
+        <v>19.9</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.95</v>
       </c>
       <c r="E17" t="n">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="F17" t="n">
-        <v>33.1</v>
+        <v>33.2</v>
       </c>
       <c r="G17" t="n">
-        <v>19.7</v>
+        <v>19.9</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.3</v>
       </c>
       <c r="E18" t="n">
-        <v>12.7</v>
+        <v>13</v>
       </c>
       <c r="F18" t="n">
-        <v>21.7</v>
+        <v>21.8</v>
       </c>
       <c r="G18" t="n">
-        <v>19</v>
+        <v>19.2</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.78</v>
       </c>
       <c r="E19" t="n">
-        <v>10.2</v>
+        <v>10.4</v>
       </c>
       <c r="F19" t="n">
-        <v>21.7</v>
+        <v>21.8</v>
       </c>
       <c r="G19" t="n">
-        <v>18.2</v>
+        <v>18.4</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>7.38</v>
       </c>
       <c r="E20" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="F20" t="n">
-        <v>24.8</v>
+        <v>25</v>
       </c>
       <c r="G20" t="n">
-        <v>17.8</v>
+        <v>18</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>3.14</v>
       </c>
       <c r="E21" t="n">
-        <v>9.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F21" t="n">
-        <v>15.3</v>
+        <v>15.5</v>
       </c>
       <c r="G21" t="n">
-        <v>13.6</v>
+        <v>13.8</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>0.61</v>
       </c>
       <c r="E22" t="n">
-        <v>35.7</v>
+        <v>35.8</v>
       </c>
       <c r="F22" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="G22" t="n">
-        <v>12</v>
+        <v>12.3</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>3.52</v>
       </c>
       <c r="E23" t="n">
-        <v>3.2</v>
+        <v>3.5</v>
       </c>
       <c r="F23" t="n">
-        <v>15</v>
+        <v>15.2</v>
       </c>
       <c r="G23" t="n">
-        <v>11.4</v>
+        <v>11.7</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>3.45</v>
       </c>
       <c r="E24" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="F24" t="n">
-        <v>10.5</v>
+        <v>10.8</v>
       </c>
       <c r="G24" t="n">
-        <v>7.9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.99</v>
       </c>
       <c r="E25" t="n">
-        <v>13.7</v>
+        <v>13.9</v>
       </c>
       <c r="F25" t="n">
-        <v>4.1</v>
+        <v>4.4</v>
       </c>
       <c r="G25" t="n">
-        <v>7</v>
+        <v>7.3</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.26</v>
       </c>
       <c r="E26" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="F26" t="n">
-        <v>8.300000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="G26" t="n">
-        <v>6.6</v>
+        <v>6.8</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.7</v>
       </c>
       <c r="E27" t="n">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="F27" t="n">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="G27" t="n">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>1.17</v>
       </c>
       <c r="E28" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="F28" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="G28" t="n">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.4</v>
       </c>
       <c r="E29" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="F29" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="G29" t="n">
-        <v>3.7</v>
+        <v>4</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>3.66</v>
       </c>
       <c r="E30" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="F30" t="n">
-        <v>3.2</v>
+        <v>3.5</v>
       </c>
       <c r="G30" t="n">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.04</v>
       </c>
       <c r="E31" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="F31" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="G31" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.79</v>
       </c>
       <c r="E32" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="F32" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="G32" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun Oct  4 15:00:04 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.7</v>
       </c>
       <c r="E2" t="n">
-        <v>98.7</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>96.8</v>
+        <v>96.5</v>
       </c>
       <c r="G2" t="n">
-        <v>97.8</v>
+        <v>97.5</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>2.77</v>
       </c>
       <c r="E3" t="n">
-        <v>68.7</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>88.3</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>78.5</v>
+        <v>78.3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>0.98</v>
       </c>
       <c r="E4" t="n">
-        <v>67.40000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="F4" t="n">
         <v>54.7</v>
       </c>
       <c r="G4" t="n">
-        <v>61.1</v>
+        <v>61</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="5">
@@ -582,7 +582,7 @@
         <v>3.54</v>
       </c>
       <c r="E5" t="n">
-        <v>38.6</v>
+        <v>38.7</v>
       </c>
       <c r="F5" t="n">
         <v>56.6</v>
@@ -591,7 +591,7 @@
         <v>47.6</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="6">
@@ -621,7 +621,7 @@
         <v>45.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.81</v>
       </c>
       <c r="E7" t="n">
-        <v>17.4</v>
+        <v>17.6</v>
       </c>
       <c r="F7" t="n">
-        <v>74.40000000000001</v>
+        <v>74.2</v>
       </c>
       <c r="G7" t="n">
         <v>45.9</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>25</v>
+        <v>25.2</v>
       </c>
       <c r="F8" t="n">
-        <v>63.6</v>
+        <v>63.5</v>
       </c>
       <c r="G8" t="n">
         <v>44.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.33</v>
       </c>
       <c r="E9" t="n">
-        <v>22.8</v>
+        <v>23</v>
       </c>
       <c r="F9" t="n">
-        <v>53.2</v>
+        <v>53.1</v>
       </c>
       <c r="G9" t="n">
-        <v>38</v>
+        <v>38.1</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.4</v>
       </c>
       <c r="E10" t="n">
-        <v>21.8</v>
+        <v>22</v>
       </c>
       <c r="F10" t="n">
-        <v>53.2</v>
+        <v>53.1</v>
       </c>
       <c r="G10" t="n">
-        <v>37.5</v>
+        <v>37.6</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.63</v>
       </c>
       <c r="E11" t="n">
-        <v>35.1</v>
+        <v>35.2</v>
       </c>
       <c r="F11" t="n">
-        <v>36.1</v>
+        <v>36.2</v>
       </c>
       <c r="G11" t="n">
-        <v>35.6</v>
+        <v>35.7</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>1.97</v>
       </c>
       <c r="E12" t="n">
-        <v>25.3</v>
+        <v>25.5</v>
       </c>
       <c r="F12" t="n">
-        <v>38.9</v>
+        <v>39</v>
       </c>
       <c r="G12" t="n">
-        <v>32.1</v>
+        <v>32.2</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.7</v>
       </c>
       <c r="E13" t="n">
-        <v>59.8</v>
+        <v>59.7</v>
       </c>
       <c r="F13" t="n">
-        <v>16.8</v>
+        <v>17</v>
       </c>
       <c r="G13" t="n">
-        <v>29.7</v>
+        <v>29.8</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.21</v>
       </c>
       <c r="E14" t="n">
-        <v>19</v>
+        <v>19.2</v>
       </c>
       <c r="F14" t="n">
-        <v>38.3</v>
+        <v>38.4</v>
       </c>
       <c r="G14" t="n">
-        <v>28.6</v>
+        <v>28.8</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.91</v>
       </c>
       <c r="E15" t="n">
-        <v>68.7</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="F15" t="n">
-        <v>6.3</v>
+        <v>6.6</v>
       </c>
       <c r="G15" t="n">
-        <v>25</v>
+        <v>25.2</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>2.28</v>
       </c>
       <c r="E16" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="F16" t="n">
-        <v>35.1</v>
+        <v>35.2</v>
       </c>
       <c r="G16" t="n">
-        <v>19.9</v>
+        <v>20.1</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.95</v>
       </c>
       <c r="E17" t="n">
-        <v>6.6</v>
+        <v>6.9</v>
       </c>
       <c r="F17" t="n">
-        <v>33.2</v>
+        <v>33.3</v>
       </c>
       <c r="G17" t="n">
-        <v>19.9</v>
+        <v>20.1</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.3</v>
       </c>
       <c r="E18" t="n">
-        <v>13</v>
+        <v>13.2</v>
       </c>
       <c r="F18" t="n">
-        <v>21.8</v>
+        <v>22</v>
       </c>
       <c r="G18" t="n">
-        <v>19.2</v>
+        <v>19.4</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.78</v>
       </c>
       <c r="E19" t="n">
-        <v>10.4</v>
+        <v>10.7</v>
       </c>
       <c r="F19" t="n">
-        <v>21.8</v>
+        <v>22</v>
       </c>
       <c r="G19" t="n">
-        <v>18.4</v>
+        <v>18.6</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>7.38</v>
       </c>
       <c r="E20" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="F20" t="n">
-        <v>25</v>
+        <v>25.2</v>
       </c>
       <c r="G20" t="n">
-        <v>18</v>
+        <v>18.2</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>3.14</v>
       </c>
       <c r="E21" t="n">
-        <v>9.800000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="F21" t="n">
-        <v>15.5</v>
+        <v>15.7</v>
       </c>
       <c r="G21" t="n">
-        <v>13.8</v>
+        <v>14</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="22">
@@ -1095,13 +1095,13 @@
         <v>35.8</v>
       </c>
       <c r="F22" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="G22" t="n">
-        <v>12.3</v>
+        <v>12.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>3.52</v>
       </c>
       <c r="E23" t="n">
-        <v>3.5</v>
+        <v>3.8</v>
       </c>
       <c r="F23" t="n">
-        <v>15.2</v>
+        <v>15.4</v>
       </c>
       <c r="G23" t="n">
-        <v>11.7</v>
+        <v>11.9</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>3.45</v>
       </c>
       <c r="E24" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="F24" t="n">
-        <v>10.8</v>
+        <v>11</v>
       </c>
       <c r="G24" t="n">
-        <v>8.199999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.99</v>
       </c>
       <c r="E25" t="n">
-        <v>13.9</v>
+        <v>14.2</v>
       </c>
       <c r="F25" t="n">
-        <v>4.4</v>
+        <v>4.7</v>
       </c>
       <c r="G25" t="n">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.26</v>
       </c>
       <c r="E26" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="F26" t="n">
-        <v>8.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G26" t="n">
-        <v>6.8</v>
+        <v>7.1</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.7</v>
       </c>
       <c r="E27" t="n">
-        <v>6.6</v>
+        <v>6.9</v>
       </c>
       <c r="F27" t="n">
-        <v>6.6</v>
+        <v>6.9</v>
       </c>
       <c r="G27" t="n">
-        <v>6.6</v>
+        <v>6.9</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>1.17</v>
       </c>
       <c r="E28" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="F28" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="G28" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.4</v>
       </c>
       <c r="E29" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="F29" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="G29" t="n">
-        <v>4</v>
+        <v>4.3</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>3.66</v>
       </c>
       <c r="E30" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="F30" t="n">
-        <v>3.5</v>
+        <v>3.8</v>
       </c>
       <c r="G30" t="n">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.04</v>
       </c>
       <c r="E31" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="F31" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="G31" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.79</v>
       </c>
       <c r="E32" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="F32" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="G32" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon Oct  5 18:50:54 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.7</v>
       </c>
       <c r="E2" t="n">
-        <v>98.40000000000001</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>96.5</v>
+        <v>96.2</v>
       </c>
       <c r="G2" t="n">
-        <v>97.5</v>
+        <v>97.2</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>2.77</v>
       </c>
       <c r="E3" t="n">
-        <v>68.59999999999999</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>88.09999999999999</v>
+        <v>87.8</v>
       </c>
       <c r="G3" t="n">
-        <v>78.3</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +552,16 @@
         <v>0.98</v>
       </c>
       <c r="E4" t="n">
-        <v>67.3</v>
+        <v>67.2</v>
       </c>
       <c r="F4" t="n">
         <v>54.7</v>
       </c>
       <c r="G4" t="n">
-        <v>61</v>
+        <v>60.9</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>3.54</v>
       </c>
       <c r="E5" t="n">
-        <v>38.7</v>
+        <v>38.8</v>
       </c>
       <c r="F5" t="n">
         <v>56.6</v>
       </c>
       <c r="G5" t="n">
-        <v>47.6</v>
+        <v>47.7</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="6">
@@ -612,7 +612,7 @@
         <v>2.05</v>
       </c>
       <c r="E6" t="n">
-        <v>42.1</v>
+        <v>42.2</v>
       </c>
       <c r="F6" t="n">
         <v>49.7</v>
@@ -621,7 +621,7 @@
         <v>45.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.81</v>
       </c>
       <c r="E7" t="n">
-        <v>17.6</v>
+        <v>17.8</v>
       </c>
       <c r="F7" t="n">
-        <v>74.2</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="G7" t="n">
         <v>45.9</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>25.2</v>
+        <v>25.3</v>
       </c>
       <c r="F8" t="n">
-        <v>63.5</v>
+        <v>63.4</v>
       </c>
       <c r="G8" t="n">
-        <v>44.3</v>
+        <v>44.4</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="9">
@@ -702,7 +702,7 @@
         <v>1.33</v>
       </c>
       <c r="E9" t="n">
-        <v>23</v>
+        <v>23.1</v>
       </c>
       <c r="F9" t="n">
         <v>53.1</v>
@@ -711,7 +711,7 @@
         <v>38.1</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>2.4</v>
       </c>
       <c r="E10" t="n">
-        <v>22</v>
+        <v>22.2</v>
       </c>
       <c r="F10" t="n">
         <v>53.1</v>
       </c>
       <c r="G10" t="n">
-        <v>37.6</v>
+        <v>37.7</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.63</v>
       </c>
       <c r="E11" t="n">
-        <v>35.2</v>
+        <v>35.3</v>
       </c>
       <c r="F11" t="n">
         <v>36.2</v>
       </c>
       <c r="G11" t="n">
-        <v>35.7</v>
+        <v>35.8</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>1.97</v>
       </c>
       <c r="E12" t="n">
-        <v>25.5</v>
+        <v>25.6</v>
       </c>
       <c r="F12" t="n">
-        <v>39</v>
+        <v>39.1</v>
       </c>
       <c r="G12" t="n">
-        <v>32.2</v>
+        <v>32.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="13">
@@ -825,13 +825,13 @@
         <v>59.7</v>
       </c>
       <c r="F13" t="n">
-        <v>17</v>
+        <v>17.2</v>
       </c>
       <c r="G13" t="n">
-        <v>29.8</v>
+        <v>29.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.21</v>
       </c>
       <c r="E14" t="n">
-        <v>19.2</v>
+        <v>19.4</v>
       </c>
       <c r="F14" t="n">
         <v>38.4</v>
       </c>
       <c r="G14" t="n">
-        <v>28.8</v>
+        <v>28.9</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.91</v>
       </c>
       <c r="E15" t="n">
-        <v>68.59999999999999</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>6.6</v>
+        <v>6.9</v>
       </c>
       <c r="G15" t="n">
-        <v>25.2</v>
+        <v>25.3</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>2.28</v>
       </c>
       <c r="E16" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="F16" t="n">
-        <v>35.2</v>
+        <v>35.3</v>
       </c>
       <c r="G16" t="n">
-        <v>20.1</v>
+        <v>20.3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.95</v>
       </c>
       <c r="E17" t="n">
-        <v>6.9</v>
+        <v>7.2</v>
       </c>
       <c r="F17" t="n">
-        <v>33.3</v>
+        <v>33.4</v>
       </c>
       <c r="G17" t="n">
-        <v>20.1</v>
+        <v>20.3</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.3</v>
       </c>
       <c r="E18" t="n">
-        <v>13.2</v>
+        <v>13.4</v>
       </c>
       <c r="F18" t="n">
-        <v>22</v>
+        <v>22.2</v>
       </c>
       <c r="G18" t="n">
-        <v>19.4</v>
+        <v>19.6</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.78</v>
       </c>
       <c r="E19" t="n">
-        <v>10.7</v>
+        <v>10.9</v>
       </c>
       <c r="F19" t="n">
-        <v>22</v>
+        <v>22.2</v>
       </c>
       <c r="G19" t="n">
-        <v>18.6</v>
+        <v>18.8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>7.38</v>
       </c>
       <c r="E20" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="F20" t="n">
-        <v>25.2</v>
+        <v>25.3</v>
       </c>
       <c r="G20" t="n">
-        <v>18.2</v>
+        <v>18.4</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>3.14</v>
       </c>
       <c r="E21" t="n">
-        <v>10.1</v>
+        <v>10.3</v>
       </c>
       <c r="F21" t="n">
-        <v>15.7</v>
+        <v>15.9</v>
       </c>
       <c r="G21" t="n">
-        <v>14</v>
+        <v>14.2</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>0.61</v>
       </c>
       <c r="E22" t="n">
-        <v>35.8</v>
+        <v>35.9</v>
       </c>
       <c r="F22" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="G22" t="n">
-        <v>12.5</v>
+        <v>12.8</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>3.52</v>
       </c>
       <c r="E23" t="n">
-        <v>3.8</v>
+        <v>4.1</v>
       </c>
       <c r="F23" t="n">
-        <v>15.4</v>
+        <v>15.6</v>
       </c>
       <c r="G23" t="n">
-        <v>11.9</v>
+        <v>12.2</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>3.45</v>
       </c>
       <c r="E24" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="F24" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="G24" t="n">
-        <v>8.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.99</v>
       </c>
       <c r="E25" t="n">
-        <v>14.2</v>
+        <v>14.4</v>
       </c>
       <c r="F25" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="G25" t="n">
-        <v>7.5</v>
+        <v>7.8</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.26</v>
       </c>
       <c r="E26" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="F26" t="n">
-        <v>8.800000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="G26" t="n">
-        <v>7.1</v>
+        <v>7.4</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.7</v>
       </c>
       <c r="E27" t="n">
-        <v>6.9</v>
+        <v>7.2</v>
       </c>
       <c r="F27" t="n">
-        <v>6.9</v>
+        <v>7.2</v>
       </c>
       <c r="G27" t="n">
-        <v>6.9</v>
+        <v>7.2</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>1.17</v>
       </c>
       <c r="E28" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="F28" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="G28" t="n">
-        <v>4.5</v>
+        <v>4.8</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.4</v>
       </c>
       <c r="E29" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="F29" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="G29" t="n">
-        <v>4.3</v>
+        <v>4.6</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>3.66</v>
       </c>
       <c r="E30" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="F30" t="n">
-        <v>3.8</v>
+        <v>4.1</v>
       </c>
       <c r="G30" t="n">
-        <v>3.2</v>
+        <v>3.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.04</v>
       </c>
       <c r="E31" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="F31" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="G31" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.79</v>
       </c>
       <c r="E32" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="F32" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="G32" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue Oct  6 16:17:22 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.7</v>
       </c>
       <c r="E2" t="n">
-        <v>98.09999999999999</v>
+        <v>97.8</v>
       </c>
       <c r="F2" t="n">
-        <v>96.2</v>
+        <v>96</v>
       </c>
       <c r="G2" t="n">
-        <v>97.2</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>2.77</v>
       </c>
       <c r="E3" t="n">
-        <v>68.40000000000001</v>
+        <v>68.3</v>
       </c>
       <c r="F3" t="n">
-        <v>87.8</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>78.09999999999999</v>
+        <v>78</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="4">
@@ -552,7 +552,7 @@
         <v>0.98</v>
       </c>
       <c r="E4" t="n">
-        <v>67.2</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="F4" t="n">
         <v>54.7</v>
@@ -561,7 +561,7 @@
         <v>60.9</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="5">
@@ -585,13 +585,13 @@
         <v>38.8</v>
       </c>
       <c r="F5" t="n">
-        <v>56.6</v>
+        <v>56.5</v>
       </c>
       <c r="G5" t="n">
         <v>47.7</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="6">
@@ -618,10 +618,10 @@
         <v>49.7</v>
       </c>
       <c r="G6" t="n">
-        <v>45.9</v>
+        <v>46</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>1.81</v>
       </c>
       <c r="E7" t="n">
-        <v>17.8</v>
+        <v>18</v>
       </c>
       <c r="F7" t="n">
-        <v>74.09999999999999</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>45.9</v>
+        <v>46</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="8">
@@ -672,7 +672,7 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>25.3</v>
+        <v>25.5</v>
       </c>
       <c r="F8" t="n">
         <v>63.4</v>
@@ -681,7 +681,7 @@
         <v>44.4</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.33</v>
       </c>
       <c r="E9" t="n">
-        <v>23.1</v>
+        <v>23.3</v>
       </c>
       <c r="F9" t="n">
         <v>53.1</v>
       </c>
       <c r="G9" t="n">
-        <v>38.1</v>
+        <v>38.2</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="10">
@@ -732,7 +732,7 @@
         <v>2.4</v>
       </c>
       <c r="E10" t="n">
-        <v>22.2</v>
+        <v>22.4</v>
       </c>
       <c r="F10" t="n">
         <v>53.1</v>
@@ -741,7 +741,7 @@
         <v>37.7</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.63</v>
       </c>
       <c r="E11" t="n">
-        <v>35.3</v>
+        <v>35.4</v>
       </c>
       <c r="F11" t="n">
-        <v>36.2</v>
+        <v>36.3</v>
       </c>
       <c r="G11" t="n">
-        <v>35.8</v>
+        <v>35.9</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>1.97</v>
       </c>
       <c r="E12" t="n">
-        <v>25.6</v>
+        <v>25.8</v>
       </c>
       <c r="F12" t="n">
         <v>39.1</v>
       </c>
       <c r="G12" t="n">
-        <v>32.3</v>
+        <v>32.5</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.7</v>
       </c>
       <c r="E13" t="n">
-        <v>59.7</v>
+        <v>59.6</v>
       </c>
       <c r="F13" t="n">
-        <v>17.2</v>
+        <v>17.4</v>
       </c>
       <c r="G13" t="n">
-        <v>29.9</v>
+        <v>30.1</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>1.21</v>
       </c>
       <c r="E14" t="n">
-        <v>19.4</v>
+        <v>19.6</v>
       </c>
       <c r="F14" t="n">
-        <v>38.4</v>
+        <v>38.5</v>
       </c>
       <c r="G14" t="n">
-        <v>28.9</v>
+        <v>29</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.91</v>
       </c>
       <c r="E15" t="n">
-        <v>68.40000000000001</v>
+        <v>68.3</v>
       </c>
       <c r="F15" t="n">
-        <v>6.9</v>
+        <v>7.1</v>
       </c>
       <c r="G15" t="n">
-        <v>25.3</v>
+        <v>25.5</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>2.28</v>
       </c>
       <c r="E16" t="n">
-        <v>5.3</v>
+        <v>5.6</v>
       </c>
       <c r="F16" t="n">
-        <v>35.3</v>
+        <v>35.4</v>
       </c>
       <c r="G16" t="n">
-        <v>20.3</v>
+        <v>20.5</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>1.95</v>
       </c>
       <c r="E17" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="F17" t="n">
-        <v>33.4</v>
+        <v>33.5</v>
       </c>
       <c r="G17" t="n">
-        <v>20.3</v>
+        <v>20.5</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.3</v>
       </c>
       <c r="E18" t="n">
-        <v>13.4</v>
+        <v>13.7</v>
       </c>
       <c r="F18" t="n">
-        <v>22.2</v>
+        <v>22.4</v>
       </c>
       <c r="G18" t="n">
-        <v>19.6</v>
+        <v>19.8</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.78</v>
       </c>
       <c r="E19" t="n">
-        <v>10.9</v>
+        <v>11.2</v>
       </c>
       <c r="F19" t="n">
-        <v>22.2</v>
+        <v>22.4</v>
       </c>
       <c r="G19" t="n">
-        <v>18.8</v>
+        <v>19</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>7.38</v>
       </c>
       <c r="E20" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="F20" t="n">
-        <v>25.3</v>
+        <v>25.5</v>
       </c>
       <c r="G20" t="n">
-        <v>18.4</v>
+        <v>18.6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>3.14</v>
       </c>
       <c r="E21" t="n">
-        <v>10.3</v>
+        <v>10.6</v>
       </c>
       <c r="F21" t="n">
-        <v>15.9</v>
+        <v>16.1</v>
       </c>
       <c r="G21" t="n">
-        <v>14.2</v>
+        <v>14.5</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>0.61</v>
       </c>
       <c r="E22" t="n">
-        <v>35.9</v>
+        <v>36</v>
       </c>
       <c r="F22" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="G22" t="n">
-        <v>12.8</v>
+        <v>13</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>3.52</v>
       </c>
       <c r="E23" t="n">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
       <c r="F23" t="n">
-        <v>15.6</v>
+        <v>15.8</v>
       </c>
       <c r="G23" t="n">
-        <v>12.2</v>
+        <v>12.4</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>3.45</v>
       </c>
       <c r="E24" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="F24" t="n">
-        <v>11.2</v>
+        <v>11.5</v>
       </c>
       <c r="G24" t="n">
-        <v>8.699999999999999</v>
+        <v>9</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>1.99</v>
       </c>
       <c r="E25" t="n">
-        <v>14.4</v>
+        <v>14.6</v>
       </c>
       <c r="F25" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="G25" t="n">
-        <v>7.8</v>
+        <v>8.1</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.26</v>
       </c>
       <c r="E26" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="F26" t="n">
-        <v>9.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G26" t="n">
-        <v>7.4</v>
+        <v>7.6</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>2.7</v>
       </c>
       <c r="E27" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="F27" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="G27" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>1.17</v>
       </c>
       <c r="E28" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="F28" t="n">
-        <v>5.3</v>
+        <v>5.6</v>
       </c>
       <c r="G28" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.4</v>
       </c>
       <c r="E29" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="F29" t="n">
-        <v>5.3</v>
+        <v>5.6</v>
       </c>
       <c r="G29" t="n">
-        <v>4.6</v>
+        <v>4.8</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>3.66</v>
       </c>
       <c r="E30" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="F30" t="n">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
       <c r="G30" t="n">
-        <v>3.5</v>
+        <v>3.8</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.04</v>
       </c>
       <c r="E31" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="F31" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="G31" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.79</v>
       </c>
       <c r="E32" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="F32" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="G32" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu Oct  8 16:58:15 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,52 +486,52 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.43</v>
+        <v>7.49</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7</v>
+        <v>0.71</v>
       </c>
       <c r="E2" t="n">
-        <v>97.8</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>96.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28.81</v>
+        <v>20.39</v>
       </c>
       <c r="D3" t="n">
-        <v>2.77</v>
+        <v>1.73</v>
       </c>
       <c r="E3" t="n">
-        <v>68.3</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>87.59999999999999</v>
+        <v>43.5</v>
       </c>
       <c r="G3" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="4">
@@ -546,82 +546,82 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>19.97</v>
+        <v>20.05</v>
       </c>
       <c r="D4" t="n">
         <v>0.98</v>
       </c>
       <c r="E4" t="n">
-        <v>67.09999999999999</v>
+        <v>69.8</v>
       </c>
       <c r="F4" t="n">
-        <v>54.7</v>
+        <v>54.6</v>
       </c>
       <c r="G4" t="n">
-        <v>60.9</v>
+        <v>62.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>19.76</v>
+        <v>13.08</v>
       </c>
       <c r="D5" t="n">
-        <v>3.54</v>
+        <v>1.37</v>
       </c>
       <c r="E5" t="n">
-        <v>38.8</v>
+        <v>39.5</v>
       </c>
       <c r="F5" t="n">
-        <v>56.5</v>
+        <v>76.2</v>
       </c>
       <c r="G5" t="n">
-        <v>47.7</v>
+        <v>57.9</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>22.01</v>
+        <v>14.61</v>
       </c>
       <c r="D6" t="n">
-        <v>2.05</v>
+        <v>1.23</v>
       </c>
       <c r="E6" t="n">
-        <v>42.2</v>
+        <v>45.7</v>
       </c>
       <c r="F6" t="n">
-        <v>49.7</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>46</v>
+        <v>56.6</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="7">
@@ -636,112 +636,112 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>16.83</v>
+        <v>16.94</v>
       </c>
       <c r="D7" t="n">
-        <v>1.81</v>
+        <v>1.83</v>
       </c>
       <c r="E7" t="n">
-        <v>18</v>
+        <v>25.3</v>
       </c>
       <c r="F7" t="n">
-        <v>73.90000000000001</v>
+        <v>81.8</v>
       </c>
       <c r="G7" t="n">
-        <v>46</v>
+        <v>53.5</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>9.07</v>
+        <v>19.78</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>3.55</v>
       </c>
       <c r="E8" t="n">
-        <v>25.5</v>
+        <v>43.5</v>
       </c>
       <c r="F8" t="n">
-        <v>63.4</v>
+        <v>62.7</v>
       </c>
       <c r="G8" t="n">
-        <v>44.4</v>
+        <v>53.1</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>12.71</v>
+        <v>28.1</v>
       </c>
       <c r="D9" t="n">
-        <v>1.33</v>
+        <v>2.7</v>
       </c>
       <c r="E9" t="n">
-        <v>23.3</v>
+        <v>40.7</v>
       </c>
       <c r="F9" t="n">
-        <v>53.1</v>
+        <v>62.7</v>
       </c>
       <c r="G9" t="n">
-        <v>38.2</v>
+        <v>51.7</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>26.83</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="D10" t="n">
-        <v>2.4</v>
+        <v>1.01</v>
       </c>
       <c r="E10" t="n">
-        <v>22.4</v>
+        <v>27.8</v>
       </c>
       <c r="F10" t="n">
-        <v>53.1</v>
+        <v>69.8</v>
       </c>
       <c r="G10" t="n">
-        <v>37.7</v>
+        <v>48.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="11">
@@ -756,202 +756,202 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>19.5</v>
+        <v>19.54</v>
       </c>
       <c r="D11" t="n">
         <v>1.63</v>
       </c>
       <c r="E11" t="n">
-        <v>35.4</v>
+        <v>42.6</v>
       </c>
       <c r="F11" t="n">
-        <v>36.3</v>
+        <v>36.4</v>
       </c>
       <c r="G11" t="n">
-        <v>35.9</v>
+        <v>39.5</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>23.53</v>
+        <v>21.83</v>
       </c>
       <c r="D12" t="n">
-        <v>1.97</v>
+        <v>2.03</v>
       </c>
       <c r="E12" t="n">
-        <v>25.8</v>
+        <v>32.4</v>
       </c>
       <c r="F12" t="n">
-        <v>39.1</v>
+        <v>42.3</v>
       </c>
       <c r="G12" t="n">
-        <v>32.5</v>
+        <v>37.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>20.03</v>
+        <v>26.7</v>
       </c>
       <c r="D13" t="n">
-        <v>1.7</v>
+        <v>2.39</v>
       </c>
       <c r="E13" t="n">
-        <v>59.6</v>
+        <v>13.9</v>
       </c>
       <c r="F13" t="n">
-        <v>17.4</v>
+        <v>46.6</v>
       </c>
       <c r="G13" t="n">
-        <v>30.1</v>
+        <v>30.2</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>14.35</v>
+        <v>31.78</v>
       </c>
       <c r="D14" t="n">
-        <v>1.21</v>
+        <v>1.91</v>
       </c>
       <c r="E14" t="n">
-        <v>19.6</v>
+        <v>66</v>
       </c>
       <c r="F14" t="n">
-        <v>38.5</v>
+        <v>7.4</v>
       </c>
       <c r="G14" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>31.87</v>
+        <v>14.88</v>
       </c>
       <c r="D15" t="n">
-        <v>1.91</v>
+        <v>2.28</v>
       </c>
       <c r="E15" t="n">
-        <v>68.3</v>
+        <v>8</v>
       </c>
       <c r="F15" t="n">
-        <v>7.1</v>
+        <v>35.5</v>
       </c>
       <c r="G15" t="n">
-        <v>25.5</v>
+        <v>21.8</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>14.87</v>
+        <v>30.98</v>
       </c>
       <c r="D16" t="n">
-        <v>2.28</v>
+        <v>1.93</v>
       </c>
       <c r="E16" t="n">
-        <v>5.6</v>
+        <v>3.1</v>
       </c>
       <c r="F16" t="n">
-        <v>35.4</v>
+        <v>29.6</v>
       </c>
       <c r="G16" t="n">
-        <v>20.5</v>
+        <v>21.7</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>31.41</v>
+        <v>23.01</v>
       </c>
       <c r="D17" t="n">
-        <v>1.95</v>
+        <v>1.93</v>
       </c>
       <c r="E17" t="n">
-        <v>7.5</v>
+        <v>8.6</v>
       </c>
       <c r="F17" t="n">
-        <v>33.5</v>
+        <v>23.5</v>
       </c>
       <c r="G17" t="n">
-        <v>20.5</v>
+        <v>19</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="18">
@@ -966,232 +966,232 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>29.33</v>
+        <v>29.24</v>
       </c>
       <c r="D18" t="n">
         <v>2.3</v>
       </c>
       <c r="E18" t="n">
-        <v>13.7</v>
+        <v>10.5</v>
       </c>
       <c r="F18" t="n">
-        <v>22.4</v>
+        <v>22.5</v>
       </c>
       <c r="G18" t="n">
-        <v>19.8</v>
+        <v>18.9</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>20.92</v>
+        <v>10.49</v>
       </c>
       <c r="D19" t="n">
-        <v>1.78</v>
+        <v>0.62</v>
       </c>
       <c r="E19" t="n">
-        <v>11.2</v>
+        <v>36.1</v>
       </c>
       <c r="F19" t="n">
-        <v>22.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>19</v>
+        <v>16.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>49.74</v>
+        <v>20.81</v>
       </c>
       <c r="D20" t="n">
-        <v>7.38</v>
+        <v>1.77</v>
       </c>
       <c r="E20" t="n">
-        <v>2.5</v>
+        <v>4.9</v>
       </c>
       <c r="F20" t="n">
-        <v>25.5</v>
+        <v>17.6</v>
       </c>
       <c r="G20" t="n">
-        <v>18.6</v>
+        <v>13.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>35.69</v>
+        <v>50.45</v>
       </c>
       <c r="D21" t="n">
-        <v>3.14</v>
+        <v>3.46</v>
       </c>
       <c r="E21" t="n">
-        <v>10.6</v>
+        <v>6.2</v>
       </c>
       <c r="F21" t="n">
-        <v>16.1</v>
+        <v>14.2</v>
       </c>
       <c r="G21" t="n">
-        <v>14.5</v>
+        <v>11.8</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>10.49</v>
+        <v>66.19</v>
       </c>
       <c r="D22" t="n">
-        <v>0.61</v>
+        <v>3.51</v>
       </c>
       <c r="E22" t="n">
-        <v>36</v>
+        <v>2.5</v>
       </c>
       <c r="F22" t="n">
-        <v>3.1</v>
+        <v>13</v>
       </c>
       <c r="G22" t="n">
-        <v>13</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>66.34999999999999</v>
+        <v>34.79</v>
       </c>
       <c r="D23" t="n">
-        <v>3.52</v>
+        <v>3.06</v>
       </c>
       <c r="E23" t="n">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
       <c r="F23" t="n">
-        <v>15.8</v>
+        <v>10.5</v>
       </c>
       <c r="G23" t="n">
-        <v>12.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>50.37</v>
+        <v>47.34</v>
       </c>
       <c r="D24" t="n">
-        <v>3.45</v>
+        <v>7.03</v>
       </c>
       <c r="E24" t="n">
-        <v>3.1</v>
+        <v>0.6</v>
       </c>
       <c r="F24" t="n">
-        <v>11.5</v>
+        <v>12.3</v>
       </c>
       <c r="G24" t="n">
-        <v>9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>22.19</v>
+        <v>18.4</v>
       </c>
       <c r="D25" t="n">
-        <v>1.99</v>
+        <v>1.41</v>
       </c>
       <c r="E25" t="n">
-        <v>14.6</v>
+        <v>6.2</v>
       </c>
       <c r="F25" t="n">
-        <v>5.3</v>
+        <v>9.9</v>
       </c>
       <c r="G25" t="n">
-        <v>8.1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="26">
@@ -1206,22 +1206,22 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>21.6</v>
+        <v>21.67</v>
       </c>
       <c r="D26" t="n">
         <v>2.26</v>
       </c>
       <c r="E26" t="n">
-        <v>3.7</v>
+        <v>6.2</v>
       </c>
       <c r="F26" t="n">
-        <v>9.300000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="G26" t="n">
-        <v>7.6</v>
+        <v>8.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="27">
@@ -1236,172 +1236,172 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>28.13</v>
+        <v>27.62</v>
       </c>
       <c r="D27" t="n">
-        <v>2.7</v>
+        <v>2.66</v>
       </c>
       <c r="E27" t="n">
-        <v>7.5</v>
+        <v>1.9</v>
       </c>
       <c r="F27" t="n">
-        <v>7.5</v>
+        <v>5.6</v>
       </c>
       <c r="G27" t="n">
-        <v>7.5</v>
+        <v>4.4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>7.56</v>
+        <v>21.78</v>
       </c>
       <c r="D28" t="n">
-        <v>1.17</v>
+        <v>1.95</v>
       </c>
       <c r="E28" t="n">
-        <v>3.7</v>
+        <v>3.1</v>
       </c>
       <c r="F28" t="n">
-        <v>5.6</v>
+        <v>1.2</v>
       </c>
       <c r="G28" t="n">
-        <v>5</v>
+        <v>1.8</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>18.35</v>
+        <v>15.93</v>
       </c>
       <c r="D29" t="n">
-        <v>1.4</v>
+        <v>3</v>
       </c>
       <c r="E29" t="n">
-        <v>3.1</v>
+        <v>1.2</v>
       </c>
       <c r="F29" t="n">
-        <v>5.6</v>
+        <v>1.9</v>
       </c>
       <c r="G29" t="n">
-        <v>4.8</v>
+        <v>1.7</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>39.28</v>
+        <v>24.6</v>
       </c>
       <c r="D30" t="n">
-        <v>3.66</v>
+        <v>2.77</v>
       </c>
       <c r="E30" t="n">
-        <v>2.5</v>
+        <v>1.2</v>
       </c>
       <c r="F30" t="n">
-        <v>4.3</v>
+        <v>1.5</v>
       </c>
       <c r="G30" t="n">
-        <v>3.8</v>
+        <v>1.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>16.15</v>
+        <v>7.45</v>
       </c>
       <c r="D31" t="n">
-        <v>3.04</v>
+        <v>1.15</v>
       </c>
       <c r="E31" t="n">
-        <v>3.7</v>
+        <v>0.6</v>
       </c>
       <c r="F31" t="n">
-        <v>3.7</v>
+        <v>0.6</v>
       </c>
       <c r="G31" t="n">
-        <v>3.7</v>
+        <v>0.6</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>24.73</v>
+        <v>38.54</v>
       </c>
       <c r="D32" t="n">
-        <v>2.79</v>
+        <v>3.59</v>
       </c>
       <c r="E32" t="n">
-        <v>3.7</v>
+        <v>0.6</v>
       </c>
       <c r="F32" t="n">
-        <v>3.7</v>
+        <v>0.6</v>
       </c>
       <c r="G32" t="n">
-        <v>3.7</v>
+        <v>0.6</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri Oct  9 16:37:47 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,502 +486,502 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.49</v>
+        <v>7.41</v>
       </c>
       <c r="D2" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>94.2</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.39</v>
+        <v>17.25</v>
       </c>
       <c r="D3" t="n">
-        <v>1.73</v>
+        <v>1.86</v>
       </c>
       <c r="E3" t="n">
-        <v>82.40000000000001</v>
+        <v>34.7</v>
       </c>
       <c r="F3" t="n">
-        <v>43.5</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>63</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>20.05</v>
+        <v>14.71</v>
       </c>
       <c r="D4" t="n">
-        <v>0.98</v>
+        <v>1.24</v>
       </c>
       <c r="E4" t="n">
-        <v>69.8</v>
+        <v>51.5</v>
       </c>
       <c r="F4" t="n">
-        <v>54.6</v>
+        <v>75.5</v>
       </c>
       <c r="G4" t="n">
-        <v>62.2</v>
+        <v>63.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>13.08</v>
+        <v>20.41</v>
       </c>
       <c r="D5" t="n">
-        <v>1.37</v>
+        <v>1.73</v>
       </c>
       <c r="E5" t="n">
-        <v>39.5</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>76.2</v>
+        <v>43.6</v>
       </c>
       <c r="G5" t="n">
-        <v>57.9</v>
+        <v>63.5</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>14.61</v>
+        <v>19.9</v>
       </c>
       <c r="D6" t="n">
-        <v>1.23</v>
+        <v>3.57</v>
       </c>
       <c r="E6" t="n">
-        <v>45.7</v>
+        <v>54.9</v>
       </c>
       <c r="F6" t="n">
-        <v>67.59999999999999</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>56.6</v>
+        <v>62.3</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>16.94</v>
+        <v>20.03</v>
       </c>
       <c r="D7" t="n">
-        <v>1.83</v>
+        <v>0.98</v>
       </c>
       <c r="E7" t="n">
-        <v>25.3</v>
+        <v>69.3</v>
       </c>
       <c r="F7" t="n">
-        <v>81.8</v>
+        <v>54.6</v>
       </c>
       <c r="G7" t="n">
-        <v>53.5</v>
+        <v>62</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19.78</v>
+        <v>19.88</v>
       </c>
       <c r="D8" t="n">
-        <v>3.55</v>
+        <v>1.66</v>
       </c>
       <c r="E8" t="n">
-        <v>43.5</v>
+        <v>63.2</v>
       </c>
       <c r="F8" t="n">
-        <v>62.7</v>
+        <v>56.1</v>
       </c>
       <c r="G8" t="n">
-        <v>53.1</v>
+        <v>59.7</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>28.1</v>
+        <v>24.24</v>
       </c>
       <c r="D9" t="n">
-        <v>2.7</v>
+        <v>2.03</v>
       </c>
       <c r="E9" t="n">
-        <v>40.7</v>
+        <v>53.4</v>
       </c>
       <c r="F9" t="n">
-        <v>62.7</v>
+        <v>65</v>
       </c>
       <c r="G9" t="n">
-        <v>51.7</v>
+        <v>59.2</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9.109999999999999</v>
+        <v>28.25</v>
       </c>
       <c r="D10" t="n">
-        <v>1.01</v>
+        <v>2.72</v>
       </c>
       <c r="E10" t="n">
-        <v>27.8</v>
+        <v>49.1</v>
       </c>
       <c r="F10" t="n">
-        <v>69.8</v>
+        <v>67.8</v>
       </c>
       <c r="G10" t="n">
-        <v>48.8</v>
+        <v>58.4</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>19.54</v>
+        <v>13.01</v>
       </c>
       <c r="D11" t="n">
-        <v>1.63</v>
+        <v>1.37</v>
       </c>
       <c r="E11" t="n">
-        <v>42.6</v>
+        <v>36.5</v>
       </c>
       <c r="F11" t="n">
-        <v>36.4</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>39.5</v>
+        <v>56.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>21.83</v>
+        <v>27.2</v>
       </c>
       <c r="D12" t="n">
-        <v>2.03</v>
+        <v>2.43</v>
       </c>
       <c r="E12" t="n">
-        <v>32.4</v>
+        <v>36.2</v>
       </c>
       <c r="F12" t="n">
-        <v>42.3</v>
+        <v>62.6</v>
       </c>
       <c r="G12" t="n">
-        <v>37.3</v>
+        <v>49.4</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>26.7</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="D13" t="n">
-        <v>2.39</v>
+        <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>13.9</v>
+        <v>23.3</v>
       </c>
       <c r="F13" t="n">
-        <v>46.6</v>
+        <v>62.9</v>
       </c>
       <c r="G13" t="n">
-        <v>30.2</v>
+        <v>43.1</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>31.78</v>
+        <v>21.96</v>
       </c>
       <c r="D14" t="n">
-        <v>1.91</v>
+        <v>2.04</v>
       </c>
       <c r="E14" t="n">
-        <v>66</v>
+        <v>39.9</v>
       </c>
       <c r="F14" t="n">
-        <v>7.4</v>
+        <v>46.3</v>
       </c>
       <c r="G14" t="n">
-        <v>25</v>
+        <v>43.1</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>14.88</v>
+        <v>32.76</v>
       </c>
       <c r="D15" t="n">
-        <v>2.28</v>
+        <v>1.97</v>
       </c>
       <c r="E15" t="n">
-        <v>8</v>
+        <v>84.7</v>
       </c>
       <c r="F15" t="n">
-        <v>35.5</v>
+        <v>22.7</v>
       </c>
       <c r="G15" t="n">
-        <v>21.8</v>
+        <v>41.3</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>30.98</v>
+        <v>14.97</v>
       </c>
       <c r="D16" t="n">
-        <v>1.93</v>
+        <v>2.3</v>
       </c>
       <c r="E16" t="n">
-        <v>3.1</v>
+        <v>12.3</v>
       </c>
       <c r="F16" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="G16" t="n">
         <v>29.6</v>
       </c>
-      <c r="G16" t="n">
-        <v>21.7</v>
-      </c>
       <c r="H16" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>23.01</v>
+        <v>29.59</v>
       </c>
       <c r="D17" t="n">
-        <v>1.93</v>
+        <v>2.32</v>
       </c>
       <c r="E17" t="n">
-        <v>8.6</v>
+        <v>24.5</v>
       </c>
       <c r="F17" t="n">
-        <v>23.5</v>
+        <v>33.4</v>
       </c>
       <c r="G17" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>29.24</v>
+        <v>21.24</v>
       </c>
       <c r="D18" t="n">
-        <v>2.3</v>
+        <v>1.8</v>
       </c>
       <c r="E18" t="n">
-        <v>10.5</v>
+        <v>22.7</v>
       </c>
       <c r="F18" t="n">
-        <v>22.5</v>
+        <v>31.3</v>
       </c>
       <c r="G18" t="n">
-        <v>18.9</v>
+        <v>27</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="19">
@@ -996,142 +996,142 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>10.49</v>
+        <v>10.5</v>
       </c>
       <c r="D19" t="n">
         <v>0.62</v>
       </c>
       <c r="E19" t="n">
-        <v>36.1</v>
+        <v>39</v>
       </c>
       <c r="F19" t="n">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="G19" t="n">
-        <v>16.7</v>
+        <v>17.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>20.81</v>
+        <v>30.46</v>
       </c>
       <c r="D20" t="n">
-        <v>1.77</v>
+        <v>1.9</v>
       </c>
       <c r="E20" t="n">
-        <v>4.9</v>
+        <v>2.5</v>
       </c>
       <c r="F20" t="n">
-        <v>17.6</v>
+        <v>21.2</v>
       </c>
       <c r="G20" t="n">
-        <v>13.8</v>
+        <v>15.6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>50.45</v>
+        <v>21.8</v>
       </c>
       <c r="D21" t="n">
-        <v>3.46</v>
+        <v>2.28</v>
       </c>
       <c r="E21" t="n">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="F21" t="n">
-        <v>14.2</v>
+        <v>16.3</v>
       </c>
       <c r="G21" t="n">
-        <v>11.8</v>
+        <v>13.4</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>66.19</v>
+        <v>18.5</v>
       </c>
       <c r="D22" t="n">
-        <v>3.51</v>
+        <v>1.42</v>
       </c>
       <c r="E22" t="n">
-        <v>2.5</v>
+        <v>7.4</v>
       </c>
       <c r="F22" t="n">
-        <v>13</v>
+        <v>14.7</v>
       </c>
       <c r="G22" t="n">
-        <v>9.800000000000001</v>
+        <v>12.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>34.79</v>
+        <v>66</v>
       </c>
       <c r="D23" t="n">
-        <v>3.06</v>
+        <v>3.5</v>
       </c>
       <c r="E23" t="n">
-        <v>6.2</v>
+        <v>1.8</v>
       </c>
       <c r="F23" t="n">
-        <v>10.5</v>
+        <v>12.6</v>
       </c>
       <c r="G23" t="n">
-        <v>9.199999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="24">
@@ -1146,262 +1146,262 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>47.34</v>
+        <v>46.89</v>
       </c>
       <c r="D24" t="n">
-        <v>7.03</v>
+        <v>6.96</v>
       </c>
       <c r="E24" t="n">
         <v>0.6</v>
       </c>
       <c r="F24" t="n">
-        <v>12.3</v>
+        <v>11.7</v>
       </c>
       <c r="G24" t="n">
-        <v>8.800000000000001</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>18.4</v>
+        <v>39.37</v>
       </c>
       <c r="D25" t="n">
-        <v>1.41</v>
+        <v>3.67</v>
       </c>
       <c r="E25" t="n">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
       <c r="F25" t="n">
-        <v>9.9</v>
+        <v>8.9</v>
       </c>
       <c r="G25" t="n">
-        <v>8.800000000000001</v>
+        <v>8</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>21.67</v>
+        <v>34.38</v>
       </c>
       <c r="D26" t="n">
-        <v>2.26</v>
+        <v>3.02</v>
       </c>
       <c r="E26" t="n">
-        <v>6.2</v>
+        <v>5.5</v>
       </c>
       <c r="F26" t="n">
-        <v>9.6</v>
+        <v>8</v>
       </c>
       <c r="G26" t="n">
-        <v>8.5</v>
+        <v>7.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>27.62</v>
+        <v>16.2</v>
       </c>
       <c r="D27" t="n">
-        <v>2.66</v>
+        <v>3.05</v>
       </c>
       <c r="E27" t="n">
-        <v>1.9</v>
+        <v>6.7</v>
       </c>
       <c r="F27" t="n">
-        <v>5.6</v>
+        <v>7.1</v>
       </c>
       <c r="G27" t="n">
-        <v>4.4</v>
+        <v>7</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>21.78</v>
+        <v>7.54</v>
       </c>
       <c r="D28" t="n">
-        <v>1.95</v>
+        <v>1.17</v>
       </c>
       <c r="E28" t="n">
-        <v>3.1</v>
+        <v>2.5</v>
       </c>
       <c r="F28" t="n">
-        <v>1.2</v>
+        <v>6.4</v>
       </c>
       <c r="G28" t="n">
-        <v>1.8</v>
+        <v>5.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>15.93</v>
+        <v>22.01</v>
       </c>
       <c r="D29" t="n">
-        <v>3</v>
+        <v>1.98</v>
       </c>
       <c r="E29" t="n">
-        <v>1.2</v>
+        <v>6.1</v>
       </c>
       <c r="F29" t="n">
-        <v>1.9</v>
+        <v>2.8</v>
       </c>
       <c r="G29" t="n">
-        <v>1.7</v>
+        <v>3.8</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>24.6</v>
+        <v>27.49</v>
       </c>
       <c r="D30" t="n">
-        <v>2.77</v>
+        <v>2.64</v>
       </c>
       <c r="E30" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="F30" t="n">
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="G30" t="n">
-        <v>1.5</v>
+        <v>3.3</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>7.45</v>
+        <v>24.71</v>
       </c>
       <c r="D31" t="n">
-        <v>1.15</v>
+        <v>2.78</v>
       </c>
       <c r="E31" t="n">
-        <v>0.6</v>
+        <v>2.5</v>
       </c>
       <c r="F31" t="n">
-        <v>0.6</v>
+        <v>2.5</v>
       </c>
       <c r="G31" t="n">
-        <v>0.6</v>
+        <v>2.5</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>38.54</v>
+        <v>49.36</v>
       </c>
       <c r="D32" t="n">
-        <v>3.59</v>
+        <v>3.38</v>
       </c>
       <c r="E32" t="n">
         <v>0.6</v>
       </c>
       <c r="F32" t="n">
-        <v>0.6</v>
+        <v>3.4</v>
       </c>
       <c r="G32" t="n">
-        <v>0.6</v>
+        <v>2.5</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat Oct 10 15:35:04 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.7</v>
       </c>
       <c r="E2" t="n">
-        <v>94.2</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>95.09999999999999</v>
+        <v>94.8</v>
       </c>
       <c r="G2" t="n">
-        <v>94.59999999999999</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>1.86</v>
       </c>
       <c r="E3" t="n">
-        <v>34.7</v>
+        <v>34.8</v>
       </c>
       <c r="F3" t="n">
-        <v>93.59999999999999</v>
+        <v>93.3</v>
       </c>
       <c r="G3" t="n">
-        <v>64.09999999999999</v>
+        <v>64</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="4">
@@ -555,13 +555,13 @@
         <v>51.5</v>
       </c>
       <c r="F4" t="n">
-        <v>75.5</v>
+        <v>75.3</v>
       </c>
       <c r="G4" t="n">
-        <v>63.5</v>
+        <v>63.4</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>1.73</v>
       </c>
       <c r="E5" t="n">
-        <v>83.40000000000001</v>
+        <v>83.2</v>
       </c>
       <c r="F5" t="n">
         <v>43.6</v>
       </c>
       <c r="G5" t="n">
-        <v>63.5</v>
+        <v>63.4</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="6">
@@ -615,13 +615,13 @@
         <v>54.9</v>
       </c>
       <c r="F6" t="n">
-        <v>69.59999999999999</v>
+        <v>69.5</v>
       </c>
       <c r="G6" t="n">
-        <v>62.3</v>
+        <v>62.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>0.98</v>
       </c>
       <c r="E7" t="n">
-        <v>69.3</v>
+        <v>69.2</v>
       </c>
       <c r="F7" t="n">
         <v>54.6</v>
       </c>
       <c r="G7" t="n">
-        <v>62</v>
+        <v>61.9</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>1.66</v>
       </c>
       <c r="E8" t="n">
-        <v>63.2</v>
+        <v>63.1</v>
       </c>
       <c r="F8" t="n">
         <v>56.1</v>
       </c>
       <c r="G8" t="n">
-        <v>59.7</v>
+        <v>59.6</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="9">
@@ -705,13 +705,13 @@
         <v>53.4</v>
       </c>
       <c r="F9" t="n">
-        <v>65</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>59.2</v>
+        <v>59.1</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="10">
@@ -735,13 +735,13 @@
         <v>49.1</v>
       </c>
       <c r="F10" t="n">
-        <v>67.8</v>
+        <v>67.7</v>
       </c>
       <c r="G10" t="n">
         <v>58.4</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.37</v>
       </c>
       <c r="E11" t="n">
-        <v>36.5</v>
+        <v>36.6</v>
       </c>
       <c r="F11" t="n">
-        <v>76.09999999999999</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>56.3</v>
+        <v>56.2</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>2.43</v>
       </c>
       <c r="E12" t="n">
-        <v>36.2</v>
+        <v>36.3</v>
       </c>
       <c r="F12" t="n">
-        <v>62.6</v>
+        <v>62.5</v>
       </c>
       <c r="G12" t="n">
         <v>49.4</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>23.3</v>
+        <v>23.5</v>
       </c>
       <c r="F13" t="n">
-        <v>62.9</v>
+        <v>62.8</v>
       </c>
       <c r="G13" t="n">
         <v>43.1</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="14">
@@ -861,7 +861,7 @@
         <v>43.1</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.97</v>
       </c>
       <c r="E15" t="n">
-        <v>84.7</v>
+        <v>84.5</v>
       </c>
       <c r="F15" t="n">
-        <v>22.7</v>
+        <v>22.9</v>
       </c>
       <c r="G15" t="n">
         <v>41.3</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>2.3</v>
       </c>
       <c r="E16" t="n">
-        <v>12.3</v>
+        <v>12.5</v>
       </c>
       <c r="F16" t="n">
-        <v>46.9</v>
+        <v>47</v>
       </c>
       <c r="G16" t="n">
-        <v>29.6</v>
+        <v>29.7</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>2.32</v>
       </c>
       <c r="E17" t="n">
-        <v>24.5</v>
+        <v>24.7</v>
       </c>
       <c r="F17" t="n">
-        <v>33.4</v>
+        <v>33.5</v>
       </c>
       <c r="G17" t="n">
-        <v>29</v>
+        <v>29.1</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>1.8</v>
       </c>
       <c r="E18" t="n">
-        <v>22.7</v>
+        <v>22.9</v>
       </c>
       <c r="F18" t="n">
-        <v>31.3</v>
+        <v>31.4</v>
       </c>
       <c r="G18" t="n">
-        <v>27</v>
+        <v>27.1</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="19">
@@ -1005,13 +1005,13 @@
         <v>39</v>
       </c>
       <c r="F19" t="n">
-        <v>8.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>17.7</v>
+        <v>17.9</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>1.9</v>
       </c>
       <c r="E20" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="F20" t="n">
-        <v>21.2</v>
+        <v>21.3</v>
       </c>
       <c r="G20" t="n">
-        <v>15.6</v>
+        <v>15.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>2.28</v>
       </c>
       <c r="E21" t="n">
-        <v>6.7</v>
+        <v>7</v>
       </c>
       <c r="F21" t="n">
-        <v>16.3</v>
+        <v>16.5</v>
       </c>
       <c r="G21" t="n">
-        <v>13.4</v>
+        <v>13.6</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.42</v>
       </c>
       <c r="E22" t="n">
-        <v>7.4</v>
+        <v>7.6</v>
       </c>
       <c r="F22" t="n">
-        <v>14.7</v>
+        <v>14.9</v>
       </c>
       <c r="G22" t="n">
-        <v>12.5</v>
+        <v>12.7</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>3.5</v>
       </c>
       <c r="E23" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="F23" t="n">
-        <v>12.6</v>
+        <v>12.8</v>
       </c>
       <c r="G23" t="n">
-        <v>9.4</v>
+        <v>9.6</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>6.96</v>
       </c>
       <c r="E24" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="F24" t="n">
-        <v>11.7</v>
+        <v>11.9</v>
       </c>
       <c r="G24" t="n">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>3.67</v>
       </c>
       <c r="E25" t="n">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
       <c r="F25" t="n">
-        <v>8.9</v>
+        <v>9.1</v>
       </c>
       <c r="G25" t="n">
-        <v>8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>3.02</v>
       </c>
       <c r="E26" t="n">
-        <v>5.5</v>
+        <v>5.8</v>
       </c>
       <c r="F26" t="n">
-        <v>8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G26" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>3.05</v>
       </c>
       <c r="E27" t="n">
-        <v>6.7</v>
+        <v>7</v>
       </c>
       <c r="F27" t="n">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
       <c r="G27" t="n">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>1.17</v>
       </c>
       <c r="E28" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="F28" t="n">
-        <v>6.4</v>
+        <v>6.7</v>
       </c>
       <c r="G28" t="n">
-        <v>5.2</v>
+        <v>5.5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.98</v>
       </c>
       <c r="E29" t="n">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
       <c r="F29" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="G29" t="n">
-        <v>3.8</v>
+        <v>4.1</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="30">
@@ -1332,76 +1332,76 @@
         <v>2.64</v>
       </c>
       <c r="E30" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="F30" t="n">
-        <v>4</v>
+        <v>4.3</v>
       </c>
       <c r="G30" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>24.71</v>
+        <v>49.36</v>
       </c>
       <c r="D31" t="n">
-        <v>2.78</v>
+        <v>3.38</v>
       </c>
       <c r="E31" t="n">
-        <v>2.5</v>
+        <v>0.9</v>
       </c>
       <c r="F31" t="n">
-        <v>2.5</v>
+        <v>3.7</v>
       </c>
       <c r="G31" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>49.36</v>
+        <v>24.71</v>
       </c>
       <c r="D32" t="n">
-        <v>3.38</v>
+        <v>2.78</v>
       </c>
       <c r="E32" t="n">
-        <v>0.6</v>
+        <v>2.7</v>
       </c>
       <c r="F32" t="n">
-        <v>3.4</v>
+        <v>2.7</v>
       </c>
       <c r="G32" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun Oct 11 15:58:52 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.7</v>
       </c>
       <c r="E2" t="n">
-        <v>93.90000000000001</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>94.8</v>
+        <v>94.5</v>
       </c>
       <c r="G2" t="n">
-        <v>94.40000000000001</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="3">
@@ -525,13 +525,13 @@
         <v>34.8</v>
       </c>
       <c r="F3" t="n">
-        <v>93.3</v>
+        <v>93</v>
       </c>
       <c r="G3" t="n">
-        <v>64</v>
+        <v>63.9</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="4">
@@ -555,13 +555,13 @@
         <v>51.5</v>
       </c>
       <c r="F4" t="n">
-        <v>75.3</v>
+        <v>75.2</v>
       </c>
       <c r="G4" t="n">
-        <v>63.4</v>
+        <v>63.3</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="5">
@@ -582,16 +582,16 @@
         <v>1.73</v>
       </c>
       <c r="E5" t="n">
-        <v>83.2</v>
+        <v>83</v>
       </c>
       <c r="F5" t="n">
         <v>43.6</v>
       </c>
       <c r="G5" t="n">
-        <v>63.4</v>
+        <v>63.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="6">
@@ -612,16 +612,16 @@
         <v>3.57</v>
       </c>
       <c r="E6" t="n">
-        <v>54.9</v>
+        <v>54.8</v>
       </c>
       <c r="F6" t="n">
-        <v>69.5</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>62.2</v>
+        <v>62.1</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>0.98</v>
       </c>
       <c r="E7" t="n">
-        <v>69.2</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="F7" t="n">
-        <v>54.6</v>
+        <v>54.5</v>
       </c>
       <c r="G7" t="n">
-        <v>61.9</v>
+        <v>61.8</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>1.66</v>
       </c>
       <c r="E8" t="n">
-        <v>63.1</v>
+        <v>63</v>
       </c>
       <c r="F8" t="n">
         <v>56.1</v>
       </c>
       <c r="G8" t="n">
-        <v>59.6</v>
+        <v>59.5</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>2.03</v>
       </c>
       <c r="E9" t="n">
-        <v>53.4</v>
+        <v>53.3</v>
       </c>
       <c r="F9" t="n">
-        <v>64.90000000000001</v>
+        <v>64.8</v>
       </c>
       <c r="G9" t="n">
         <v>59.1</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="10">
@@ -735,13 +735,13 @@
         <v>49.1</v>
       </c>
       <c r="F10" t="n">
-        <v>67.7</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="G10" t="n">
-        <v>58.4</v>
+        <v>58.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.37</v>
       </c>
       <c r="E11" t="n">
-        <v>36.6</v>
+        <v>36.7</v>
       </c>
       <c r="F11" t="n">
-        <v>75.90000000000001</v>
+        <v>75.8</v>
       </c>
       <c r="G11" t="n">
         <v>56.2</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>2.43</v>
       </c>
       <c r="E12" t="n">
-        <v>36.3</v>
+        <v>36.4</v>
       </c>
       <c r="F12" t="n">
-        <v>62.5</v>
+        <v>62.4</v>
       </c>
       <c r="G12" t="n">
         <v>49.4</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>23.5</v>
+        <v>23.6</v>
       </c>
       <c r="F13" t="n">
-        <v>62.8</v>
+        <v>62.7</v>
       </c>
       <c r="G13" t="n">
-        <v>43.1</v>
+        <v>43.2</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2.04</v>
       </c>
       <c r="E14" t="n">
-        <v>39.9</v>
+        <v>40</v>
       </c>
       <c r="F14" t="n">
-        <v>46.3</v>
+        <v>46.4</v>
       </c>
       <c r="G14" t="n">
-        <v>43.1</v>
+        <v>43.2</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>1.97</v>
       </c>
       <c r="E15" t="n">
-        <v>84.5</v>
+        <v>84.2</v>
       </c>
       <c r="F15" t="n">
-        <v>22.9</v>
+        <v>23</v>
       </c>
       <c r="G15" t="n">
-        <v>41.3</v>
+        <v>41.4</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>2.3</v>
       </c>
       <c r="E16" t="n">
-        <v>12.5</v>
+        <v>12.7</v>
       </c>
       <c r="F16" t="n">
         <v>47</v>
       </c>
       <c r="G16" t="n">
-        <v>29.7</v>
+        <v>29.8</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>2.32</v>
       </c>
       <c r="E17" t="n">
-        <v>24.7</v>
+        <v>24.8</v>
       </c>
       <c r="F17" t="n">
-        <v>33.5</v>
+        <v>33.6</v>
       </c>
       <c r="G17" t="n">
-        <v>29.1</v>
+        <v>29.2</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>1.8</v>
       </c>
       <c r="E18" t="n">
-        <v>22.9</v>
+        <v>23</v>
       </c>
       <c r="F18" t="n">
-        <v>31.4</v>
+        <v>31.5</v>
       </c>
       <c r="G18" t="n">
-        <v>27.1</v>
+        <v>27.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>0.62</v>
       </c>
       <c r="E19" t="n">
-        <v>39</v>
+        <v>39.1</v>
       </c>
       <c r="F19" t="n">
-        <v>8.800000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="G19" t="n">
-        <v>17.9</v>
+        <v>18.1</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>1.9</v>
       </c>
       <c r="E20" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
-        <v>21.3</v>
+        <v>21.5</v>
       </c>
       <c r="G20" t="n">
-        <v>15.8</v>
+        <v>16</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>2.28</v>
       </c>
       <c r="E21" t="n">
-        <v>7</v>
+        <v>7.3</v>
       </c>
       <c r="F21" t="n">
-        <v>16.5</v>
+        <v>16.7</v>
       </c>
       <c r="G21" t="n">
-        <v>13.6</v>
+        <v>13.8</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>1.42</v>
       </c>
       <c r="E22" t="n">
-        <v>7.6</v>
+        <v>7.9</v>
       </c>
       <c r="F22" t="n">
-        <v>14.9</v>
+        <v>15.2</v>
       </c>
       <c r="G22" t="n">
-        <v>12.7</v>
+        <v>13</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>3.5</v>
       </c>
       <c r="E23" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="F23" t="n">
-        <v>12.8</v>
+        <v>13</v>
       </c>
       <c r="G23" t="n">
-        <v>9.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>6.96</v>
       </c>
       <c r="E24" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="F24" t="n">
-        <v>11.9</v>
+        <v>12.1</v>
       </c>
       <c r="G24" t="n">
-        <v>8.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>3.67</v>
       </c>
       <c r="E25" t="n">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
       <c r="F25" t="n">
-        <v>9.1</v>
+        <v>9.4</v>
       </c>
       <c r="G25" t="n">
-        <v>8.199999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>3.02</v>
       </c>
       <c r="E26" t="n">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
       <c r="F26" t="n">
-        <v>8.199999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="G26" t="n">
-        <v>7.5</v>
+        <v>7.8</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>3.05</v>
       </c>
       <c r="E27" t="n">
-        <v>7</v>
+        <v>7.3</v>
       </c>
       <c r="F27" t="n">
-        <v>7.3</v>
+        <v>7.6</v>
       </c>
       <c r="G27" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>1.17</v>
       </c>
       <c r="E28" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="F28" t="n">
-        <v>6.7</v>
+        <v>7</v>
       </c>
       <c r="G28" t="n">
-        <v>5.5</v>
+        <v>5.8</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.98</v>
       </c>
       <c r="E29" t="n">
-        <v>6.4</v>
+        <v>6.7</v>
       </c>
       <c r="F29" t="n">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="G29" t="n">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>2.64</v>
       </c>
       <c r="E30" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="F30" t="n">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="G30" t="n">
-        <v>3.6</v>
+        <v>3.9</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>3.38</v>
       </c>
       <c r="E31" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="F31" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="G31" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>2.78</v>
       </c>
       <c r="E32" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="F32" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="G32" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon Oct 12 19:21:01 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.41</v>
+        <v>7.61</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="E2" t="n">
-        <v>93.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>94.5</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>94.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="3">
@@ -516,262 +516,262 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>17.25</v>
+        <v>17.3</v>
       </c>
       <c r="D3" t="n">
-        <v>1.86</v>
+        <v>1.87</v>
       </c>
       <c r="E3" t="n">
-        <v>34.8</v>
+        <v>39.2</v>
       </c>
       <c r="F3" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="G3" t="n">
-        <v>63.9</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>14.71</v>
+        <v>24.6</v>
       </c>
       <c r="D4" t="n">
-        <v>1.24</v>
+        <v>2.06</v>
       </c>
       <c r="E4" t="n">
-        <v>51.5</v>
+        <v>63.9</v>
       </c>
       <c r="F4" t="n">
-        <v>75.2</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>63.3</v>
+        <v>67.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>20.41</v>
+        <v>20.06</v>
       </c>
       <c r="D5" t="n">
-        <v>1.73</v>
+        <v>3.6</v>
       </c>
       <c r="E5" t="n">
-        <v>83</v>
+        <v>60.2</v>
       </c>
       <c r="F5" t="n">
-        <v>43.6</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>63.3</v>
+        <v>67.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>19.9</v>
+        <v>20.39</v>
       </c>
       <c r="D6" t="n">
-        <v>3.57</v>
+        <v>1.73</v>
       </c>
       <c r="E6" t="n">
-        <v>54.8</v>
+        <v>80.7</v>
       </c>
       <c r="F6" t="n">
-        <v>69.40000000000001</v>
+        <v>43.7</v>
       </c>
       <c r="G6" t="n">
-        <v>62.1</v>
+        <v>62.2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>20.03</v>
+        <v>14.63</v>
       </c>
       <c r="D7" t="n">
-        <v>0.98</v>
+        <v>1.24</v>
       </c>
       <c r="E7" t="n">
-        <v>69.09999999999999</v>
+        <v>45.2</v>
       </c>
       <c r="F7" t="n">
-        <v>54.5</v>
+        <v>75</v>
       </c>
       <c r="G7" t="n">
-        <v>61.8</v>
+        <v>60.1</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19.88</v>
+        <v>13.09</v>
       </c>
       <c r="D8" t="n">
-        <v>1.66</v>
+        <v>1.37</v>
       </c>
       <c r="E8" t="n">
-        <v>63</v>
+        <v>41</v>
       </c>
       <c r="F8" t="n">
-        <v>56.1</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>59.5</v>
+        <v>58.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>24.24</v>
+        <v>19.97</v>
       </c>
       <c r="D9" t="n">
-        <v>2.03</v>
+        <v>0.97</v>
       </c>
       <c r="E9" t="n">
-        <v>53.3</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>64.8</v>
+        <v>45.2</v>
       </c>
       <c r="G9" t="n">
-        <v>59.1</v>
+        <v>55.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>28.25</v>
+        <v>19.63</v>
       </c>
       <c r="D10" t="n">
-        <v>2.72</v>
+        <v>1.64</v>
       </c>
       <c r="E10" t="n">
-        <v>49.1</v>
+        <v>49.4</v>
       </c>
       <c r="F10" t="n">
-        <v>67.59999999999999</v>
+        <v>45.2</v>
       </c>
       <c r="G10" t="n">
-        <v>58.3</v>
+        <v>47.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>13.01</v>
+        <v>27.93</v>
       </c>
       <c r="D11" t="n">
-        <v>1.37</v>
+        <v>2.68</v>
       </c>
       <c r="E11" t="n">
-        <v>36.7</v>
+        <v>31.9</v>
       </c>
       <c r="F11" t="n">
-        <v>75.8</v>
+        <v>53.9</v>
       </c>
       <c r="G11" t="n">
-        <v>56.2</v>
+        <v>42.9</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="12">
@@ -786,52 +786,52 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>27.2</v>
+        <v>26.93</v>
       </c>
       <c r="D12" t="n">
-        <v>2.43</v>
+        <v>2.41</v>
       </c>
       <c r="E12" t="n">
-        <v>36.4</v>
+        <v>25.3</v>
       </c>
       <c r="F12" t="n">
-        <v>62.4</v>
+        <v>56.9</v>
       </c>
       <c r="G12" t="n">
-        <v>49.4</v>
+        <v>41.1</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>8.949999999999999</v>
+        <v>32.59</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>1.96</v>
       </c>
       <c r="E13" t="n">
-        <v>23.6</v>
+        <v>82.8</v>
       </c>
       <c r="F13" t="n">
-        <v>62.7</v>
+        <v>18.7</v>
       </c>
       <c r="G13" t="n">
-        <v>43.2</v>
+        <v>37.9</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="14">
@@ -846,52 +846,52 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>21.96</v>
+        <v>21.85</v>
       </c>
       <c r="D14" t="n">
-        <v>2.04</v>
+        <v>2.03</v>
       </c>
       <c r="E14" t="n">
-        <v>40</v>
+        <v>33.4</v>
       </c>
       <c r="F14" t="n">
-        <v>46.4</v>
+        <v>41.6</v>
       </c>
       <c r="G14" t="n">
-        <v>43.2</v>
+        <v>37.5</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>32.76</v>
+        <v>8.84</v>
       </c>
       <c r="D15" t="n">
-        <v>1.97</v>
+        <v>0.98</v>
       </c>
       <c r="E15" t="n">
-        <v>84.2</v>
+        <v>22.9</v>
       </c>
       <c r="F15" t="n">
-        <v>23</v>
+        <v>49.7</v>
       </c>
       <c r="G15" t="n">
-        <v>41.4</v>
+        <v>36.3</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="16">
@@ -906,442 +906,442 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>14.97</v>
+        <v>15.02</v>
       </c>
       <c r="D16" t="n">
         <v>2.3</v>
       </c>
       <c r="E16" t="n">
-        <v>12.7</v>
+        <v>17.8</v>
       </c>
       <c r="F16" t="n">
         <v>47</v>
       </c>
       <c r="G16" t="n">
-        <v>29.8</v>
+        <v>32.4</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>29.59</v>
+        <v>20.97</v>
       </c>
       <c r="D17" t="n">
-        <v>2.32</v>
+        <v>1.78</v>
       </c>
       <c r="E17" t="n">
-        <v>24.8</v>
+        <v>15.1</v>
       </c>
       <c r="F17" t="n">
-        <v>33.6</v>
+        <v>22.6</v>
       </c>
       <c r="G17" t="n">
-        <v>29.2</v>
+        <v>20.3</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>21.24</v>
+        <v>10.55</v>
       </c>
       <c r="D18" t="n">
-        <v>1.8</v>
+        <v>0.62</v>
       </c>
       <c r="E18" t="n">
-        <v>23</v>
+        <v>43.4</v>
       </c>
       <c r="F18" t="n">
-        <v>31.5</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>27.3</v>
+        <v>19.5</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>10.5</v>
+        <v>29.28</v>
       </c>
       <c r="D19" t="n">
-        <v>0.62</v>
+        <v>2.29</v>
       </c>
       <c r="E19" t="n">
-        <v>39.1</v>
+        <v>10.8</v>
       </c>
       <c r="F19" t="n">
-        <v>9.1</v>
+        <v>16</v>
       </c>
       <c r="G19" t="n">
-        <v>18.1</v>
+        <v>14.4</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>30.46</v>
+        <v>7.58</v>
       </c>
       <c r="D20" t="n">
-        <v>1.9</v>
+        <v>1.18</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>8.4</v>
       </c>
       <c r="F20" t="n">
-        <v>21.5</v>
+        <v>15.1</v>
       </c>
       <c r="G20" t="n">
-        <v>16</v>
+        <v>13.1</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>21.8</v>
+        <v>29.87</v>
       </c>
       <c r="D21" t="n">
-        <v>2.28</v>
+        <v>1.86</v>
       </c>
       <c r="E21" t="n">
-        <v>7.3</v>
+        <v>1.2</v>
       </c>
       <c r="F21" t="n">
-        <v>16.7</v>
+        <v>15.4</v>
       </c>
       <c r="G21" t="n">
-        <v>13.8</v>
+        <v>11.1</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>18.5</v>
+        <v>64.28</v>
       </c>
       <c r="D22" t="n">
-        <v>1.42</v>
+        <v>3.41</v>
       </c>
       <c r="E22" t="n">
-        <v>7.9</v>
+        <v>1.2</v>
       </c>
       <c r="F22" t="n">
-        <v>15.2</v>
+        <v>10.2</v>
       </c>
       <c r="G22" t="n">
-        <v>13</v>
+        <v>7.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>66</v>
+        <v>45.17</v>
       </c>
       <c r="D23" t="n">
-        <v>3.5</v>
+        <v>6.71</v>
       </c>
       <c r="E23" t="n">
-        <v>2.4</v>
+        <v>0.6</v>
       </c>
       <c r="F23" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G23" t="n">
-        <v>9.800000000000001</v>
+        <v>6.5</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>46.89</v>
+        <v>33.73</v>
       </c>
       <c r="D24" t="n">
-        <v>6.96</v>
+        <v>2.97</v>
       </c>
       <c r="E24" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="F24" t="n">
-        <v>12.1</v>
+        <v>5.7</v>
       </c>
       <c r="G24" t="n">
-        <v>8.800000000000001</v>
+        <v>4.5</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>39.37</v>
+        <v>21.92</v>
       </c>
       <c r="D25" t="n">
-        <v>3.67</v>
+        <v>1.97</v>
       </c>
       <c r="E25" t="n">
-        <v>6.4</v>
+        <v>4.2</v>
       </c>
       <c r="F25" t="n">
-        <v>9.4</v>
+        <v>1.8</v>
       </c>
       <c r="G25" t="n">
-        <v>8.5</v>
+        <v>2.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>34.38</v>
+        <v>39.06</v>
       </c>
       <c r="D26" t="n">
-        <v>3.02</v>
+        <v>3.64</v>
       </c>
       <c r="E26" t="n">
-        <v>6.1</v>
+        <v>1.2</v>
       </c>
       <c r="F26" t="n">
-        <v>8.5</v>
+        <v>3</v>
       </c>
       <c r="G26" t="n">
-        <v>7.8</v>
+        <v>2.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>16.2</v>
+        <v>21.21</v>
       </c>
       <c r="D27" t="n">
-        <v>3.05</v>
+        <v>2.22</v>
       </c>
       <c r="E27" t="n">
-        <v>7.3</v>
+        <v>0.6</v>
       </c>
       <c r="F27" t="n">
-        <v>7.6</v>
+        <v>3</v>
       </c>
       <c r="G27" t="n">
-        <v>7.5</v>
+        <v>2.3</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>7.54</v>
+        <v>18.22</v>
       </c>
       <c r="D28" t="n">
-        <v>1.17</v>
+        <v>1.39</v>
       </c>
       <c r="E28" t="n">
-        <v>3</v>
+        <v>0.6</v>
       </c>
       <c r="F28" t="n">
-        <v>7</v>
+        <v>2.4</v>
       </c>
       <c r="G28" t="n">
-        <v>5.8</v>
+        <v>1.9</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>22.01</v>
+        <v>26.86</v>
       </c>
       <c r="D29" t="n">
-        <v>1.98</v>
+        <v>2.58</v>
       </c>
       <c r="E29" t="n">
-        <v>6.7</v>
+        <v>1.2</v>
       </c>
       <c r="F29" t="n">
-        <v>3.3</v>
+        <v>1.8</v>
       </c>
       <c r="G29" t="n">
-        <v>4.3</v>
+        <v>1.6</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>27.49</v>
+        <v>24.59</v>
       </c>
       <c r="D30" t="n">
-        <v>2.64</v>
+        <v>2.77</v>
       </c>
       <c r="E30" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="F30" t="n">
-        <v>4.5</v>
+        <v>1.8</v>
       </c>
       <c r="G30" t="n">
-        <v>3.9</v>
+        <v>1.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="31">
@@ -1356,52 +1356,52 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>49.36</v>
+        <v>48.29</v>
       </c>
       <c r="D31" t="n">
-        <v>3.38</v>
+        <v>3.31</v>
       </c>
       <c r="E31" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G31" t="n">
         <v>1.2</v>
       </c>
-      <c r="F31" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="G31" t="n">
-        <v>3.1</v>
-      </c>
       <c r="H31" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>24.71</v>
+        <v>15.7</v>
       </c>
       <c r="D32" t="n">
-        <v>2.78</v>
+        <v>2.95</v>
       </c>
       <c r="E32" t="n">
-        <v>3</v>
+        <v>0.6</v>
       </c>
       <c r="F32" t="n">
-        <v>3</v>
+        <v>0.9</v>
       </c>
       <c r="G32" t="n">
-        <v>3</v>
+        <v>0.8</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue Oct 13 17:14:12 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,7 +486,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.61</v>
+        <v>7.63</v>
       </c>
       <c r="D2" t="n">
         <v>0.72</v>
@@ -495,13 +495,13 @@
         <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>99.7</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="3">
@@ -516,202 +516,202 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>17.3</v>
+        <v>17.37</v>
       </c>
       <c r="D3" t="n">
         <v>1.87</v>
       </c>
       <c r="E3" t="n">
-        <v>39.2</v>
+        <v>41</v>
       </c>
       <c r="F3" t="n">
-        <v>97</v>
+        <v>96.7</v>
       </c>
       <c r="G3" t="n">
-        <v>68.09999999999999</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>24.6</v>
+        <v>14.78</v>
       </c>
       <c r="D4" t="n">
-        <v>2.06</v>
+        <v>1.25</v>
       </c>
       <c r="E4" t="n">
-        <v>63.9</v>
+        <v>55.1</v>
       </c>
       <c r="F4" t="n">
-        <v>71.09999999999999</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="G4" t="n">
         <v>67.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>20.06</v>
+        <v>24.57</v>
       </c>
       <c r="D5" t="n">
-        <v>3.6</v>
+        <v>2.06</v>
       </c>
       <c r="E5" t="n">
-        <v>60.2</v>
+        <v>63.5</v>
       </c>
       <c r="F5" t="n">
-        <v>74.40000000000001</v>
+        <v>71</v>
       </c>
       <c r="G5" t="n">
-        <v>67.3</v>
+        <v>67.2</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>20.39</v>
+        <v>13.29</v>
       </c>
       <c r="D6" t="n">
-        <v>1.73</v>
+        <v>1.39</v>
       </c>
       <c r="E6" t="n">
-        <v>80.7</v>
+        <v>45.5</v>
       </c>
       <c r="F6" t="n">
-        <v>43.7</v>
+        <v>82.3</v>
       </c>
       <c r="G6" t="n">
-        <v>62.2</v>
+        <v>63.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>14.63</v>
+        <v>19.98</v>
       </c>
       <c r="D7" t="n">
-        <v>1.24</v>
+        <v>0.98</v>
       </c>
       <c r="E7" t="n">
-        <v>45.2</v>
+        <v>67.7</v>
       </c>
       <c r="F7" t="n">
-        <v>75</v>
+        <v>54.8</v>
       </c>
       <c r="G7" t="n">
-        <v>60.1</v>
+        <v>61.2</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>13.09</v>
+        <v>19.87</v>
       </c>
       <c r="D8" t="n">
-        <v>1.37</v>
+        <v>3.56</v>
       </c>
       <c r="E8" t="n">
-        <v>41</v>
+        <v>52.4</v>
       </c>
       <c r="F8" t="n">
-        <v>75.59999999999999</v>
+        <v>65.3</v>
       </c>
       <c r="G8" t="n">
-        <v>58.3</v>
+        <v>58.8</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>19.97</v>
+        <v>20.25</v>
       </c>
       <c r="D9" t="n">
-        <v>0.97</v>
+        <v>1.72</v>
       </c>
       <c r="E9" t="n">
-        <v>65.40000000000001</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>45.2</v>
+        <v>33.5</v>
       </c>
       <c r="G9" t="n">
-        <v>55.3</v>
+        <v>52.7</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="10">
@@ -726,22 +726,22 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>19.63</v>
+        <v>19.68</v>
       </c>
       <c r="D10" t="n">
         <v>1.64</v>
       </c>
       <c r="E10" t="n">
-        <v>49.4</v>
+        <v>52.7</v>
       </c>
       <c r="F10" t="n">
         <v>45.2</v>
       </c>
       <c r="G10" t="n">
-        <v>47.3</v>
+        <v>49</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="11">
@@ -756,22 +756,22 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>27.93</v>
+        <v>27.64</v>
       </c>
       <c r="D11" t="n">
-        <v>2.68</v>
+        <v>2.66</v>
       </c>
       <c r="E11" t="n">
-        <v>31.9</v>
+        <v>24.6</v>
       </c>
       <c r="F11" t="n">
-        <v>53.9</v>
+        <v>48.5</v>
       </c>
       <c r="G11" t="n">
-        <v>42.9</v>
+        <v>36.5</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="12">
@@ -786,22 +786,22 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>26.93</v>
+        <v>26.82</v>
       </c>
       <c r="D12" t="n">
-        <v>2.41</v>
+        <v>2.4</v>
       </c>
       <c r="E12" t="n">
-        <v>25.3</v>
+        <v>19.8</v>
       </c>
       <c r="F12" t="n">
-        <v>56.9</v>
+        <v>52.1</v>
       </c>
       <c r="G12" t="n">
-        <v>41.1</v>
+        <v>35.9</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="13">
@@ -816,22 +816,22 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>32.59</v>
+        <v>32.42</v>
       </c>
       <c r="D13" t="n">
-        <v>1.96</v>
+        <v>1.94</v>
       </c>
       <c r="E13" t="n">
-        <v>82.8</v>
+        <v>80.5</v>
       </c>
       <c r="F13" t="n">
-        <v>18.7</v>
+        <v>13.5</v>
       </c>
       <c r="G13" t="n">
-        <v>37.9</v>
+        <v>33.6</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="14">
@@ -846,22 +846,22 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>21.85</v>
+        <v>21.73</v>
       </c>
       <c r="D14" t="n">
-        <v>2.03</v>
+        <v>2.02</v>
       </c>
       <c r="E14" t="n">
-        <v>33.4</v>
+        <v>27.2</v>
       </c>
       <c r="F14" t="n">
-        <v>41.6</v>
+        <v>36.2</v>
       </c>
       <c r="G14" t="n">
-        <v>37.5</v>
+        <v>31.7</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="15">
@@ -876,52 +876,52 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>8.84</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="E15" t="n">
-        <v>22.9</v>
+        <v>13.2</v>
       </c>
       <c r="F15" t="n">
-        <v>49.7</v>
+        <v>42.8</v>
       </c>
       <c r="G15" t="n">
-        <v>36.3</v>
+        <v>28</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>15.02</v>
+        <v>29.42</v>
       </c>
       <c r="D16" t="n">
-        <v>2.3</v>
+        <v>2.31</v>
       </c>
       <c r="E16" t="n">
-        <v>17.8</v>
+        <v>21</v>
       </c>
       <c r="F16" t="n">
-        <v>47</v>
+        <v>30.2</v>
       </c>
       <c r="G16" t="n">
-        <v>32.4</v>
+        <v>25.6</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="17">
@@ -936,172 +936,172 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>20.97</v>
+        <v>21.11</v>
       </c>
       <c r="D17" t="n">
-        <v>1.78</v>
+        <v>1.79</v>
       </c>
       <c r="E17" t="n">
-        <v>15.1</v>
+        <v>21.6</v>
       </c>
       <c r="F17" t="n">
-        <v>22.6</v>
+        <v>27.2</v>
       </c>
       <c r="G17" t="n">
-        <v>20.3</v>
+        <v>25.5</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>10.55</v>
+        <v>14.93</v>
       </c>
       <c r="D18" t="n">
-        <v>0.62</v>
+        <v>2.29</v>
       </c>
       <c r="E18" t="n">
-        <v>43.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F18" t="n">
-        <v>9.300000000000001</v>
+        <v>41</v>
       </c>
       <c r="G18" t="n">
-        <v>19.5</v>
+        <v>25.1</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>29.28</v>
+        <v>10.56</v>
       </c>
       <c r="D19" t="n">
-        <v>2.29</v>
+        <v>0.62</v>
       </c>
       <c r="E19" t="n">
-        <v>10.8</v>
+        <v>44.3</v>
       </c>
       <c r="F19" t="n">
-        <v>16</v>
+        <v>9.6</v>
       </c>
       <c r="G19" t="n">
-        <v>14.4</v>
+        <v>20</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>7.58</v>
+        <v>29.8</v>
       </c>
       <c r="D20" t="n">
-        <v>1.18</v>
+        <v>1.87</v>
       </c>
       <c r="E20" t="n">
-        <v>8.4</v>
+        <v>1.2</v>
       </c>
       <c r="F20" t="n">
-        <v>15.1</v>
+        <v>18</v>
       </c>
       <c r="G20" t="n">
-        <v>13.1</v>
+        <v>12.9</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>29.87</v>
+        <v>65.3</v>
       </c>
       <c r="D21" t="n">
-        <v>1.86</v>
+        <v>3.47</v>
       </c>
       <c r="E21" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="F21" t="n">
-        <v>15.4</v>
+        <v>12</v>
       </c>
       <c r="G21" t="n">
-        <v>11.1</v>
+        <v>8.9</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>64.28</v>
+        <v>49.78</v>
       </c>
       <c r="D22" t="n">
         <v>3.41</v>
       </c>
       <c r="E22" t="n">
-        <v>1.2</v>
+        <v>3</v>
       </c>
       <c r="F22" t="n">
-        <v>10.2</v>
+        <v>8.4</v>
       </c>
       <c r="G22" t="n">
-        <v>7.5</v>
+        <v>6.8</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="23">
@@ -1116,10 +1116,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>45.17</v>
+        <v>45.14</v>
       </c>
       <c r="D23" t="n">
-        <v>6.71</v>
+        <v>6.7</v>
       </c>
       <c r="E23" t="n">
         <v>0.6</v>
@@ -1131,7 +1131,7 @@
         <v>6.5</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="24">
@@ -1146,82 +1146,82 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>33.73</v>
+        <v>33.97</v>
       </c>
       <c r="D24" t="n">
-        <v>2.97</v>
+        <v>2.99</v>
       </c>
       <c r="E24" t="n">
-        <v>1.8</v>
+        <v>4.8</v>
       </c>
       <c r="F24" t="n">
-        <v>5.7</v>
+        <v>6.6</v>
       </c>
       <c r="G24" t="n">
-        <v>4.5</v>
+        <v>6</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>21.92</v>
+        <v>39.09</v>
       </c>
       <c r="D25" t="n">
-        <v>1.97</v>
+        <v>3.64</v>
       </c>
       <c r="E25" t="n">
-        <v>4.2</v>
+        <v>1.8</v>
       </c>
       <c r="F25" t="n">
-        <v>1.8</v>
+        <v>3.3</v>
       </c>
       <c r="G25" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>39.06</v>
+        <v>27.21</v>
       </c>
       <c r="D26" t="n">
-        <v>3.64</v>
+        <v>2.61</v>
       </c>
       <c r="E26" t="n">
-        <v>1.2</v>
+        <v>2.4</v>
       </c>
       <c r="F26" t="n">
-        <v>3</v>
+        <v>2.4</v>
       </c>
       <c r="G26" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="27">
@@ -1236,10 +1236,10 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>21.21</v>
+        <v>21.15</v>
       </c>
       <c r="D27" t="n">
-        <v>2.22</v>
+        <v>2.21</v>
       </c>
       <c r="E27" t="n">
         <v>0.6</v>
@@ -1251,115 +1251,115 @@
         <v>2.3</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>18.22</v>
+        <v>7.48</v>
       </c>
       <c r="D28" t="n">
-        <v>1.39</v>
+        <v>1.16</v>
       </c>
       <c r="E28" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="F28" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="G28" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>26.86</v>
+        <v>15.77</v>
       </c>
       <c r="D29" t="n">
-        <v>2.58</v>
+        <v>2.97</v>
       </c>
       <c r="E29" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="F29" t="n">
         <v>1.8</v>
       </c>
       <c r="G29" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>24.59</v>
+        <v>21.63</v>
       </c>
       <c r="D30" t="n">
-        <v>2.77</v>
+        <v>1.94</v>
       </c>
       <c r="E30" t="n">
         <v>1.2</v>
       </c>
       <c r="F30" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="G30" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>48.29</v>
+        <v>18.1</v>
       </c>
       <c r="D31" t="n">
-        <v>3.31</v>
+        <v>1.38</v>
       </c>
       <c r="E31" t="n">
         <v>0.6</v>
@@ -1371,37 +1371,37 @@
         <v>1.2</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>15.7</v>
+        <v>24.05</v>
       </c>
       <c r="D32" t="n">
-        <v>2.95</v>
+        <v>2.71</v>
       </c>
       <c r="E32" t="n">
         <v>0.6</v>
       </c>
       <c r="F32" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="G32" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Wed Oct 14 14:40:48 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,82 +486,82 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.63</v>
+        <v>7.61</v>
       </c>
       <c r="D2" t="n">
         <v>0.72</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>99.7</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>99.90000000000001</v>
+        <v>99.3</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>17.37</v>
+        <v>14.94</v>
       </c>
       <c r="D3" t="n">
-        <v>1.87</v>
+        <v>1.26</v>
       </c>
       <c r="E3" t="n">
-        <v>41</v>
+        <v>67</v>
       </c>
       <c r="F3" t="n">
-        <v>96.7</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>68.90000000000001</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>14.78</v>
+        <v>17.68</v>
       </c>
       <c r="D4" t="n">
-        <v>1.25</v>
+        <v>1.91</v>
       </c>
       <c r="E4" t="n">
-        <v>55.1</v>
+        <v>45.8</v>
       </c>
       <c r="F4" t="n">
-        <v>79.90000000000001</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>67.5</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="5">
@@ -576,22 +576,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>24.57</v>
+        <v>24.95</v>
       </c>
       <c r="D5" t="n">
-        <v>2.06</v>
+        <v>2.09</v>
       </c>
       <c r="E5" t="n">
-        <v>63.5</v>
+        <v>70.5</v>
       </c>
       <c r="F5" t="n">
-        <v>71</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>67.2</v>
+        <v>72.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="6">
@@ -606,52 +606,52 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>13.29</v>
+        <v>13.68</v>
       </c>
       <c r="D6" t="n">
-        <v>1.39</v>
+        <v>1.43</v>
       </c>
       <c r="E6" t="n">
-        <v>45.5</v>
+        <v>48.5</v>
       </c>
       <c r="F6" t="n">
-        <v>82.3</v>
+        <v>90.8</v>
       </c>
       <c r="G6" t="n">
-        <v>63.9</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>19.98</v>
+        <v>20.49</v>
       </c>
       <c r="D7" t="n">
-        <v>0.98</v>
+        <v>1.74</v>
       </c>
       <c r="E7" t="n">
-        <v>67.7</v>
+        <v>87.5</v>
       </c>
       <c r="F7" t="n">
-        <v>54.8</v>
+        <v>51.8</v>
       </c>
       <c r="G7" t="n">
-        <v>61.2</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="8">
@@ -666,52 +666,52 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19.87</v>
+        <v>19.99</v>
       </c>
       <c r="D8" t="n">
-        <v>3.56</v>
+        <v>3.58</v>
       </c>
       <c r="E8" t="n">
-        <v>52.4</v>
+        <v>59.2</v>
       </c>
       <c r="F8" t="n">
-        <v>65.3</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>58.8</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>20.25</v>
+        <v>20.06</v>
       </c>
       <c r="D9" t="n">
-        <v>1.72</v>
+        <v>0.98</v>
       </c>
       <c r="E9" t="n">
-        <v>71.90000000000001</v>
+        <v>70.8</v>
       </c>
       <c r="F9" t="n">
-        <v>33.5</v>
+        <v>54.8</v>
       </c>
       <c r="G9" t="n">
-        <v>52.7</v>
+        <v>62.8</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="10">
@@ -726,670 +726,670 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>19.68</v>
+        <v>19.59</v>
       </c>
       <c r="D10" t="n">
         <v>1.64</v>
       </c>
       <c r="E10" t="n">
-        <v>52.7</v>
+        <v>47.3</v>
       </c>
       <c r="F10" t="n">
         <v>45.2</v>
       </c>
       <c r="G10" t="n">
-        <v>49</v>
+        <v>46.3</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>27.64</v>
+        <v>32.15</v>
       </c>
       <c r="D11" t="n">
-        <v>2.66</v>
+        <v>1.93</v>
       </c>
       <c r="E11" t="n">
-        <v>24.6</v>
+        <v>75</v>
       </c>
       <c r="F11" t="n">
-        <v>48.5</v>
+        <v>12.5</v>
       </c>
       <c r="G11" t="n">
-        <v>36.5</v>
+        <v>31.2</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>26.82</v>
+        <v>27.36</v>
       </c>
       <c r="D12" t="n">
-        <v>2.4</v>
+        <v>2.63</v>
       </c>
       <c r="E12" t="n">
-        <v>19.8</v>
+        <v>20.8</v>
       </c>
       <c r="F12" t="n">
-        <v>52.1</v>
+        <v>41.1</v>
       </c>
       <c r="G12" t="n">
-        <v>35.9</v>
+        <v>31</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>32.42</v>
+        <v>21.47</v>
       </c>
       <c r="D13" t="n">
-        <v>1.94</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>80.5</v>
+        <v>17.9</v>
       </c>
       <c r="F13" t="n">
-        <v>13.5</v>
+        <v>31.5</v>
       </c>
       <c r="G13" t="n">
-        <v>33.6</v>
+        <v>24.7</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>21.73</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="D14" t="n">
-        <v>2.02</v>
+        <v>0.96</v>
       </c>
       <c r="E14" t="n">
-        <v>27.2</v>
+        <v>9.5</v>
       </c>
       <c r="F14" t="n">
-        <v>36.2</v>
+        <v>36.3</v>
       </c>
       <c r="G14" t="n">
-        <v>31.7</v>
+        <v>22.9</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>8.619999999999999</v>
+        <v>26.46</v>
       </c>
       <c r="D15" t="n">
-        <v>0.97</v>
+        <v>2.37</v>
       </c>
       <c r="E15" t="n">
-        <v>13.2</v>
+        <v>10.7</v>
       </c>
       <c r="F15" t="n">
-        <v>42.8</v>
+        <v>34.8</v>
       </c>
       <c r="G15" t="n">
-        <v>28</v>
+        <v>22.8</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801210.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>社会服务</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>29.42</v>
+        <v>14.87</v>
       </c>
       <c r="D16" t="n">
-        <v>2.31</v>
+        <v>2.28</v>
       </c>
       <c r="E16" t="n">
-        <v>21</v>
+        <v>5.7</v>
       </c>
       <c r="F16" t="n">
-        <v>30.2</v>
+        <v>34.5</v>
       </c>
       <c r="G16" t="n">
-        <v>25.6</v>
+        <v>20.1</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801720.SI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>建筑装饰</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>21.11</v>
+        <v>10.53</v>
       </c>
       <c r="D17" t="n">
-        <v>1.79</v>
+        <v>0.62</v>
       </c>
       <c r="E17" t="n">
-        <v>21.6</v>
+        <v>42.9</v>
       </c>
       <c r="F17" t="n">
-        <v>27.2</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>25.5</v>
+        <v>19.7</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801210.SI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>社会服务</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>14.93</v>
+        <v>29.16</v>
       </c>
       <c r="D18" t="n">
         <v>2.29</v>
       </c>
       <c r="E18" t="n">
-        <v>9.300000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="F18" t="n">
-        <v>41</v>
+        <v>16.1</v>
       </c>
       <c r="G18" t="n">
-        <v>25.1</v>
+        <v>14.3</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801720.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>建筑装饰</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>10.56</v>
+        <v>20.82</v>
       </c>
       <c r="D19" t="n">
-        <v>0.62</v>
+        <v>1.77</v>
       </c>
       <c r="E19" t="n">
-        <v>44.3</v>
+        <v>5.4</v>
       </c>
       <c r="F19" t="n">
-        <v>9.6</v>
+        <v>17.3</v>
       </c>
       <c r="G19" t="n">
-        <v>20</v>
+        <v>13.7</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>29.8</v>
+        <v>64.11</v>
       </c>
       <c r="D20" t="n">
-        <v>1.87</v>
+        <v>3.4</v>
       </c>
       <c r="E20" t="n">
         <v>1.2</v>
       </c>
       <c r="F20" t="n">
-        <v>18</v>
+        <v>10.1</v>
       </c>
       <c r="G20" t="n">
-        <v>12.9</v>
+        <v>7.4</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>65.3</v>
+        <v>43.86</v>
       </c>
       <c r="D21" t="n">
-        <v>3.47</v>
+        <v>6.51</v>
       </c>
       <c r="E21" t="n">
-        <v>1.8</v>
+        <v>0.6</v>
       </c>
       <c r="F21" t="n">
-        <v>12</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>8.9</v>
+        <v>6</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>49.78</v>
+        <v>28.76</v>
       </c>
       <c r="D22" t="n">
-        <v>3.41</v>
+        <v>1.79</v>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>1.2</v>
       </c>
       <c r="F22" t="n">
-        <v>8.4</v>
+        <v>4.5</v>
       </c>
       <c r="G22" t="n">
-        <v>6.8</v>
+        <v>3.5</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>45.14</v>
+        <v>49.31</v>
       </c>
       <c r="D23" t="n">
-        <v>6.7</v>
+        <v>3.37</v>
       </c>
       <c r="E23" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="F23" t="n">
-        <v>9</v>
+        <v>3.6</v>
       </c>
       <c r="G23" t="n">
-        <v>6.5</v>
+        <v>2.9</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>33.97</v>
+        <v>26.68</v>
       </c>
       <c r="D24" t="n">
-        <v>2.99</v>
+        <v>2.56</v>
       </c>
       <c r="E24" t="n">
-        <v>4.8</v>
+        <v>1.2</v>
       </c>
       <c r="F24" t="n">
-        <v>6.6</v>
+        <v>1.8</v>
       </c>
       <c r="G24" t="n">
-        <v>6</v>
+        <v>1.6</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>39.09</v>
+        <v>33.13</v>
       </c>
       <c r="D25" t="n">
-        <v>3.64</v>
+        <v>2.91</v>
       </c>
       <c r="E25" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="F25" t="n">
-        <v>3.3</v>
+        <v>1.5</v>
       </c>
       <c r="G25" t="n">
-        <v>2.8</v>
+        <v>1.4</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>27.21</v>
+        <v>20.79</v>
       </c>
       <c r="D26" t="n">
-        <v>2.61</v>
+        <v>2.17</v>
       </c>
       <c r="E26" t="n">
-        <v>2.4</v>
+        <v>0.6</v>
       </c>
       <c r="F26" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="G26" t="n">
-        <v>2.4</v>
+        <v>1</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>21.15</v>
+        <v>21.23</v>
       </c>
       <c r="D27" t="n">
-        <v>2.21</v>
+        <v>1.9</v>
       </c>
       <c r="E27" t="n">
         <v>0.6</v>
       </c>
       <c r="F27" t="n">
-        <v>3</v>
+        <v>1.2</v>
       </c>
       <c r="G27" t="n">
-        <v>2.3</v>
+        <v>1</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>7.48</v>
+        <v>38.52</v>
       </c>
       <c r="D28" t="n">
-        <v>1.16</v>
+        <v>3.59</v>
       </c>
       <c r="E28" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="F28" t="n">
-        <v>2.1</v>
+        <v>0.9</v>
       </c>
       <c r="G28" t="n">
-        <v>1.8</v>
+        <v>0.8</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>15.77</v>
+        <v>7.41</v>
       </c>
       <c r="D29" t="n">
-        <v>2.97</v>
+        <v>1.15</v>
       </c>
       <c r="E29" t="n">
-        <v>1.5</v>
+        <v>0.6</v>
       </c>
       <c r="F29" t="n">
-        <v>1.8</v>
+        <v>0.9</v>
       </c>
       <c r="G29" t="n">
-        <v>1.7</v>
+        <v>0.8</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>21.63</v>
+        <v>15.45</v>
       </c>
       <c r="D30" t="n">
-        <v>1.94</v>
+        <v>2.91</v>
       </c>
       <c r="E30" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="F30" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="G30" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>18.1</v>
+        <v>23.33</v>
       </c>
       <c r="D31" t="n">
-        <v>1.38</v>
+        <v>2.63</v>
       </c>
       <c r="E31" t="n">
         <v>0.6</v>
       </c>
       <c r="F31" t="n">
-        <v>1.5</v>
+        <v>0.6</v>
       </c>
       <c r="G31" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>24.05</v>
+        <v>17.9</v>
       </c>
       <c r="D32" t="n">
-        <v>2.71</v>
+        <v>1.37</v>
       </c>
       <c r="E32" t="n">
         <v>0.6</v>
@@ -1401,7 +1401,7 @@
         <v>0.6</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Thu Oct 15 14:26:00 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,52 +486,52 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.61</v>
+        <v>7.63</v>
       </c>
       <c r="D2" t="n">
         <v>0.72</v>
       </c>
       <c r="E2" t="n">
+        <v>99.7</v>
+      </c>
+      <c r="F2" t="n">
         <v>99.09999999999999</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>99.40000000000001</v>
       </c>
-      <c r="G2" t="n">
-        <v>99.3</v>
-      </c>
       <c r="H2" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801120.SI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>14.94</v>
+        <v>20.18</v>
       </c>
       <c r="D3" t="n">
-        <v>1.26</v>
+        <v>3.62</v>
       </c>
       <c r="E3" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F3" t="n">
-        <v>83.90000000000001</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>75.40000000000001</v>
+        <v>72.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="4">
@@ -546,22 +546,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>17.68</v>
+        <v>17.43</v>
       </c>
       <c r="D4" t="n">
-        <v>1.91</v>
+        <v>1.88</v>
       </c>
       <c r="E4" t="n">
-        <v>45.8</v>
+        <v>44.4</v>
       </c>
       <c r="F4" t="n">
-        <v>99.40000000000001</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>72.59999999999999</v>
+        <v>71</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="5">
@@ -576,22 +576,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>24.95</v>
+        <v>24.57</v>
       </c>
       <c r="D5" t="n">
-        <v>2.09</v>
+        <v>2.06</v>
       </c>
       <c r="E5" t="n">
-        <v>70.5</v>
+        <v>63</v>
       </c>
       <c r="F5" t="n">
-        <v>74.09999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>72.3</v>
+        <v>66.7</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="6">
@@ -606,322 +606,322 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>13.68</v>
+        <v>13.44</v>
       </c>
       <c r="D6" t="n">
-        <v>1.43</v>
+        <v>1.41</v>
       </c>
       <c r="E6" t="n">
-        <v>48.5</v>
+        <v>45.6</v>
       </c>
       <c r="F6" t="n">
-        <v>90.8</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>69.59999999999999</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>20.49</v>
+        <v>19.59</v>
       </c>
       <c r="D7" t="n">
-        <v>1.74</v>
+        <v>0.96</v>
       </c>
       <c r="E7" t="n">
-        <v>87.5</v>
+        <v>56.8</v>
       </c>
       <c r="F7" t="n">
-        <v>51.8</v>
+        <v>39.3</v>
       </c>
       <c r="G7" t="n">
-        <v>69.59999999999999</v>
+        <v>48.1</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801120.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>食品饮料</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19.99</v>
+        <v>14.49</v>
       </c>
       <c r="D8" t="n">
-        <v>3.58</v>
+        <v>1.22</v>
       </c>
       <c r="E8" t="n">
-        <v>59.2</v>
+        <v>33.1</v>
       </c>
       <c r="F8" t="n">
-        <v>72.59999999999999</v>
+        <v>52.7</v>
       </c>
       <c r="G8" t="n">
-        <v>65.90000000000001</v>
+        <v>42.9</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>20.06</v>
+        <v>20.15</v>
       </c>
       <c r="D9" t="n">
-        <v>0.98</v>
+        <v>1.71</v>
       </c>
       <c r="E9" t="n">
-        <v>70.8</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="F9" t="n">
-        <v>54.8</v>
+        <v>25.4</v>
       </c>
       <c r="G9" t="n">
-        <v>62.8</v>
+        <v>37.3</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>19.59</v>
+        <v>27.36</v>
       </c>
       <c r="D10" t="n">
-        <v>1.64</v>
+        <v>2.63</v>
       </c>
       <c r="E10" t="n">
-        <v>47.3</v>
+        <v>21</v>
       </c>
       <c r="F10" t="n">
-        <v>45.2</v>
+        <v>41.1</v>
       </c>
       <c r="G10" t="n">
-        <v>46.3</v>
+        <v>31.1</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>32.15</v>
+        <v>26.22</v>
       </c>
       <c r="D11" t="n">
-        <v>1.93</v>
+        <v>2.35</v>
       </c>
       <c r="E11" t="n">
-        <v>75</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>12.5</v>
+        <v>29</v>
       </c>
       <c r="G11" t="n">
-        <v>31.2</v>
+        <v>22.8</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>27.36</v>
+        <v>31.27</v>
       </c>
       <c r="D12" t="n">
-        <v>2.63</v>
+        <v>1.88</v>
       </c>
       <c r="E12" t="n">
-        <v>20.8</v>
+        <v>59.5</v>
       </c>
       <c r="F12" t="n">
-        <v>41.1</v>
+        <v>2.1</v>
       </c>
       <c r="G12" t="n">
-        <v>31</v>
+        <v>19.3</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>21.47</v>
+        <v>19.22</v>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>1.61</v>
       </c>
       <c r="E13" t="n">
-        <v>17.9</v>
+        <v>15.4</v>
       </c>
       <c r="F13" t="n">
-        <v>31.5</v>
+        <v>19.8</v>
       </c>
       <c r="G13" t="n">
-        <v>24.7</v>
+        <v>18.5</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>8.539999999999999</v>
+        <v>14.75</v>
       </c>
       <c r="D14" t="n">
-        <v>0.96</v>
+        <v>2.26</v>
       </c>
       <c r="E14" t="n">
-        <v>9.5</v>
+        <v>1.8</v>
       </c>
       <c r="F14" t="n">
-        <v>36.3</v>
+        <v>23.4</v>
       </c>
       <c r="G14" t="n">
-        <v>22.9</v>
+        <v>16.9</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>26.46</v>
+        <v>20.97</v>
       </c>
       <c r="D15" t="n">
-        <v>2.37</v>
+        <v>1.95</v>
       </c>
       <c r="E15" t="n">
-        <v>10.7</v>
+        <v>7.1</v>
       </c>
       <c r="F15" t="n">
-        <v>34.8</v>
+        <v>15.4</v>
       </c>
       <c r="G15" t="n">
-        <v>22.8</v>
+        <v>12.9</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>14.87</v>
+        <v>8.33</v>
       </c>
       <c r="D16" t="n">
-        <v>2.28</v>
+        <v>0.93</v>
       </c>
       <c r="E16" t="n">
-        <v>5.7</v>
+        <v>3.3</v>
       </c>
       <c r="F16" t="n">
-        <v>34.5</v>
+        <v>16.6</v>
       </c>
       <c r="G16" t="n">
-        <v>20.1</v>
+        <v>12.6</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="17">
@@ -936,22 +936,22 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>10.53</v>
+        <v>10.29</v>
       </c>
       <c r="D17" t="n">
-        <v>0.62</v>
+        <v>0.61</v>
       </c>
       <c r="E17" t="n">
-        <v>42.9</v>
+        <v>27.2</v>
       </c>
       <c r="F17" t="n">
-        <v>9.800000000000001</v>
+        <v>3.3</v>
       </c>
       <c r="G17" t="n">
-        <v>19.7</v>
+        <v>10.4</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="18">
@@ -966,22 +966,22 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>29.16</v>
+        <v>28.44</v>
       </c>
       <c r="D18" t="n">
-        <v>2.29</v>
+        <v>2.23</v>
       </c>
       <c r="E18" t="n">
-        <v>10.1</v>
+        <v>6.5</v>
       </c>
       <c r="F18" t="n">
-        <v>16.1</v>
+        <v>9.5</v>
       </c>
       <c r="G18" t="n">
-        <v>14.3</v>
+        <v>8.6</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="19">
@@ -996,22 +996,22 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>20.82</v>
+        <v>20.4</v>
       </c>
       <c r="D19" t="n">
-        <v>1.77</v>
+        <v>1.73</v>
       </c>
       <c r="E19" t="n">
-        <v>5.4</v>
+        <v>0.6</v>
       </c>
       <c r="F19" t="n">
-        <v>17.3</v>
+        <v>10.7</v>
       </c>
       <c r="G19" t="n">
-        <v>13.7</v>
+        <v>7.6</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="20">
@@ -1026,22 +1026,22 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>64.11</v>
+        <v>62.13</v>
       </c>
       <c r="D20" t="n">
-        <v>3.4</v>
+        <v>3.29</v>
       </c>
       <c r="E20" t="n">
         <v>1.2</v>
       </c>
       <c r="F20" t="n">
-        <v>10.1</v>
+        <v>6.5</v>
       </c>
       <c r="G20" t="n">
-        <v>7.4</v>
+        <v>4.9</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="21">
@@ -1056,22 +1056,22 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>43.86</v>
+        <v>42.51</v>
       </c>
       <c r="D21" t="n">
-        <v>6.51</v>
+        <v>6.31</v>
       </c>
       <c r="E21" t="n">
         <v>0.6</v>
       </c>
       <c r="F21" t="n">
-        <v>8.300000000000001</v>
+        <v>4.1</v>
       </c>
       <c r="G21" t="n">
-        <v>6</v>
+        <v>3.1</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="22">
@@ -1086,52 +1086,52 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>28.76</v>
+        <v>27.69</v>
       </c>
       <c r="D22" t="n">
-        <v>1.79</v>
+        <v>1.72</v>
       </c>
       <c r="E22" t="n">
         <v>1.2</v>
       </c>
       <c r="F22" t="n">
-        <v>4.5</v>
+        <v>1.8</v>
       </c>
       <c r="G22" t="n">
-        <v>3.5</v>
+        <v>1.6</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>49.31</v>
+        <v>7.43</v>
       </c>
       <c r="D23" t="n">
-        <v>3.37</v>
+        <v>1.15</v>
       </c>
       <c r="E23" t="n">
         <v>1.2</v>
       </c>
       <c r="F23" t="n">
-        <v>3.6</v>
+        <v>1.2</v>
       </c>
       <c r="G23" t="n">
-        <v>2.9</v>
+        <v>1.2</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="24">
@@ -1146,190 +1146,190 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>26.68</v>
+        <v>26.1</v>
       </c>
       <c r="D24" t="n">
-        <v>2.56</v>
+        <v>2.51</v>
       </c>
       <c r="E24" t="n">
         <v>1.2</v>
       </c>
       <c r="F24" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="G24" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>33.13</v>
+        <v>20.81</v>
       </c>
       <c r="D25" t="n">
-        <v>2.91</v>
+        <v>1.86</v>
       </c>
       <c r="E25" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F25" t="n">
         <v>1.2</v>
       </c>
-      <c r="F25" t="n">
-        <v>1.5</v>
-      </c>
       <c r="G25" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>20.79</v>
+        <v>14.87</v>
       </c>
       <c r="D26" t="n">
-        <v>2.17</v>
+        <v>2.8</v>
       </c>
       <c r="E26" t="n">
         <v>0.6</v>
       </c>
       <c r="F26" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="G26" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>21.23</v>
+        <v>20.12</v>
       </c>
       <c r="D27" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="E27" t="n">
         <v>0.6</v>
       </c>
       <c r="F27" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="G27" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>38.52</v>
+        <v>22.83</v>
       </c>
       <c r="D28" t="n">
-        <v>3.59</v>
+        <v>2.57</v>
       </c>
       <c r="E28" t="n">
         <v>0.6</v>
       </c>
       <c r="F28" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="G28" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>7.41</v>
+        <v>32</v>
       </c>
       <c r="D29" t="n">
-        <v>1.15</v>
+        <v>2.81</v>
       </c>
       <c r="E29" t="n">
         <v>0.6</v>
       </c>
       <c r="F29" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="G29" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>15.45</v>
+        <v>37.75</v>
       </c>
       <c r="D30" t="n">
-        <v>2.91</v>
+        <v>3.52</v>
       </c>
       <c r="E30" t="n">
         <v>0.6</v>
@@ -1341,25 +1341,25 @@
         <v>0.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>23.33</v>
+        <v>47.39</v>
       </c>
       <c r="D31" t="n">
-        <v>2.63</v>
+        <v>3.24</v>
       </c>
       <c r="E31" t="n">
         <v>0.6</v>
@@ -1371,7 +1371,7 @@
         <v>0.6</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="32">
@@ -1386,10 +1386,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>17.9</v>
+        <v>17.41</v>
       </c>
       <c r="D32" t="n">
-        <v>1.37</v>
+        <v>1.33</v>
       </c>
       <c r="E32" t="n">
         <v>0.6</v>
@@ -1401,7 +1401,7 @@
         <v>0.6</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Fri Oct 16 14:17:47 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.63</v>
+        <v>7.61</v>
       </c>
       <c r="D2" t="n">
         <v>0.72</v>
       </c>
       <c r="E2" t="n">
-        <v>99.7</v>
+        <v>98.2</v>
       </c>
       <c r="F2" t="n">
-        <v>99.09999999999999</v>
+        <v>98.8</v>
       </c>
       <c r="G2" t="n">
-        <v>99.40000000000001</v>
+        <v>98.5</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="3">
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.18</v>
+        <v>20.36</v>
       </c>
       <c r="D3" t="n">
-        <v>3.62</v>
+        <v>3.65</v>
       </c>
       <c r="E3" t="n">
-        <v>68</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>76.90000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>72.5</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="4">
@@ -546,82 +546,82 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>17.43</v>
+        <v>17.56</v>
       </c>
       <c r="D4" t="n">
-        <v>1.88</v>
+        <v>1.89</v>
       </c>
       <c r="E4" t="n">
-        <v>44.4</v>
+        <v>45.3</v>
       </c>
       <c r="F4" t="n">
-        <v>97.59999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="G4" t="n">
-        <v>71</v>
+        <v>71.8</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>24.57</v>
+        <v>13.57</v>
       </c>
       <c r="D5" t="n">
-        <v>2.06</v>
+        <v>1.42</v>
       </c>
       <c r="E5" t="n">
-        <v>63</v>
+        <v>46.8</v>
       </c>
       <c r="F5" t="n">
-        <v>70.40000000000001</v>
+        <v>88.2</v>
       </c>
       <c r="G5" t="n">
-        <v>66.7</v>
+        <v>67.5</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>13.44</v>
+        <v>24.21</v>
       </c>
       <c r="D6" t="n">
-        <v>1.41</v>
+        <v>2.03</v>
       </c>
       <c r="E6" t="n">
-        <v>45.6</v>
+        <v>50.6</v>
       </c>
       <c r="F6" t="n">
-        <v>84.59999999999999</v>
+        <v>63.2</v>
       </c>
       <c r="G6" t="n">
-        <v>65.09999999999999</v>
+        <v>56.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="7">
@@ -636,22 +636,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>19.59</v>
+        <v>19.8</v>
       </c>
       <c r="D7" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="E7" t="n">
-        <v>56.8</v>
+        <v>58.8</v>
       </c>
       <c r="F7" t="n">
-        <v>39.3</v>
+        <v>45</v>
       </c>
       <c r="G7" t="n">
-        <v>48.1</v>
+        <v>51.9</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="8">
@@ -666,22 +666,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>14.49</v>
+        <v>14.47</v>
       </c>
       <c r="D8" t="n">
         <v>1.22</v>
       </c>
       <c r="E8" t="n">
-        <v>33.1</v>
+        <v>30</v>
       </c>
       <c r="F8" t="n">
-        <v>52.7</v>
+        <v>52.6</v>
       </c>
       <c r="G8" t="n">
-        <v>42.9</v>
+        <v>41.3</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="9">
@@ -696,232 +696,232 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>20.15</v>
+        <v>20.17</v>
       </c>
       <c r="D9" t="n">
         <v>1.71</v>
       </c>
       <c r="E9" t="n">
-        <v>65.09999999999999</v>
+        <v>65.3</v>
       </c>
       <c r="F9" t="n">
-        <v>25.4</v>
+        <v>25.6</v>
       </c>
       <c r="G9" t="n">
-        <v>37.3</v>
+        <v>37.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>27.36</v>
+        <v>8.66</v>
       </c>
       <c r="D10" t="n">
-        <v>2.63</v>
+        <v>0.95</v>
       </c>
       <c r="E10" t="n">
-        <v>21</v>
+        <v>16.8</v>
       </c>
       <c r="F10" t="n">
-        <v>41.1</v>
+        <v>29.4</v>
       </c>
       <c r="G10" t="n">
-        <v>31.1</v>
+        <v>25.6</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>26.22</v>
+        <v>19.34</v>
       </c>
       <c r="D11" t="n">
-        <v>2.35</v>
+        <v>1.62</v>
       </c>
       <c r="E11" t="n">
-        <v>8.300000000000001</v>
+        <v>24.4</v>
       </c>
       <c r="F11" t="n">
-        <v>29</v>
+        <v>25.6</v>
       </c>
       <c r="G11" t="n">
-        <v>22.8</v>
+        <v>25.2</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>31.27</v>
+        <v>27.05</v>
       </c>
       <c r="D12" t="n">
-        <v>1.88</v>
+        <v>2.6</v>
       </c>
       <c r="E12" t="n">
-        <v>59.5</v>
+        <v>18.2</v>
       </c>
       <c r="F12" t="n">
-        <v>2.1</v>
+        <v>31.5</v>
       </c>
       <c r="G12" t="n">
-        <v>19.3</v>
+        <v>24.9</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>19.22</v>
+        <v>31.6</v>
       </c>
       <c r="D13" t="n">
-        <v>1.61</v>
+        <v>1.89</v>
       </c>
       <c r="E13" t="n">
-        <v>15.4</v>
+        <v>63.5</v>
       </c>
       <c r="F13" t="n">
-        <v>19.8</v>
+        <v>4.7</v>
       </c>
       <c r="G13" t="n">
-        <v>18.5</v>
+        <v>22.4</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>14.75</v>
+        <v>26.4</v>
       </c>
       <c r="D14" t="n">
-        <v>2.26</v>
+        <v>2.36</v>
       </c>
       <c r="E14" t="n">
-        <v>1.8</v>
+        <v>11.2</v>
       </c>
       <c r="F14" t="n">
-        <v>23.4</v>
+        <v>32.1</v>
       </c>
       <c r="G14" t="n">
-        <v>16.9</v>
+        <v>21.6</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>20.97</v>
+        <v>14.79</v>
       </c>
       <c r="D15" t="n">
-        <v>1.95</v>
+        <v>2.27</v>
       </c>
       <c r="E15" t="n">
-        <v>7.1</v>
+        <v>2.4</v>
       </c>
       <c r="F15" t="n">
-        <v>15.4</v>
+        <v>27.6</v>
       </c>
       <c r="G15" t="n">
-        <v>12.9</v>
+        <v>20.1</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>8.33</v>
+        <v>21.11</v>
       </c>
       <c r="D16" t="n">
-        <v>0.93</v>
+        <v>1.96</v>
       </c>
       <c r="E16" t="n">
-        <v>3.3</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F16" t="n">
-        <v>16.6</v>
+        <v>19.4</v>
       </c>
       <c r="G16" t="n">
-        <v>12.6</v>
+        <v>16.1</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="17">
@@ -936,22 +936,22 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>10.29</v>
+        <v>10.39</v>
       </c>
       <c r="D17" t="n">
         <v>0.61</v>
       </c>
       <c r="E17" t="n">
-        <v>27.2</v>
+        <v>30.3</v>
       </c>
       <c r="F17" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="G17" t="n">
-        <v>10.4</v>
+        <v>11.6</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="18">
@@ -966,22 +966,22 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>28.44</v>
+        <v>28.51</v>
       </c>
       <c r="D18" t="n">
-        <v>2.23</v>
+        <v>2.24</v>
       </c>
       <c r="E18" t="n">
-        <v>6.5</v>
+        <v>7.1</v>
       </c>
       <c r="F18" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="G18" t="n">
-        <v>8.6</v>
+        <v>10.1</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="19">
@@ -996,7 +996,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>20.4</v>
+        <v>20.33</v>
       </c>
       <c r="D19" t="n">
         <v>1.73</v>
@@ -1005,13 +1005,13 @@
         <v>0.6</v>
       </c>
       <c r="F19" t="n">
-        <v>10.7</v>
+        <v>10.9</v>
       </c>
       <c r="G19" t="n">
-        <v>7.6</v>
+        <v>7.8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="20">
@@ -1026,172 +1026,172 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>62.13</v>
+        <v>62.31</v>
       </c>
       <c r="D20" t="n">
-        <v>3.29</v>
+        <v>3.31</v>
       </c>
       <c r="E20" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="F20" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G20" t="n">
         <v>6.5</v>
       </c>
-      <c r="G20" t="n">
-        <v>4.9</v>
-      </c>
       <c r="H20" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>42.51</v>
+        <v>48.67</v>
       </c>
       <c r="D21" t="n">
-        <v>6.31</v>
+        <v>3.33</v>
       </c>
       <c r="E21" t="n">
-        <v>0.6</v>
+        <v>1.8</v>
       </c>
       <c r="F21" t="n">
         <v>4.1</v>
       </c>
       <c r="G21" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>27.69</v>
+        <v>42.53</v>
       </c>
       <c r="D22" t="n">
-        <v>1.72</v>
+        <v>6.31</v>
       </c>
       <c r="E22" t="n">
         <v>1.2</v>
       </c>
       <c r="F22" t="n">
-        <v>1.8</v>
+        <v>4.4</v>
       </c>
       <c r="G22" t="n">
-        <v>1.6</v>
+        <v>3.4</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>7.43</v>
+        <v>28.05</v>
       </c>
       <c r="D23" t="n">
-        <v>1.15</v>
+        <v>1.74</v>
       </c>
       <c r="E23" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="F23" t="n">
-        <v>1.2</v>
+        <v>2.4</v>
       </c>
       <c r="G23" t="n">
-        <v>1.2</v>
+        <v>2.2</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>26.1</v>
+        <v>21.11</v>
       </c>
       <c r="D24" t="n">
-        <v>2.51</v>
+        <v>1.89</v>
       </c>
       <c r="E24" t="n">
         <v>1.2</v>
       </c>
       <c r="F24" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="G24" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>20.81</v>
+        <v>20.3</v>
       </c>
       <c r="D25" t="n">
-        <v>1.86</v>
+        <v>2.12</v>
       </c>
       <c r="E25" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="F25" t="n">
         <v>1.2</v>
       </c>
       <c r="G25" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="26">
@@ -1206,190 +1206,190 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>14.87</v>
+        <v>14.94</v>
       </c>
       <c r="D26" t="n">
-        <v>2.8</v>
+        <v>2.81</v>
       </c>
       <c r="E26" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="F26" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="G26" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>20.12</v>
+        <v>7.4</v>
       </c>
       <c r="D27" t="n">
-        <v>2.1</v>
+        <v>1.15</v>
       </c>
       <c r="E27" t="n">
         <v>0.6</v>
       </c>
       <c r="F27" t="n">
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="G27" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>22.83</v>
+        <v>32.03</v>
       </c>
       <c r="D28" t="n">
-        <v>2.57</v>
+        <v>2.82</v>
       </c>
       <c r="E28" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="F28" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="G28" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>32</v>
+        <v>17.47</v>
       </c>
       <c r="D29" t="n">
-        <v>2.81</v>
+        <v>1.34</v>
       </c>
       <c r="E29" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="F29" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="G29" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>37.75</v>
+        <v>26.05</v>
       </c>
       <c r="D30" t="n">
-        <v>3.52</v>
+        <v>2.5</v>
       </c>
       <c r="E30" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="F30" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="G30" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>47.39</v>
+        <v>22.81</v>
       </c>
       <c r="D31" t="n">
-        <v>3.24</v>
+        <v>2.57</v>
       </c>
       <c r="E31" t="n">
         <v>0.6</v>
       </c>
       <c r="F31" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="G31" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>17.41</v>
+        <v>37.64</v>
       </c>
       <c r="D32" t="n">
-        <v>1.33</v>
+        <v>3.51</v>
       </c>
       <c r="E32" t="n">
         <v>0.6</v>
@@ -1401,7 +1401,7 @@
         <v>0.6</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sat Oct 17 13:14:22 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.72</v>
       </c>
       <c r="E2" t="n">
+        <v>98</v>
+      </c>
+      <c r="F2" t="n">
+        <v>98.5</v>
+      </c>
+      <c r="G2" t="n">
         <v>98.2</v>
       </c>
-      <c r="F2" t="n">
-        <v>98.8</v>
-      </c>
-      <c r="G2" t="n">
-        <v>98.5</v>
-      </c>
       <c r="H2" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>3.65</v>
       </c>
       <c r="E3" t="n">
-        <v>75.90000000000001</v>
+        <v>75.7</v>
       </c>
       <c r="F3" t="n">
-        <v>82.90000000000001</v>
+        <v>82.7</v>
       </c>
       <c r="G3" t="n">
-        <v>79.40000000000001</v>
+        <v>79.2</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="4">
@@ -555,13 +555,13 @@
         <v>45.3</v>
       </c>
       <c r="F4" t="n">
-        <v>98.2</v>
+        <v>98</v>
       </c>
       <c r="G4" t="n">
-        <v>71.8</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="5">
@@ -585,13 +585,13 @@
         <v>46.8</v>
       </c>
       <c r="F5" t="n">
-        <v>88.2</v>
+        <v>88</v>
       </c>
       <c r="G5" t="n">
-        <v>67.5</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="6">
@@ -621,7 +621,7 @@
         <v>56.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="7">
@@ -651,7 +651,7 @@
         <v>51.9</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="8">
@@ -672,16 +672,16 @@
         <v>1.22</v>
       </c>
       <c r="E8" t="n">
-        <v>30</v>
+        <v>30.1</v>
       </c>
       <c r="F8" t="n">
         <v>52.6</v>
       </c>
       <c r="G8" t="n">
-        <v>41.3</v>
+        <v>41.4</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.71</v>
       </c>
       <c r="E9" t="n">
-        <v>65.3</v>
+        <v>65.2</v>
       </c>
       <c r="F9" t="n">
-        <v>25.6</v>
+        <v>25.7</v>
       </c>
       <c r="G9" t="n">
-        <v>37.5</v>
+        <v>37.6</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>0.95</v>
       </c>
       <c r="E10" t="n">
-        <v>16.8</v>
+        <v>17</v>
       </c>
       <c r="F10" t="n">
-        <v>29.4</v>
+        <v>29.5</v>
       </c>
       <c r="G10" t="n">
-        <v>25.6</v>
+        <v>25.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.62</v>
       </c>
       <c r="E11" t="n">
-        <v>24.4</v>
+        <v>24.6</v>
       </c>
       <c r="F11" t="n">
-        <v>25.6</v>
+        <v>25.7</v>
       </c>
       <c r="G11" t="n">
-        <v>25.2</v>
+        <v>25.4</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>2.6</v>
       </c>
       <c r="E12" t="n">
-        <v>18.2</v>
+        <v>18.4</v>
       </c>
       <c r="F12" t="n">
-        <v>31.5</v>
+        <v>31.6</v>
       </c>
       <c r="G12" t="n">
-        <v>24.9</v>
+        <v>25</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="13">
@@ -825,13 +825,13 @@
         <v>63.5</v>
       </c>
       <c r="F13" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="G13" t="n">
-        <v>22.4</v>
+        <v>22.5</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2.36</v>
       </c>
       <c r="E14" t="n">
-        <v>11.2</v>
+        <v>11.4</v>
       </c>
       <c r="F14" t="n">
-        <v>32.1</v>
+        <v>32.2</v>
       </c>
       <c r="G14" t="n">
-        <v>21.6</v>
+        <v>21.8</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>2.27</v>
       </c>
       <c r="E15" t="n">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="F15" t="n">
-        <v>27.6</v>
+        <v>27.8</v>
       </c>
       <c r="G15" t="n">
-        <v>20.1</v>
+        <v>20.2</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>1.96</v>
       </c>
       <c r="E16" t="n">
-        <v>8.199999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="F16" t="n">
-        <v>19.4</v>
+        <v>19.6</v>
       </c>
       <c r="G16" t="n">
-        <v>16.1</v>
+        <v>16.3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>0.61</v>
       </c>
       <c r="E17" t="n">
-        <v>30.3</v>
+        <v>30.4</v>
       </c>
       <c r="F17" t="n">
-        <v>3.5</v>
+        <v>3.8</v>
       </c>
       <c r="G17" t="n">
-        <v>11.6</v>
+        <v>11.8</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.24</v>
       </c>
       <c r="E18" t="n">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
       <c r="F18" t="n">
-        <v>11.5</v>
+        <v>11.7</v>
       </c>
       <c r="G18" t="n">
-        <v>10.1</v>
+        <v>10.4</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.73</v>
       </c>
       <c r="E19" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="F19" t="n">
-        <v>10.9</v>
+        <v>11.1</v>
       </c>
       <c r="G19" t="n">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>3.31</v>
       </c>
       <c r="E20" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>8.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>6.5</v>
+        <v>6.8</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>3.33</v>
       </c>
       <c r="E21" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>4.1</v>
+        <v>4.4</v>
       </c>
       <c r="G21" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>6.31</v>
       </c>
       <c r="E22" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="F22" t="n">
-        <v>4.4</v>
+        <v>4.7</v>
       </c>
       <c r="G22" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>1.74</v>
       </c>
       <c r="E23" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="G23" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="24">
@@ -1152,16 +1152,16 @@
         <v>1.89</v>
       </c>
       <c r="E24" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="F24" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="G24" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="25">
@@ -1182,16 +1182,16 @@
         <v>2.12</v>
       </c>
       <c r="E25" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="F25" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G25" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="26">
@@ -1212,16 +1212,16 @@
         <v>2.81</v>
       </c>
       <c r="E26" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="F26" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G26" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="27">
@@ -1242,16 +1242,16 @@
         <v>1.15</v>
       </c>
       <c r="E27" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="F27" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="G27" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.82</v>
       </c>
       <c r="E28" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="F28" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G28" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.34</v>
       </c>
       <c r="E29" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="F29" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G29" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>2.5</v>
       </c>
       <c r="E30" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="F30" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G30" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>2.57</v>
       </c>
       <c r="E31" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="F31" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="G31" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>3.51</v>
       </c>
       <c r="E32" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="F32" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="G32" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Sun Oct 18 13:35:33 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -492,16 +492,16 @@
         <v>0.72</v>
       </c>
       <c r="E2" t="n">
+        <v>97.7</v>
+      </c>
+      <c r="F2" t="n">
+        <v>98.3</v>
+      </c>
+      <c r="G2" t="n">
         <v>98</v>
       </c>
-      <c r="F2" t="n">
-        <v>98.5</v>
-      </c>
-      <c r="G2" t="n">
-        <v>98.2</v>
-      </c>
       <c r="H2" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="3">
@@ -522,16 +522,16 @@
         <v>3.65</v>
       </c>
       <c r="E3" t="n">
-        <v>75.7</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>82.7</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>79.2</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="4">
@@ -555,13 +555,13 @@
         <v>45.3</v>
       </c>
       <c r="F4" t="n">
-        <v>98</v>
+        <v>97.7</v>
       </c>
       <c r="G4" t="n">
-        <v>71.59999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="5">
@@ -585,13 +585,13 @@
         <v>46.8</v>
       </c>
       <c r="F5" t="n">
-        <v>88</v>
+        <v>87.8</v>
       </c>
       <c r="G5" t="n">
-        <v>67.40000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="6">
@@ -615,13 +615,13 @@
         <v>50.6</v>
       </c>
       <c r="F6" t="n">
-        <v>63.2</v>
+        <v>63.1</v>
       </c>
       <c r="G6" t="n">
-        <v>56.9</v>
+        <v>56.8</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="7">
@@ -642,16 +642,16 @@
         <v>0.97</v>
       </c>
       <c r="E7" t="n">
-        <v>58.8</v>
+        <v>58.7</v>
       </c>
       <c r="F7" t="n">
-        <v>45</v>
+        <v>45.1</v>
       </c>
       <c r="G7" t="n">
         <v>51.9</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="8">
@@ -672,7 +672,7 @@
         <v>1.22</v>
       </c>
       <c r="E8" t="n">
-        <v>30.1</v>
+        <v>30.2</v>
       </c>
       <c r="F8" t="n">
         <v>52.6</v>
@@ -681,7 +681,7 @@
         <v>41.4</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="9">
@@ -702,16 +702,16 @@
         <v>1.71</v>
       </c>
       <c r="E9" t="n">
-        <v>65.2</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="F9" t="n">
-        <v>25.7</v>
+        <v>25.9</v>
       </c>
       <c r="G9" t="n">
         <v>37.6</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         <v>0.95</v>
       </c>
       <c r="E10" t="n">
-        <v>17</v>
+        <v>17.2</v>
       </c>
       <c r="F10" t="n">
-        <v>29.5</v>
+        <v>29.7</v>
       </c>
       <c r="G10" t="n">
-        <v>25.8</v>
+        <v>25.9</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="11">
@@ -762,16 +762,16 @@
         <v>1.62</v>
       </c>
       <c r="E11" t="n">
-        <v>24.6</v>
+        <v>24.7</v>
       </c>
       <c r="F11" t="n">
-        <v>25.7</v>
+        <v>25.9</v>
       </c>
       <c r="G11" t="n">
-        <v>25.4</v>
+        <v>25.5</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="12">
@@ -792,16 +792,16 @@
         <v>2.6</v>
       </c>
       <c r="E12" t="n">
-        <v>18.4</v>
+        <v>18.6</v>
       </c>
       <c r="F12" t="n">
-        <v>31.6</v>
+        <v>31.7</v>
       </c>
       <c r="G12" t="n">
-        <v>25</v>
+        <v>25.1</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="13">
@@ -822,16 +822,16 @@
         <v>1.89</v>
       </c>
       <c r="E13" t="n">
-        <v>63.5</v>
+        <v>63.4</v>
       </c>
       <c r="F13" t="n">
-        <v>5</v>
+        <v>5.2</v>
       </c>
       <c r="G13" t="n">
-        <v>22.5</v>
+        <v>22.7</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="14">
@@ -852,16 +852,16 @@
         <v>2.36</v>
       </c>
       <c r="E14" t="n">
-        <v>11.4</v>
+        <v>11.6</v>
       </c>
       <c r="F14" t="n">
-        <v>32.2</v>
+        <v>32.3</v>
       </c>
       <c r="G14" t="n">
-        <v>21.8</v>
+        <v>21.9</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="15">
@@ -882,16 +882,16 @@
         <v>2.27</v>
       </c>
       <c r="E15" t="n">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="F15" t="n">
-        <v>27.8</v>
+        <v>27.9</v>
       </c>
       <c r="G15" t="n">
-        <v>20.2</v>
+        <v>20.4</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="16">
@@ -912,16 +912,16 @@
         <v>1.96</v>
       </c>
       <c r="E16" t="n">
-        <v>8.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F16" t="n">
-        <v>19.6</v>
+        <v>19.8</v>
       </c>
       <c r="G16" t="n">
-        <v>16.3</v>
+        <v>16.5</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="17">
@@ -942,16 +942,16 @@
         <v>0.61</v>
       </c>
       <c r="E17" t="n">
-        <v>30.4</v>
+        <v>30.5</v>
       </c>
       <c r="F17" t="n">
-        <v>3.8</v>
+        <v>4.1</v>
       </c>
       <c r="G17" t="n">
-        <v>11.8</v>
+        <v>12</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="18">
@@ -972,16 +972,16 @@
         <v>2.24</v>
       </c>
       <c r="E18" t="n">
-        <v>7.3</v>
+        <v>7.6</v>
       </c>
       <c r="F18" t="n">
-        <v>11.7</v>
+        <v>11.9</v>
       </c>
       <c r="G18" t="n">
-        <v>10.4</v>
+        <v>10.6</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="19">
@@ -1002,16 +1002,16 @@
         <v>1.73</v>
       </c>
       <c r="E19" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="F19" t="n">
-        <v>11.1</v>
+        <v>11.3</v>
       </c>
       <c r="G19" t="n">
-        <v>8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="20">
@@ -1032,16 +1032,16 @@
         <v>3.31</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="F20" t="n">
-        <v>8.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="G20" t="n">
-        <v>6.8</v>
+        <v>7</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="21">
@@ -1062,16 +1062,16 @@
         <v>3.33</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="F21" t="n">
-        <v>4.4</v>
+        <v>4.7</v>
       </c>
       <c r="G21" t="n">
-        <v>3.7</v>
+        <v>4</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="22">
@@ -1092,16 +1092,16 @@
         <v>6.31</v>
       </c>
       <c r="E22" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="F22" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="G22" t="n">
-        <v>3.7</v>
+        <v>4</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="23">
@@ -1122,16 +1122,16 @@
         <v>1.74</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="F23" t="n">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="G23" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="24">
@@ -1152,46 +1152,46 @@
         <v>1.89</v>
       </c>
       <c r="E24" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="G24" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>20.3</v>
+        <v>7.4</v>
       </c>
       <c r="D25" t="n">
-        <v>2.12</v>
+        <v>1.15</v>
       </c>
       <c r="E25" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="F25" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="G25" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="26">
@@ -1212,46 +1212,46 @@
         <v>2.81</v>
       </c>
       <c r="E26" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="F26" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="G26" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>7.4</v>
+        <v>20.3</v>
       </c>
       <c r="D27" t="n">
-        <v>1.15</v>
+        <v>2.12</v>
       </c>
       <c r="E27" t="n">
-        <v>0.9</v>
+        <v>1.7</v>
       </c>
       <c r="F27" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="G27" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="28">
@@ -1272,16 +1272,16 @@
         <v>2.82</v>
       </c>
       <c r="E28" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="F28" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="G28" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="29">
@@ -1302,16 +1302,16 @@
         <v>1.34</v>
       </c>
       <c r="E29" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="F29" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="G29" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="30">
@@ -1332,16 +1332,16 @@
         <v>2.5</v>
       </c>
       <c r="E30" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="F30" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="G30" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="31">
@@ -1362,16 +1362,16 @@
         <v>2.57</v>
       </c>
       <c r="E31" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="F31" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G31" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="32">
@@ -1392,16 +1392,16 @@
         <v>3.51</v>
       </c>
       <c r="E32" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="F32" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="G32" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Mon Oct 19 16:38:59 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.61</v>
+        <v>7.75</v>
       </c>
       <c r="D2" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="E2" t="n">
-        <v>97.7</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>98.3</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="3">
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.36</v>
+        <v>20.32</v>
       </c>
       <c r="D3" t="n">
-        <v>3.65</v>
+        <v>3.64</v>
       </c>
       <c r="E3" t="n">
-        <v>75.59999999999999</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>82.59999999999999</v>
+        <v>79.8</v>
       </c>
       <c r="G3" t="n">
-        <v>79.09999999999999</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="4">
@@ -546,22 +546,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>17.56</v>
+        <v>17.76</v>
       </c>
       <c r="D4" t="n">
-        <v>1.89</v>
+        <v>1.92</v>
       </c>
       <c r="E4" t="n">
-        <v>45.3</v>
+        <v>48.6</v>
       </c>
       <c r="F4" t="n">
-        <v>97.7</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>71.5</v>
+        <v>74</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="5">
@@ -576,352 +576,352 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>13.57</v>
+        <v>13.61</v>
       </c>
       <c r="D5" t="n">
-        <v>1.42</v>
+        <v>1.43</v>
       </c>
       <c r="E5" t="n">
-        <v>46.8</v>
+        <v>48.6</v>
       </c>
       <c r="F5" t="n">
-        <v>87.8</v>
+        <v>90.8</v>
       </c>
       <c r="G5" t="n">
-        <v>67.3</v>
+        <v>69.7</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>24.21</v>
+        <v>20.29</v>
       </c>
       <c r="D6" t="n">
-        <v>2.03</v>
+        <v>1.72</v>
       </c>
       <c r="E6" t="n">
-        <v>50.6</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>63.1</v>
+        <v>35</v>
       </c>
       <c r="G6" t="n">
-        <v>56.8</v>
+        <v>55.1</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>19.8</v>
+        <v>24.16</v>
       </c>
       <c r="D7" t="n">
-        <v>0.97</v>
+        <v>2.02</v>
       </c>
       <c r="E7" t="n">
-        <v>58.7</v>
+        <v>49.1</v>
       </c>
       <c r="F7" t="n">
-        <v>45.1</v>
+        <v>58.1</v>
       </c>
       <c r="G7" t="n">
-        <v>51.9</v>
+        <v>53.6</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801170.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>交通运输</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>14.47</v>
+        <v>19.91</v>
       </c>
       <c r="D8" t="n">
-        <v>1.22</v>
+        <v>0.97</v>
       </c>
       <c r="E8" t="n">
-        <v>30.2</v>
+        <v>61.8</v>
       </c>
       <c r="F8" t="n">
-        <v>52.6</v>
+        <v>45.1</v>
       </c>
       <c r="G8" t="n">
-        <v>41.4</v>
+        <v>53.5</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801170.SI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>交通运输</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>20.17</v>
+        <v>14.51</v>
       </c>
       <c r="D9" t="n">
-        <v>1.71</v>
+        <v>1.23</v>
       </c>
       <c r="E9" t="n">
-        <v>65.09999999999999</v>
+        <v>35.3</v>
       </c>
       <c r="F9" t="n">
-        <v>25.9</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>37.6</v>
+        <v>50.6</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>8.66</v>
+        <v>15.05</v>
       </c>
       <c r="D10" t="n">
-        <v>0.95</v>
+        <v>2.31</v>
       </c>
       <c r="E10" t="n">
-        <v>17.2</v>
+        <v>22.8</v>
       </c>
       <c r="F10" t="n">
-        <v>29.7</v>
+        <v>53.5</v>
       </c>
       <c r="G10" t="n">
-        <v>25.9</v>
+        <v>38.2</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801130.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>纺织服饰</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>19.34</v>
+        <v>27.23</v>
       </c>
       <c r="D11" t="n">
-        <v>1.62</v>
+        <v>2.62</v>
       </c>
       <c r="E11" t="n">
-        <v>24.7</v>
+        <v>20.2</v>
       </c>
       <c r="F11" t="n">
-        <v>25.9</v>
+        <v>38.7</v>
       </c>
       <c r="G11" t="n">
-        <v>25.5</v>
+        <v>29.5</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801130.SI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>纺织服饰</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>27.05</v>
+        <v>19.38</v>
       </c>
       <c r="D12" t="n">
-        <v>2.6</v>
+        <v>1.62</v>
       </c>
       <c r="E12" t="n">
-        <v>18.6</v>
+        <v>27.2</v>
       </c>
       <c r="F12" t="n">
-        <v>31.7</v>
+        <v>26</v>
       </c>
       <c r="G12" t="n">
-        <v>25.1</v>
+        <v>26.4</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801980.SI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>美容护理</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>31.6</v>
+        <v>26.41</v>
       </c>
       <c r="D13" t="n">
-        <v>1.89</v>
+        <v>2.37</v>
       </c>
       <c r="E13" t="n">
-        <v>63.4</v>
+        <v>12.7</v>
       </c>
       <c r="F13" t="n">
-        <v>5.2</v>
+        <v>36.4</v>
       </c>
       <c r="G13" t="n">
-        <v>22.7</v>
+        <v>24.6</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801980.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>美容护理</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>26.4</v>
+        <v>21.22</v>
       </c>
       <c r="D14" t="n">
-        <v>2.36</v>
+        <v>1.98</v>
       </c>
       <c r="E14" t="n">
-        <v>11.6</v>
+        <v>13.6</v>
       </c>
       <c r="F14" t="n">
-        <v>32.3</v>
+        <v>28.3</v>
       </c>
       <c r="G14" t="n">
-        <v>21.9</v>
+        <v>23.9</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>14.79</v>
+        <v>8.44</v>
       </c>
       <c r="D15" t="n">
-        <v>2.27</v>
+        <v>0.95</v>
       </c>
       <c r="E15" t="n">
-        <v>2.9</v>
+        <v>6.6</v>
       </c>
       <c r="F15" t="n">
-        <v>27.9</v>
+        <v>29.8</v>
       </c>
       <c r="G15" t="n">
-        <v>20.4</v>
+        <v>22.8</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>21.11</v>
+        <v>31.45</v>
       </c>
       <c r="D16" t="n">
-        <v>1.96</v>
+        <v>1.89</v>
       </c>
       <c r="E16" t="n">
-        <v>8.699999999999999</v>
+        <v>61.8</v>
       </c>
       <c r="F16" t="n">
-        <v>19.8</v>
+        <v>5.5</v>
       </c>
       <c r="G16" t="n">
-        <v>16.5</v>
+        <v>22.4</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="17">
@@ -936,22 +936,22 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>10.39</v>
+        <v>10.36</v>
       </c>
       <c r="D17" t="n">
         <v>0.61</v>
       </c>
       <c r="E17" t="n">
-        <v>30.5</v>
+        <v>29.5</v>
       </c>
       <c r="F17" t="n">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
       <c r="G17" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="18">
@@ -966,442 +966,442 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>28.51</v>
+        <v>28.38</v>
       </c>
       <c r="D18" t="n">
-        <v>2.24</v>
+        <v>2.23</v>
       </c>
       <c r="E18" t="n">
-        <v>7.6</v>
+        <v>6.4</v>
       </c>
       <c r="F18" t="n">
-        <v>11.9</v>
+        <v>9.5</v>
       </c>
       <c r="G18" t="n">
-        <v>10.6</v>
+        <v>8.6</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801200.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>商贸零售</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>20.33</v>
+        <v>49.55</v>
       </c>
       <c r="D19" t="n">
-        <v>1.73</v>
+        <v>3.39</v>
       </c>
       <c r="E19" t="n">
-        <v>1.2</v>
+        <v>5.8</v>
       </c>
       <c r="F19" t="n">
-        <v>11.3</v>
+        <v>9</v>
       </c>
       <c r="G19" t="n">
-        <v>8.300000000000001</v>
+        <v>8</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801200.SI</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>商贸零售</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>62.31</v>
+        <v>20.25</v>
       </c>
       <c r="D20" t="n">
-        <v>3.31</v>
+        <v>1.72</v>
       </c>
       <c r="E20" t="n">
-        <v>2.3</v>
+        <v>0.6</v>
       </c>
       <c r="F20" t="n">
-        <v>9</v>
+        <v>8.4</v>
       </c>
       <c r="G20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>48.67</v>
+        <v>21.37</v>
       </c>
       <c r="D21" t="n">
-        <v>3.33</v>
+        <v>1.92</v>
       </c>
       <c r="E21" t="n">
-        <v>2.3</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
-        <v>4.7</v>
+        <v>4</v>
       </c>
       <c r="G21" t="n">
         <v>4</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>42.53</v>
+        <v>26.16</v>
       </c>
       <c r="D22" t="n">
-        <v>6.31</v>
+        <v>2.51</v>
       </c>
       <c r="E22" t="n">
-        <v>1.7</v>
+        <v>3.5</v>
       </c>
       <c r="F22" t="n">
-        <v>4.9</v>
+        <v>3.2</v>
       </c>
       <c r="G22" t="n">
-        <v>4</v>
+        <v>3.3</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801890.SI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>机械设备</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>28.05</v>
+        <v>32.26</v>
       </c>
       <c r="D23" t="n">
-        <v>1.74</v>
+        <v>2.83</v>
       </c>
       <c r="E23" t="n">
-        <v>2.3</v>
+        <v>2.9</v>
       </c>
       <c r="F23" t="n">
         <v>2.9</v>
       </c>
       <c r="G23" t="n">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>21.11</v>
+        <v>17.49</v>
       </c>
       <c r="D24" t="n">
-        <v>1.89</v>
+        <v>1.34</v>
       </c>
       <c r="E24" t="n">
-        <v>1.7</v>
+        <v>2.9</v>
       </c>
       <c r="F24" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" t="n">
         <v>2.3</v>
       </c>
-      <c r="G24" t="n">
-        <v>2.2</v>
-      </c>
       <c r="H24" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>7.4</v>
+        <v>41.61</v>
       </c>
       <c r="D25" t="n">
-        <v>1.15</v>
+        <v>6.18</v>
       </c>
       <c r="E25" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="F25" t="n">
-        <v>2</v>
+        <v>2.9</v>
       </c>
       <c r="G25" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>14.94</v>
+        <v>37.18</v>
       </c>
       <c r="D26" t="n">
-        <v>2.81</v>
+        <v>3.54</v>
       </c>
       <c r="E26" t="n">
-        <v>1.7</v>
+        <v>0.6</v>
       </c>
       <c r="F26" t="n">
-        <v>1.7</v>
+        <v>2.9</v>
       </c>
       <c r="G26" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>20.3</v>
+        <v>7.4</v>
       </c>
       <c r="D27" t="n">
-        <v>2.12</v>
+        <v>1.15</v>
       </c>
       <c r="E27" t="n">
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
       <c r="F27" t="n">
-        <v>1.7</v>
+        <v>2.3</v>
       </c>
       <c r="G27" t="n">
-        <v>1.7</v>
+        <v>2.1</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801890.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>机械设备</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>32.03</v>
+        <v>27.76</v>
       </c>
       <c r="D28" t="n">
-        <v>2.82</v>
+        <v>1.73</v>
       </c>
       <c r="E28" t="n">
         <v>1.7</v>
       </c>
       <c r="F28" t="n">
-        <v>1.7</v>
+        <v>2.3</v>
       </c>
       <c r="G28" t="n">
-        <v>1.7</v>
+        <v>2.1</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>17.47</v>
+        <v>14.92</v>
       </c>
       <c r="D29" t="n">
-        <v>1.34</v>
+        <v>2.81</v>
       </c>
       <c r="E29" t="n">
-        <v>1.7</v>
+        <v>1.2</v>
       </c>
       <c r="F29" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="G29" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>26.05</v>
+        <v>19.95</v>
       </c>
       <c r="D30" t="n">
-        <v>2.5</v>
+        <v>2.12</v>
       </c>
       <c r="E30" t="n">
-        <v>1.7</v>
+        <v>0.6</v>
       </c>
       <c r="F30" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="G30" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>22.81</v>
+        <v>61.02</v>
       </c>
       <c r="D31" t="n">
-        <v>2.57</v>
+        <v>3.23</v>
       </c>
       <c r="E31" t="n">
         <v>1.2</v>
       </c>
       <c r="F31" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="G31" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>37.64</v>
+        <v>22.65</v>
       </c>
       <c r="D32" t="n">
-        <v>3.51</v>
+        <v>2.55</v>
       </c>
       <c r="E32" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="F32" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="G32" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto Update: Market & Industry Thermometer [Tue Oct 20 14:30:12 UTC 2026]
</commit_message>
<xml_diff>
--- a/A股申万一级行业温度计_最新.xlsx
+++ b/A股申万一级行业温度计_最新.xlsx
@@ -486,22 +486,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.75</v>
+        <v>7.71</v>
       </c>
       <c r="D2" t="n">
         <v>0.73</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>99.7</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="3">
@@ -522,166 +522,166 @@
         <v>3.64</v>
       </c>
       <c r="E3" t="n">
-        <v>73.09999999999999</v>
+        <v>73</v>
       </c>
       <c r="F3" t="n">
-        <v>79.8</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>76.40000000000001</v>
+        <v>76.3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>801950.SI</t>
+          <t>801960.SI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>煤炭</t>
+          <t>石油石化</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>17.76</v>
+        <v>13.7</v>
       </c>
       <c r="D4" t="n">
-        <v>1.92</v>
+        <v>1.44</v>
       </c>
       <c r="E4" t="n">
-        <v>48.6</v>
+        <v>51.1</v>
       </c>
       <c r="F4" t="n">
-        <v>99.40000000000001</v>
+        <v>91.7</v>
       </c>
       <c r="G4" t="n">
-        <v>74</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>801960.SI</t>
+          <t>801950.SI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>石油石化</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>13.61</v>
+        <v>17.56</v>
       </c>
       <c r="D5" t="n">
-        <v>1.43</v>
+        <v>1.89</v>
       </c>
       <c r="E5" t="n">
-        <v>48.6</v>
+        <v>45.1</v>
       </c>
       <c r="F5" t="n">
-        <v>90.8</v>
+        <v>96.8</v>
       </c>
       <c r="G5" t="n">
-        <v>69.7</v>
+        <v>71</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>801160.SI</t>
+          <t>801760.SI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>传媒</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>20.29</v>
+        <v>24.06</v>
       </c>
       <c r="D6" t="n">
-        <v>1.72</v>
+        <v>2.02</v>
       </c>
       <c r="E6" t="n">
-        <v>75.09999999999999</v>
+        <v>47.7</v>
       </c>
       <c r="F6" t="n">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="G6" t="n">
-        <v>55.1</v>
+        <v>52.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>801760.SI</t>
+          <t>801040.SI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>传媒</t>
+          <t>钢铁</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>24.16</v>
+        <v>19.75</v>
       </c>
       <c r="D7" t="n">
-        <v>2.02</v>
+        <v>0.97</v>
       </c>
       <c r="E7" t="n">
-        <v>49.1</v>
+        <v>57.2</v>
       </c>
       <c r="F7" t="n">
-        <v>58.1</v>
+        <v>45.1</v>
       </c>
       <c r="G7" t="n">
-        <v>53.6</v>
+        <v>51.1</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>801040.SI</t>
+          <t>801160.SI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>钢铁</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19.91</v>
+        <v>20.19</v>
       </c>
       <c r="D8" t="n">
-        <v>0.97</v>
+        <v>1.71</v>
       </c>
       <c r="E8" t="n">
-        <v>61.8</v>
+        <v>67.5</v>
       </c>
       <c r="F8" t="n">
-        <v>45.1</v>
+        <v>25.9</v>
       </c>
       <c r="G8" t="n">
-        <v>53.5</v>
+        <v>38.4</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="9">
@@ -696,82 +696,82 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>14.51</v>
+        <v>14.4</v>
       </c>
       <c r="D9" t="n">
-        <v>1.23</v>
+        <v>1.22</v>
       </c>
       <c r="E9" t="n">
-        <v>35.3</v>
+        <v>24.1</v>
       </c>
       <c r="F9" t="n">
-        <v>65.90000000000001</v>
+        <v>52.3</v>
       </c>
       <c r="G9" t="n">
-        <v>50.6</v>
+        <v>38.2</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>801110.SI</t>
+          <t>801150.SI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>家用电器</t>
+          <t>医药生物</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>15.05</v>
+        <v>27.47</v>
       </c>
       <c r="D10" t="n">
-        <v>2.31</v>
+        <v>2.64</v>
       </c>
       <c r="E10" t="n">
-        <v>22.8</v>
+        <v>24.4</v>
       </c>
       <c r="F10" t="n">
-        <v>53.5</v>
+        <v>46.8</v>
       </c>
       <c r="G10" t="n">
-        <v>38.2</v>
+        <v>35.6</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>801150.SI</t>
+          <t>801110.SI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>医药生物</t>
+          <t>家用电器</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>27.23</v>
+        <v>14.93</v>
       </c>
       <c r="D11" t="n">
-        <v>2.62</v>
+        <v>2.29</v>
       </c>
       <c r="E11" t="n">
-        <v>20.2</v>
+        <v>12.1</v>
       </c>
       <c r="F11" t="n">
-        <v>38.7</v>
+        <v>42.5</v>
       </c>
       <c r="G11" t="n">
-        <v>29.5</v>
+        <v>27.3</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="12">
@@ -786,22 +786,22 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>19.38</v>
+        <v>19.4</v>
       </c>
       <c r="D12" t="n">
         <v>1.62</v>
       </c>
       <c r="E12" t="n">
-        <v>27.2</v>
+        <v>28.2</v>
       </c>
       <c r="F12" t="n">
-        <v>26</v>
+        <v>26.1</v>
       </c>
       <c r="G12" t="n">
-        <v>26.4</v>
+        <v>26.8</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="13">
@@ -816,112 +816,112 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>26.41</v>
+        <v>26.48</v>
       </c>
       <c r="D13" t="n">
         <v>2.37</v>
       </c>
       <c r="E13" t="n">
-        <v>12.7</v>
+        <v>13.8</v>
       </c>
       <c r="F13" t="n">
-        <v>36.4</v>
+        <v>36.5</v>
       </c>
       <c r="G13" t="n">
-        <v>24.6</v>
+        <v>25.1</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>801140.SI</t>
+          <t>801010.SI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>轻工制造</t>
+          <t>农林牧渔</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>21.22</v>
+        <v>31.48</v>
       </c>
       <c r="D14" t="n">
-        <v>1.98</v>
+        <v>1.89</v>
       </c>
       <c r="E14" t="n">
-        <v>13.6</v>
+        <v>62.1</v>
       </c>
       <c r="F14" t="n">
-        <v>28.3</v>
+        <v>5.7</v>
       </c>
       <c r="G14" t="n">
-        <v>23.9</v>
+        <v>22.6</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>801180.SI</t>
+          <t>801140.SI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>房地产</t>
+          <t>轻工制造</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>8.44</v>
+        <v>21.25</v>
       </c>
       <c r="D15" t="n">
-        <v>0.95</v>
+        <v>1.97</v>
       </c>
       <c r="E15" t="n">
-        <v>6.6</v>
+        <v>14.4</v>
       </c>
       <c r="F15" t="n">
-        <v>29.8</v>
+        <v>25.6</v>
       </c>
       <c r="G15" t="n">
-        <v>22.8</v>
+        <v>22.2</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>801010.SI</t>
+          <t>801180.SI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>农林牧渔</t>
+          <t>房地产</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>31.45</v>
+        <v>8.44</v>
       </c>
       <c r="D16" t="n">
-        <v>1.89</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E16" t="n">
-        <v>61.8</v>
+        <v>6.9</v>
       </c>
       <c r="F16" t="n">
-        <v>5.5</v>
+        <v>21.6</v>
       </c>
       <c r="G16" t="n">
-        <v>22.4</v>
+        <v>17.2</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="17">
@@ -936,22 +936,22 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>10.36</v>
+        <v>10.31</v>
       </c>
       <c r="D17" t="n">
         <v>0.61</v>
       </c>
       <c r="E17" t="n">
-        <v>29.5</v>
+        <v>27</v>
       </c>
       <c r="F17" t="n">
-        <v>4.3</v>
+        <v>4.6</v>
       </c>
       <c r="G17" t="n">
-        <v>11.9</v>
+        <v>11.3</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="18">
@@ -966,52 +966,52 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>28.38</v>
+        <v>28.49</v>
       </c>
       <c r="D18" t="n">
-        <v>2.23</v>
+        <v>2.24</v>
       </c>
       <c r="E18" t="n">
-        <v>6.4</v>
+        <v>7.5</v>
       </c>
       <c r="F18" t="n">
-        <v>9.5</v>
+        <v>12.6</v>
       </c>
       <c r="G18" t="n">
-        <v>8.6</v>
+        <v>11.1</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>801740.SI</t>
+          <t>801230.SI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>国防军工</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>49.55</v>
+        <v>62.19</v>
       </c>
       <c r="D19" t="n">
-        <v>3.39</v>
+        <v>3.3</v>
       </c>
       <c r="E19" t="n">
-        <v>5.8</v>
+        <v>2.3</v>
       </c>
       <c r="F19" t="n">
-        <v>9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>8</v>
+        <v>6.5</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="20">
@@ -1026,7 +1026,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>20.25</v>
+        <v>20.24</v>
       </c>
       <c r="D20" t="n">
         <v>1.72</v>
@@ -1035,73 +1035,73 @@
         <v>0.6</v>
       </c>
       <c r="F20" t="n">
-        <v>8.4</v>
+        <v>8.6</v>
       </c>
       <c r="G20" t="n">
-        <v>6</v>
+        <v>6.2</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>801880.SI</t>
+          <t>801740.SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>汽车</t>
+          <t>国防军工</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>21.37</v>
+        <v>49.27</v>
       </c>
       <c r="D21" t="n">
-        <v>1.92</v>
+        <v>3.37</v>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>3.4</v>
       </c>
       <c r="F21" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G21" t="n">
-        <v>4</v>
+        <v>5.3</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>801770.SI</t>
+          <t>801880.SI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>通信</t>
+          <t>汽车</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>26.16</v>
+        <v>21.49</v>
       </c>
       <c r="D22" t="n">
-        <v>2.51</v>
+        <v>1.92</v>
       </c>
       <c r="E22" t="n">
-        <v>3.5</v>
+        <v>4.6</v>
       </c>
       <c r="F22" t="n">
-        <v>3.2</v>
+        <v>4.3</v>
       </c>
       <c r="G22" t="n">
-        <v>3.3</v>
+        <v>4.4</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="23">
@@ -1116,280 +1116,280 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>32.26</v>
+        <v>32.85</v>
       </c>
       <c r="D23" t="n">
-        <v>2.83</v>
+        <v>2.89</v>
       </c>
       <c r="E23" t="n">
-        <v>2.9</v>
+        <v>3.4</v>
       </c>
       <c r="F23" t="n">
-        <v>2.9</v>
+        <v>4</v>
       </c>
       <c r="G23" t="n">
-        <v>2.9</v>
+        <v>3.9</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>801970.SI</t>
+          <t>801770.SI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>环保</t>
+          <t>通信</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>17.49</v>
+        <v>26.09</v>
       </c>
       <c r="D24" t="n">
-        <v>1.34</v>
+        <v>2.51</v>
       </c>
       <c r="E24" t="n">
         <v>2.9</v>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
+        <v>3.4</v>
       </c>
       <c r="G24" t="n">
-        <v>2.3</v>
+        <v>3.3</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>801080.SI</t>
+          <t>801750.SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>电子</t>
+          <t>计算机</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>41.61</v>
+        <v>37.71</v>
       </c>
       <c r="D25" t="n">
-        <v>6.18</v>
+        <v>3.58</v>
       </c>
       <c r="E25" t="n">
-        <v>0.6</v>
+        <v>2.9</v>
       </c>
       <c r="F25" t="n">
-        <v>2.9</v>
+        <v>3.4</v>
       </c>
       <c r="G25" t="n">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>801750.SI</t>
+          <t>801710.SI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>计算机</t>
+          <t>建筑材料</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>37.18</v>
+        <v>26.46</v>
       </c>
       <c r="D26" t="n">
-        <v>3.54</v>
+        <v>1.74</v>
       </c>
       <c r="E26" t="n">
-        <v>0.6</v>
+        <v>1.1</v>
       </c>
       <c r="F26" t="n">
-        <v>2.9</v>
+        <v>3.7</v>
       </c>
       <c r="G26" t="n">
-        <v>2.2</v>
+        <v>3</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>801790.SI</t>
+          <t>801080.SI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>非银金融</t>
+          <t>电子</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>7.4</v>
+        <v>41.9</v>
       </c>
       <c r="D27" t="n">
-        <v>1.15</v>
+        <v>6.22</v>
       </c>
       <c r="E27" t="n">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
       <c r="F27" t="n">
-        <v>2.3</v>
+        <v>3.7</v>
       </c>
       <c r="G27" t="n">
-        <v>2.1</v>
+        <v>3</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>801710.SI</t>
+          <t>801030.SI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>建筑材料</t>
+          <t>基础化工</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>27.76</v>
+        <v>20.02</v>
       </c>
       <c r="D28" t="n">
-        <v>1.73</v>
+        <v>2.13</v>
       </c>
       <c r="E28" t="n">
-        <v>1.7</v>
+        <v>1.1</v>
       </c>
       <c r="F28" t="n">
-        <v>2.3</v>
+        <v>3.4</v>
       </c>
       <c r="G28" t="n">
-        <v>2.1</v>
+        <v>2.8</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>801050.SI</t>
+          <t>801970.SI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>有色金属</t>
+          <t>环保</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>14.92</v>
+        <v>17.48</v>
       </c>
       <c r="D29" t="n">
-        <v>2.81</v>
+        <v>1.34</v>
       </c>
       <c r="E29" t="n">
-        <v>1.2</v>
+        <v>2.9</v>
       </c>
       <c r="F29" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="G29" t="n">
-        <v>1.8</v>
+        <v>2.5</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>801030.SI</t>
+          <t>801050.SI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>基础化工</t>
+          <t>有色金属</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>19.95</v>
+        <v>14.7</v>
       </c>
       <c r="D30" t="n">
-        <v>2.12</v>
+        <v>2.77</v>
       </c>
       <c r="E30" t="n">
         <v>0.6</v>
       </c>
       <c r="F30" t="n">
-        <v>2</v>
+        <v>0.6</v>
       </c>
       <c r="G30" t="n">
-        <v>1.6</v>
+        <v>0.6</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>801230.SI</t>
+          <t>801730.SI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>电力设备</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>61.02</v>
+        <v>22.49</v>
       </c>
       <c r="D31" t="n">
-        <v>3.23</v>
+        <v>2.53</v>
       </c>
       <c r="E31" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="F31" t="n">
-        <v>1.7</v>
+        <v>0.6</v>
       </c>
       <c r="G31" t="n">
-        <v>1.6</v>
+        <v>0.6</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>801730.SI</t>
+          <t>801790.SI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>电力设备</t>
+          <t>非银金融</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>22.65</v>
+        <v>7.29</v>
       </c>
       <c r="D32" t="n">
-        <v>2.55</v>
+        <v>1.13</v>
       </c>
       <c r="E32" t="n">
         <v>0.6</v>
@@ -1401,7 +1401,7 @@
         <v>0.6</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
   </sheetData>

</xml_diff>